<commit_message>
Summer week with first four days operations restricted
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,23 +8,33 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{386252D1-794C-413D-B687-80495CB7B4F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{647054F9-5F24-4198-8BE9-ADF689C7AD81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="30">
   <si>
-    <t>TIME PERIOD = 1 WEEK</t>
-  </si>
-  <si>
     <t>Season</t>
   </si>
   <si>
@@ -110,6 +120,9 @@
   </si>
   <si>
     <t>RTP RATE</t>
+  </si>
+  <si>
+    <t>TIME PERIOD = 1 WEEK, Rate = TOU 3</t>
   </si>
 </sst>
 </file>
@@ -971,82 +984,82 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:U20"/>
+  <dimension ref="A1:U21"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A1" t="s">
-        <v>0</v>
+      <c r="A1" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>5</v>
       </c>
-      <c r="F2" t="s">
+      <c r="G2" t="s">
         <v>6</v>
       </c>
-      <c r="G2" t="s">
+      <c r="H2" t="s">
         <v>7</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>8</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>9</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>10</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>11</v>
       </c>
-      <c r="L2" t="s">
+      <c r="M2" t="s">
         <v>12</v>
       </c>
-      <c r="M2" t="s">
+      <c r="N2" t="s">
         <v>13</v>
       </c>
-      <c r="N2" t="s">
+      <c r="O2" t="s">
         <v>14</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>15</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>16</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>17</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>18</v>
       </c>
-      <c r="S2" t="s">
+      <c r="T2" t="s">
         <v>19</v>
-      </c>
-      <c r="T2" t="s">
-        <v>20</v>
       </c>
     </row>
     <row r="3" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="s">
         <v>21</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -1103,15 +1116,15 @@
         <v>466.95526849999999</v>
       </c>
       <c r="U3" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -1170,10 +1183,10 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A5" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C5">
         <v>0</v>
@@ -1232,10 +1245,10 @@
     </row>
     <row r="6" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C6">
         <v>0</v>
@@ -1291,10 +1304,10 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C7">
         <v>0</v>
@@ -1353,10 +1366,10 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
         <v>24</v>
-      </c>
-      <c r="B8" t="s">
-        <v>25</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -1415,10 +1428,10 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C9">
         <v>0</v>
@@ -1474,10 +1487,10 @@
     </row>
     <row r="10" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B10" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C10">
         <v>0</v>
@@ -1536,10 +1549,10 @@
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C11">
         <v>2</v>
@@ -1598,10 +1611,10 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B12" t="s">
         <v>24</v>
-      </c>
-      <c r="B12" t="s">
-        <v>25</v>
       </c>
       <c r="C12">
         <v>2</v>
@@ -1658,325 +1671,325 @@
         <v>0.68036269900000002</v>
       </c>
     </row>
-    <row r="13" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
-        <v>29</v>
-      </c>
-    </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A14" t="s">
-        <v>24</v>
-      </c>
-      <c r="B14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C14">
-        <v>0</v>
-      </c>
-      <c r="D14">
-        <v>177048.079214225</v>
-      </c>
-      <c r="E14">
-        <v>282179.697150969</v>
-      </c>
-      <c r="F14">
-        <v>1.0581911624256699</v>
-      </c>
-      <c r="G14">
-        <v>79845.342667291203</v>
-      </c>
-      <c r="H14">
-        <v>6222.1442638440503</v>
-      </c>
-      <c r="I14">
-        <v>4534.7814140862702</v>
-      </c>
-      <c r="J14">
-        <f>SUM(G14:I14)</f>
-        <v>90602.268345221528</v>
-      </c>
-      <c r="K14">
-        <v>50847.265569999399</v>
-      </c>
-      <c r="L14">
-        <v>15307.856370494001</v>
-      </c>
-      <c r="M14">
-        <v>19298.378220313502</v>
-      </c>
-      <c r="N14">
-        <v>992.31070819735999</v>
-      </c>
-      <c r="O14">
-        <v>0</v>
-      </c>
-      <c r="P14">
-        <v>298600.06174110703</v>
-      </c>
-      <c r="Q14">
-        <v>987.15586819601197</v>
-      </c>
-      <c r="R14">
-        <v>15618.4724861042</v>
-      </c>
-      <c r="S14">
-        <v>92.967098131572797</v>
-      </c>
-      <c r="T14">
-        <v>-2.5456367562447402</v>
+      <c r="A14" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B15" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C15">
         <v>0</v>
       </c>
       <c r="D15">
-        <v>114550.946983783</v>
+        <v>177048.079214225</v>
       </c>
       <c r="E15">
-        <v>282179.671291181</v>
+        <v>282179.697150969</v>
       </c>
       <c r="F15">
-        <v>0.83671133512318097</v>
+        <v>1.0581911624256699</v>
       </c>
       <c r="G15">
-        <v>21079.803315233199</v>
+        <v>79845.342667291203</v>
       </c>
       <c r="H15">
-        <v>6217.0342487801199</v>
+        <v>6222.1442638440503</v>
       </c>
       <c r="I15">
-        <v>817.27332915015802</v>
+        <v>4534.7814140862702</v>
       </c>
       <c r="J15">
         <f>SUM(G15:I15)</f>
+        <v>90602.268345221528</v>
+      </c>
+      <c r="K15">
+        <v>50847.265569999399</v>
+      </c>
+      <c r="L15">
+        <v>15307.856370494001</v>
+      </c>
+      <c r="M15">
+        <v>19298.378220313502</v>
+      </c>
+      <c r="N15">
+        <v>992.31070819735999</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <v>298600.06174110703</v>
+      </c>
+      <c r="Q15">
+        <v>987.15586819601197</v>
+      </c>
+      <c r="R15">
+        <v>15618.4724861042</v>
+      </c>
+      <c r="S15">
+        <v>92.967098131572797</v>
+      </c>
+      <c r="T15">
+        <v>-2.5456367562447402</v>
+      </c>
+    </row>
+    <row r="16" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
+      </c>
+      <c r="D16">
+        <v>114550.946983783</v>
+      </c>
+      <c r="E16">
+        <v>282179.671291181</v>
+      </c>
+      <c r="F16">
+        <v>0.83671133512318097</v>
+      </c>
+      <c r="G16">
+        <v>21079.803315233199</v>
+      </c>
+      <c r="H16">
+        <v>6217.0342487801199</v>
+      </c>
+      <c r="I16">
+        <v>817.27332915015802</v>
+      </c>
+      <c r="J16">
+        <f>SUM(G16:I16)</f>
         <v>28114.110893163477</v>
       </c>
-      <c r="K15">
+      <c r="K16">
         <v>50843.189627163199</v>
       </c>
-      <c r="L15">
+      <c r="L16">
         <v>15303.8040979052</v>
       </c>
-      <c r="M15">
+      <c r="M16">
         <v>19297.531657665499</v>
       </c>
-      <c r="N15">
+      <c r="N16">
         <v>992.31070788561601</v>
       </c>
-      <c r="O15">
-        <v>0</v>
-      </c>
-      <c r="P15">
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16">
         <v>236102.92951066399</v>
       </c>
-      <c r="Q15">
+      <c r="Q16">
         <v>986.72714338313494</v>
       </c>
-      <c r="R15">
+      <c r="R16">
         <v>15669.8633517084</v>
       </c>
-      <c r="S15">
+      <c r="S16">
         <v>93.272996141121894</v>
       </c>
-      <c r="T15">
+      <c r="T16">
         <v>-0.19839357341549399</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A17" s="1" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A18" t="s">
-        <v>1</v>
-      </c>
-      <c r="B18" t="s">
-        <v>2</v>
-      </c>
-      <c r="C18" t="s">
-        <v>3</v>
-      </c>
-      <c r="D18" t="s">
-        <v>4</v>
-      </c>
-      <c r="E18" t="s">
-        <v>5</v>
-      </c>
-      <c r="F18" t="s">
-        <v>6</v>
-      </c>
-      <c r="G18" t="s">
-        <v>7</v>
-      </c>
-      <c r="H18" t="s">
-        <v>8</v>
-      </c>
-      <c r="I18" t="s">
-        <v>9</v>
-      </c>
-      <c r="J18" t="s">
-        <v>10</v>
-      </c>
-      <c r="K18" t="s">
-        <v>11</v>
-      </c>
-      <c r="L18" t="s">
-        <v>12</v>
-      </c>
-      <c r="M18" t="s">
-        <v>13</v>
-      </c>
-      <c r="N18" t="s">
-        <v>14</v>
-      </c>
-      <c r="O18" t="s">
-        <v>15</v>
-      </c>
-      <c r="P18" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q18" t="s">
-        <v>17</v>
-      </c>
-      <c r="R18" t="s">
-        <v>18</v>
-      </c>
-      <c r="S18" t="s">
-        <v>19</v>
-      </c>
-      <c r="T18" t="s">
-        <v>20</v>
+      <c r="A18" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>0</v>
       </c>
       <c r="B19" t="s">
-        <v>22</v>
-      </c>
-      <c r="C19">
+        <v>1</v>
+      </c>
+      <c r="C19" t="s">
+        <v>2</v>
+      </c>
+      <c r="D19" t="s">
+        <v>3</v>
+      </c>
+      <c r="E19" t="s">
         <v>4</v>
       </c>
-      <c r="D19">
-        <v>29525.427309999999</v>
-      </c>
-      <c r="E19">
-        <v>80391.755990000005</v>
-      </c>
-      <c r="F19">
-        <v>0.79280104200000001</v>
-      </c>
-      <c r="G19">
-        <v>5050.6365619999997</v>
-      </c>
-      <c r="H19">
-        <v>4678.3390820000004</v>
-      </c>
-      <c r="I19">
-        <v>2508.6600360000002</v>
-      </c>
-      <c r="J19">
-        <v>12237.635679999999</v>
-      </c>
-      <c r="K19">
-        <v>13920</v>
-      </c>
-      <c r="L19">
-        <v>2841.544922</v>
-      </c>
-      <c r="M19">
-        <v>5380.5444360000001</v>
-      </c>
-      <c r="N19">
-        <v>279.27307350000001</v>
-      </c>
-      <c r="O19">
-        <v>0</v>
-      </c>
-      <c r="P19">
-        <v>63734.6679</v>
-      </c>
-      <c r="Q19">
-        <v>1078.4492829999999</v>
-      </c>
-      <c r="R19">
-        <v>624.70352849999995</v>
-      </c>
-      <c r="S19">
-        <v>13.014656840000001</v>
-      </c>
-      <c r="T19">
-        <v>27.514184579999998</v>
+      <c r="F19" t="s">
+        <v>5</v>
+      </c>
+      <c r="G19" t="s">
+        <v>6</v>
+      </c>
+      <c r="H19" t="s">
+        <v>7</v>
+      </c>
+      <c r="I19" t="s">
+        <v>8</v>
+      </c>
+      <c r="J19" t="s">
+        <v>9</v>
+      </c>
+      <c r="K19" t="s">
+        <v>10</v>
+      </c>
+      <c r="L19" t="s">
+        <v>11</v>
+      </c>
+      <c r="M19" t="s">
+        <v>12</v>
+      </c>
+      <c r="N19" t="s">
+        <v>13</v>
+      </c>
+      <c r="O19" t="s">
+        <v>14</v>
+      </c>
+      <c r="P19" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q19" t="s">
+        <v>16</v>
+      </c>
+      <c r="R19" t="s">
+        <v>17</v>
+      </c>
+      <c r="S19" t="s">
+        <v>18</v>
+      </c>
+      <c r="T19" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C20">
         <v>4</v>
       </c>
       <c r="D20">
+        <v>29525.427309999999</v>
+      </c>
+      <c r="E20">
+        <v>80391.755990000005</v>
+      </c>
+      <c r="F20">
+        <v>0.79280104200000001</v>
+      </c>
+      <c r="G20">
+        <v>5050.6365619999997</v>
+      </c>
+      <c r="H20">
+        <v>4678.3390820000004</v>
+      </c>
+      <c r="I20">
+        <v>2508.6600360000002</v>
+      </c>
+      <c r="J20">
+        <v>12237.635679999999</v>
+      </c>
+      <c r="K20">
+        <v>13920</v>
+      </c>
+      <c r="L20">
+        <v>2841.544922</v>
+      </c>
+      <c r="M20">
+        <v>5380.5444360000001</v>
+      </c>
+      <c r="N20">
+        <v>279.27307350000001</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q20">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R20">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S20">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T20">
+        <v>27.514184579999998</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21">
+        <v>4</v>
+      </c>
+      <c r="D21">
         <v>30655.78772</v>
       </c>
-      <c r="E20">
+      <c r="E21">
         <v>79415.835619999998</v>
       </c>
-      <c r="F20">
+      <c r="F21">
         <v>0.81677700399999997</v>
       </c>
-      <c r="G20">
+      <c r="G21">
         <v>5129.9926729999997</v>
       </c>
-      <c r="H20">
+      <c r="H21">
         <v>5254.1641179999997</v>
       </c>
-      <c r="I20">
+      <c r="I21">
         <v>4834.2260249999999</v>
       </c>
-      <c r="J20">
+      <c r="J21">
         <v>15218.382820000001</v>
       </c>
-      <c r="K20">
+      <c r="K21">
         <v>13875.1543</v>
       </c>
-      <c r="L20">
+      <c r="L21">
         <v>3140.6678670000001</v>
       </c>
-      <c r="M20">
+      <c r="M21">
         <v>5340.9854210000003</v>
       </c>
-      <c r="N20">
+      <c r="N21">
         <v>286.5902719</v>
       </c>
-      <c r="O20">
-        <v>0</v>
-      </c>
-      <c r="P20">
+      <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="P21">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q20">
+      <c r="Q21">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R20">
+      <c r="R21">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S20">
+      <c r="S21">
         <v>452.7322633</v>
       </c>
-      <c r="T20">
+      <c r="T21">
         <v>5.8154128590000003</v>
       </c>
     </row>

</xml_diff>

<commit_message>
summer week with plant op mode's fixed for first four days to improve solve time
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{647054F9-5F24-4198-8BE9-ADF689C7AD81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07403044-1417-41C1-8CB4-B55F621EADFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -32,8 +32,35 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={9CE96C07-E110-41BE-B453-65310D0A2128}</author>
+    <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
+  </authors>
+  <commentList>
+    <comment ref="A15" authorId="0" shapeId="0" xr:uid="{9CE96C07-E110-41BE-B453-65310D0A2128}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Summer is the summer hot weekdays + high weekends.</t>
+      </text>
+    </comment>
+    <comment ref="A16" authorId="1" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Winter is low winter weekdays + low weekends</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="31">
   <si>
     <t>Season</t>
   </si>
@@ -123,13 +150,16 @@
   </si>
   <si>
     <t>TIME PERIOD = 1 WEEK, Rate = TOU 3</t>
+  </si>
+  <si>
+    <t>Maximum Power</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -263,6 +293,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -665,6 +701,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="Churchill, Jake" id="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" userId="S::rchurchi@nrel.gov::24b6a320-1211-4379-9513-990e66715a0d" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -982,9 +1024,20 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A15" dT="2026-05-27T21:41:37.20" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9CE96C07-E110-41BE-B453-65310D0A2128}">
+    <text>Summer is the summer hot weekdays + high weekends.</text>
+  </threadedComment>
+  <threadedComment ref="A16" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <text>Winter is low winter weekdays + low weekends</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:U21"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
+  <dimension ref="A1:U25"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.4">
@@ -1042,7 +1095,7 @@
         <v>15</v>
       </c>
       <c r="Q2" t="s">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="R2" t="s">
         <v>17</v>
@@ -1802,199 +1855,200 @@
         <v>-0.19839357341549399</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A18" s="1" t="s">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A22" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A19" t="s">
-        <v>0</v>
-      </c>
-      <c r="B19" t="s">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B23" t="s">
         <v>1</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C23" t="s">
         <v>2</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D23" t="s">
         <v>3</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E23" t="s">
         <v>4</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F23" t="s">
         <v>5</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G23" t="s">
         <v>6</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H23" t="s">
         <v>7</v>
       </c>
-      <c r="I19" t="s">
+      <c r="I23" t="s">
         <v>8</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J23" t="s">
         <v>9</v>
       </c>
-      <c r="K19" t="s">
+      <c r="K23" t="s">
         <v>10</v>
       </c>
-      <c r="L19" t="s">
+      <c r="L23" t="s">
         <v>11</v>
       </c>
-      <c r="M19" t="s">
+      <c r="M23" t="s">
         <v>12</v>
       </c>
-      <c r="N19" t="s">
+      <c r="N23" t="s">
         <v>13</v>
       </c>
-      <c r="O19" t="s">
+      <c r="O23" t="s">
         <v>14</v>
       </c>
-      <c r="P19" t="s">
+      <c r="P23" t="s">
         <v>15</v>
       </c>
-      <c r="Q19" t="s">
+      <c r="Q23" t="s">
         <v>16</v>
       </c>
-      <c r="R19" t="s">
+      <c r="R23" t="s">
         <v>17</v>
       </c>
-      <c r="S19" t="s">
+      <c r="S23" t="s">
         <v>18</v>
       </c>
-      <c r="T19" t="s">
+      <c r="T23" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A20" t="s">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
         <v>20</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B24" t="s">
         <v>21</v>
       </c>
-      <c r="C20">
+      <c r="C24">
         <v>4</v>
       </c>
-      <c r="D20">
+      <c r="D24">
         <v>29525.427309999999</v>
       </c>
-      <c r="E20">
+      <c r="E24">
         <v>80391.755990000005</v>
       </c>
-      <c r="F20">
+      <c r="F24">
         <v>0.79280104200000001</v>
       </c>
-      <c r="G20">
+      <c r="G24">
         <v>5050.6365619999997</v>
       </c>
-      <c r="H20">
+      <c r="H24">
         <v>4678.3390820000004</v>
       </c>
-      <c r="I20">
+      <c r="I24">
         <v>2508.6600360000002</v>
       </c>
-      <c r="J20">
+      <c r="J24">
         <v>12237.635679999999</v>
       </c>
-      <c r="K20">
+      <c r="K24">
         <v>13920</v>
       </c>
-      <c r="L20">
+      <c r="L24">
         <v>2841.544922</v>
       </c>
-      <c r="M20">
+      <c r="M24">
         <v>5380.5444360000001</v>
       </c>
-      <c r="N20">
+      <c r="N24">
         <v>279.27307350000001</v>
       </c>
-      <c r="O20">
-        <v>0</v>
-      </c>
-      <c r="P20">
+      <c r="O24">
+        <v>0</v>
+      </c>
+      <c r="P24">
         <v>63734.6679</v>
       </c>
-      <c r="Q20">
+      <c r="Q24">
         <v>1078.4492829999999</v>
       </c>
-      <c r="R20">
+      <c r="R24">
         <v>624.70352849999995</v>
       </c>
-      <c r="S20">
+      <c r="S24">
         <v>13.014656840000001</v>
       </c>
-      <c r="T20">
+      <c r="T24">
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A21" t="s">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A25" t="s">
         <v>23</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B25" t="s">
         <v>21</v>
       </c>
-      <c r="C21">
+      <c r="C25">
         <v>4</v>
       </c>
-      <c r="D21">
+      <c r="D25">
         <v>30655.78772</v>
       </c>
-      <c r="E21">
+      <c r="E25">
         <v>79415.835619999998</v>
       </c>
-      <c r="F21">
+      <c r="F25">
         <v>0.81677700399999997</v>
       </c>
-      <c r="G21">
+      <c r="G25">
         <v>5129.9926729999997</v>
       </c>
-      <c r="H21">
+      <c r="H25">
         <v>5254.1641179999997</v>
       </c>
-      <c r="I21">
+      <c r="I25">
         <v>4834.2260249999999</v>
       </c>
-      <c r="J21">
+      <c r="J25">
         <v>15218.382820000001</v>
       </c>
-      <c r="K21">
+      <c r="K25">
         <v>13875.1543</v>
       </c>
-      <c r="L21">
+      <c r="L25">
         <v>3140.6678670000001</v>
       </c>
-      <c r="M21">
+      <c r="M25">
         <v>5340.9854210000003</v>
       </c>
-      <c r="N21">
+      <c r="N25">
         <v>286.5902719</v>
       </c>
-      <c r="O21">
-        <v>0</v>
-      </c>
-      <c r="P21">
+      <c r="O25">
+        <v>0</v>
+      </c>
+      <c r="P25">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q21">
+      <c r="Q25">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R21">
+      <c r="R25">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S21">
+      <c r="S25">
         <v>452.7322633</v>
       </c>
-      <c r="T21">
+      <c r="T25">
         <v>5.8154128590000003</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Set for results for all number of flexible trains with TOU 3 rate
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{07403044-1417-41C1-8CB4-B55F621EADFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE67A1F-12CD-4554-967D-5280A2DFBACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
   </authors>
   <commentList>
-    <comment ref="A15" authorId="0" shapeId="0" xr:uid="{9CE96C07-E110-41BE-B453-65310D0A2128}">
+    <comment ref="A17" authorId="0" shapeId="0" xr:uid="{9CE96C07-E110-41BE-B453-65310D0A2128}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -47,7 +47,7 @@
     Summer is the summer hot weekdays + high weekends.</t>
       </text>
     </comment>
-    <comment ref="A16" authorId="1" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A18" authorId="1" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="31">
   <si>
     <t>Season</t>
   </si>
@@ -159,7 +159,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -293,12 +293,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1026,10 +1020,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A15" dT="2026-05-27T21:41:37.20" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9CE96C07-E110-41BE-B453-65310D0A2128}">
+  <threadedComment ref="A17" dT="2026-05-27T21:41:37.20" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9CE96C07-E110-41BE-B453-65310D0A2128}">
     <text>Summer is the summer hot weekdays + high weekends.</text>
   </threadedComment>
-  <threadedComment ref="A16" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+  <threadedComment ref="A18" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
     <text>Winter is low winter weekdays + low weekends</text>
   </threadedComment>
 </ThreadedComments>
@@ -1037,7 +1031,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:U25"/>
+  <dimension ref="A1:U27"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <sheetData>
     <row r="1" spans="1:21" x14ac:dyDescent="0.4">
@@ -1724,325 +1718,445 @@
         <v>0.68036269900000002</v>
       </c>
     </row>
-    <row r="14" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A14" s="1" t="s">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="A16" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="15" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A15" t="s">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A17" t="s">
         <v>23</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B17" t="s">
         <v>24</v>
       </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15">
+      <c r="C17">
+        <v>0</v>
+      </c>
+      <c r="D17">
         <v>177048.079214225</v>
       </c>
-      <c r="E15">
+      <c r="E17">
         <v>282179.697150969</v>
       </c>
-      <c r="F15">
+      <c r="F17">
         <v>1.0581911624256699</v>
       </c>
-      <c r="G15">
+      <c r="G17">
         <v>79845.342667291203</v>
       </c>
-      <c r="H15">
+      <c r="H17">
         <v>6222.1442638440503</v>
       </c>
-      <c r="I15">
+      <c r="I17">
         <v>4534.7814140862702</v>
       </c>
-      <c r="J15">
-        <f>SUM(G15:I15)</f>
+      <c r="J17">
+        <f>SUM(G17:I17)</f>
         <v>90602.268345221528</v>
       </c>
-      <c r="K15">
+      <c r="K17">
         <v>50847.265569999399</v>
       </c>
-      <c r="L15">
+      <c r="L17">
         <v>15307.856370494001</v>
       </c>
-      <c r="M15">
+      <c r="M17">
         <v>19298.378220313502</v>
       </c>
-      <c r="N15">
+      <c r="N17">
         <v>992.31070819735999</v>
       </c>
-      <c r="O15">
-        <v>0</v>
-      </c>
-      <c r="P15">
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17">
         <v>298600.06174110703</v>
       </c>
-      <c r="Q15">
+      <c r="Q17">
         <v>987.15586819601197</v>
       </c>
-      <c r="R15">
+      <c r="R17">
         <v>15618.4724861042</v>
       </c>
-      <c r="S15">
+      <c r="S17">
         <v>92.967098131572797</v>
       </c>
-      <c r="T15">
+      <c r="T17">
         <v>-2.5456367562447402</v>
       </c>
     </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A16" t="s">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
         <v>20</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B18" t="s">
         <v>24</v>
       </c>
-      <c r="C16">
-        <v>0</v>
-      </c>
-      <c r="D16">
+      <c r="C18">
+        <v>0</v>
+      </c>
+      <c r="D18">
         <v>114550.946983783</v>
       </c>
-      <c r="E16">
+      <c r="E18">
         <v>282179.671291181</v>
       </c>
-      <c r="F16">
+      <c r="F18">
         <v>0.83671133512318097</v>
       </c>
-      <c r="G16">
+      <c r="G18">
         <v>21079.803315233199</v>
       </c>
-      <c r="H16">
+      <c r="H18">
         <v>6217.0342487801199</v>
       </c>
-      <c r="I16">
+      <c r="I18">
         <v>817.27332915015802</v>
       </c>
-      <c r="J16">
-        <f>SUM(G16:I16)</f>
+      <c r="J18">
+        <f>SUM(G18:I18)</f>
         <v>28114.110893163477</v>
       </c>
-      <c r="K16">
+      <c r="K18">
         <v>50843.189627163199</v>
       </c>
-      <c r="L16">
+      <c r="L18">
         <v>15303.8040979052</v>
       </c>
-      <c r="M16">
+      <c r="M18">
         <v>19297.531657665499</v>
       </c>
-      <c r="N16">
+      <c r="N18">
         <v>992.31070788561601</v>
       </c>
-      <c r="O16">
-        <v>0</v>
-      </c>
-      <c r="P16">
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18">
         <v>236102.92951066399</v>
       </c>
-      <c r="Q16">
+      <c r="Q18">
         <v>986.72714338313494</v>
       </c>
-      <c r="R16">
+      <c r="R18">
         <v>15669.8633517084</v>
       </c>
-      <c r="S16">
+      <c r="S18">
         <v>93.272996141121894</v>
       </c>
-      <c r="T16">
+      <c r="T18">
         <v>-0.19839357341549399</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A22" s="1" t="s">
-        <v>27</v>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>20</v>
+      </c>
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19">
+        <v>4</v>
+      </c>
+      <c r="D19">
+        <v>108960.613539453</v>
+      </c>
+      <c r="E19">
+        <v>282179.67123287701</v>
+      </c>
+      <c r="F19">
+        <v>0.81690008021909599</v>
+      </c>
+      <c r="G19">
+        <v>23571.632136721099</v>
+      </c>
+      <c r="H19">
+        <v>6951.9409028971204</v>
+      </c>
+      <c r="I19">
+        <v>913.88179307768496</v>
+      </c>
+      <c r="J19">
+        <f>SUM(G19:I19)</f>
+        <v>31437.454832695905</v>
+      </c>
+      <c r="K19">
+        <v>48809.460212750702</v>
+      </c>
+      <c r="L19">
+        <v>9838.1656916422507</v>
+      </c>
+      <c r="M19">
+        <v>18875.532802364902</v>
+      </c>
+      <c r="N19">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>230512.59606633501</v>
+      </c>
+      <c r="Q19">
+        <v>1103.3673370121001</v>
+      </c>
+      <c r="R19">
+        <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A23" t="s">
-        <v>0</v>
-      </c>
-      <c r="B23" t="s">
-        <v>1</v>
-      </c>
-      <c r="C23" t="s">
-        <v>2</v>
-      </c>
-      <c r="D23" t="s">
-        <v>3</v>
-      </c>
-      <c r="E23" t="s">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A20" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" t="s">
+        <v>21</v>
+      </c>
+      <c r="C20">
         <v>4</v>
       </c>
-      <c r="F23" t="s">
-        <v>5</v>
-      </c>
-      <c r="G23" t="s">
-        <v>6</v>
-      </c>
-      <c r="H23" t="s">
-        <v>7</v>
-      </c>
-      <c r="I23" t="s">
-        <v>8</v>
-      </c>
-      <c r="J23" t="s">
-        <v>9</v>
-      </c>
-      <c r="K23" t="s">
-        <v>10</v>
-      </c>
-      <c r="L23" t="s">
-        <v>11</v>
-      </c>
-      <c r="M23" t="s">
-        <v>12</v>
-      </c>
-      <c r="N23" t="s">
-        <v>13</v>
-      </c>
-      <c r="O23" t="s">
-        <v>14</v>
-      </c>
-      <c r="P23" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q23" t="s">
-        <v>16</v>
-      </c>
-      <c r="R23" t="s">
-        <v>17</v>
-      </c>
-      <c r="S23" t="s">
-        <v>18</v>
-      </c>
-      <c r="T23" t="s">
-        <v>19</v>
+      <c r="D20">
+        <v>113598.307758221</v>
+      </c>
+      <c r="E20">
+        <v>282179.67123287398</v>
+      </c>
+      <c r="F20">
+        <v>0.83333533297315499</v>
+      </c>
+      <c r="G20">
+        <v>21005.263452339499</v>
+      </c>
+      <c r="H20">
+        <v>9419.1929847336105</v>
+      </c>
+      <c r="I20">
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <f>SUM(G20:I20)</f>
+        <v>30424.45643707311</v>
+      </c>
+      <c r="K20">
+        <v>48819.627456497903</v>
+      </c>
+      <c r="L20">
+        <v>14784.690159207899</v>
+      </c>
+      <c r="M20">
+        <v>19569.533705442402</v>
+      </c>
+      <c r="N20">
+        <v>1040.9289460857101</v>
+      </c>
+      <c r="O20">
+        <v>0</v>
+      </c>
+      <c r="P20">
+        <v>235150.29028510299</v>
+      </c>
+      <c r="Q20">
+        <v>1494.95371016114</v>
+      </c>
+      <c r="R20">
+        <v>40078.803663142098</v>
+      </c>
+      <c r="S20">
+        <v>910.88190143504903</v>
+      </c>
+      <c r="T20">
+        <v>0.51068072492979899</v>
       </c>
     </row>
     <row r="24" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A24" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" t="s">
-        <v>21</v>
-      </c>
-      <c r="C24">
-        <v>4</v>
-      </c>
-      <c r="D24">
-        <v>29525.427309999999</v>
-      </c>
-      <c r="E24">
-        <v>80391.755990000005</v>
-      </c>
-      <c r="F24">
-        <v>0.79280104200000001</v>
-      </c>
-      <c r="G24">
-        <v>5050.6365619999997</v>
-      </c>
-      <c r="H24">
-        <v>4678.3390820000004</v>
-      </c>
-      <c r="I24">
-        <v>2508.6600360000002</v>
-      </c>
-      <c r="J24">
-        <v>12237.635679999999</v>
-      </c>
-      <c r="K24">
-        <v>13920</v>
-      </c>
-      <c r="L24">
-        <v>2841.544922</v>
-      </c>
-      <c r="M24">
-        <v>5380.5444360000001</v>
-      </c>
-      <c r="N24">
-        <v>279.27307350000001</v>
-      </c>
-      <c r="O24">
-        <v>0</v>
-      </c>
-      <c r="P24">
-        <v>63734.6679</v>
-      </c>
-      <c r="Q24">
-        <v>1078.4492829999999</v>
-      </c>
-      <c r="R24">
-        <v>624.70352849999995</v>
-      </c>
-      <c r="S24">
-        <v>13.014656840000001</v>
-      </c>
-      <c r="T24">
-        <v>27.514184579999998</v>
+      <c r="A24" s="1" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="25" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
+        <v>0</v>
+      </c>
+      <c r="B25" t="s">
+        <v>1</v>
+      </c>
+      <c r="C25" t="s">
+        <v>2</v>
+      </c>
+      <c r="D25" t="s">
+        <v>3</v>
+      </c>
+      <c r="E25" t="s">
+        <v>4</v>
+      </c>
+      <c r="F25" t="s">
+        <v>5</v>
+      </c>
+      <c r="G25" t="s">
+        <v>6</v>
+      </c>
+      <c r="H25" t="s">
+        <v>7</v>
+      </c>
+      <c r="I25" t="s">
+        <v>8</v>
+      </c>
+      <c r="J25" t="s">
+        <v>9</v>
+      </c>
+      <c r="K25" t="s">
+        <v>10</v>
+      </c>
+      <c r="L25" t="s">
+        <v>11</v>
+      </c>
+      <c r="M25" t="s">
+        <v>12</v>
+      </c>
+      <c r="N25" t="s">
+        <v>13</v>
+      </c>
+      <c r="O25" t="s">
+        <v>14</v>
+      </c>
+      <c r="P25" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q25" t="s">
+        <v>16</v>
+      </c>
+      <c r="R25" t="s">
+        <v>17</v>
+      </c>
+      <c r="S25" t="s">
+        <v>18</v>
+      </c>
+      <c r="T25" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A26" t="s">
+        <v>20</v>
+      </c>
+      <c r="B26" t="s">
+        <v>21</v>
+      </c>
+      <c r="C26">
+        <v>4</v>
+      </c>
+      <c r="D26">
+        <v>29525.427309999999</v>
+      </c>
+      <c r="E26">
+        <v>80391.755990000005</v>
+      </c>
+      <c r="F26">
+        <v>0.79280104200000001</v>
+      </c>
+      <c r="G26">
+        <v>5050.6365619999997</v>
+      </c>
+      <c r="H26">
+        <v>4678.3390820000004</v>
+      </c>
+      <c r="I26">
+        <v>2508.6600360000002</v>
+      </c>
+      <c r="J26">
+        <v>12237.635679999999</v>
+      </c>
+      <c r="K26">
+        <v>13920</v>
+      </c>
+      <c r="L26">
+        <v>2841.544922</v>
+      </c>
+      <c r="M26">
+        <v>5380.5444360000001</v>
+      </c>
+      <c r="N26">
+        <v>279.27307350000001</v>
+      </c>
+      <c r="O26">
+        <v>0</v>
+      </c>
+      <c r="P26">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q26">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R26">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S26">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T26">
+        <v>27.514184579999998</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A27" t="s">
         <v>23</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B27" t="s">
         <v>21</v>
       </c>
-      <c r="C25">
+      <c r="C27">
         <v>4</v>
       </c>
-      <c r="D25">
+      <c r="D27">
         <v>30655.78772</v>
       </c>
-      <c r="E25">
+      <c r="E27">
         <v>79415.835619999998</v>
       </c>
-      <c r="F25">
+      <c r="F27">
         <v>0.81677700399999997</v>
       </c>
-      <c r="G25">
+      <c r="G27">
         <v>5129.9926729999997</v>
       </c>
-      <c r="H25">
+      <c r="H27">
         <v>5254.1641179999997</v>
       </c>
-      <c r="I25">
+      <c r="I27">
         <v>4834.2260249999999</v>
       </c>
-      <c r="J25">
+      <c r="J27">
         <v>15218.382820000001</v>
       </c>
-      <c r="K25">
+      <c r="K27">
         <v>13875.1543</v>
       </c>
-      <c r="L25">
+      <c r="L27">
         <v>3140.6678670000001</v>
       </c>
-      <c r="M25">
+      <c r="M27">
         <v>5340.9854210000003</v>
       </c>
-      <c r="N25">
+      <c r="N27">
         <v>286.5902719</v>
       </c>
-      <c r="O25">
-        <v>0</v>
-      </c>
-      <c r="P25">
+      <c r="O27">
+        <v>0</v>
+      </c>
+      <c r="P27">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q25">
+      <c r="Q27">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R25">
+      <c r="R27">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S25">
+      <c r="S27">
         <v>452.7322633</v>
       </c>
-      <c r="T25">
+      <c r="T27">
         <v>5.8154128590000003</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Changed the uf recovery to always be fixed.
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CE67A1F-12CD-4554-967D-5280A2DFBACF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAC0585A-C9E4-4D65-BA13-A6B2D40A7502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57495" yWindow="8550" windowWidth="14610" windowHeight="15585" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
   </authors>
   <commentList>
-    <comment ref="A17" authorId="0" shapeId="0" xr:uid="{9CE96C07-E110-41BE-B453-65310D0A2128}">
+    <comment ref="A21" authorId="0" shapeId="0" xr:uid="{9CE96C07-E110-41BE-B453-65310D0A2128}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -47,7 +47,7 @@
     Summer is the summer hot weekdays + high weekends.</t>
       </text>
     </comment>
-    <comment ref="A18" authorId="1" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A22" authorId="1" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="30">
   <si>
     <t>Season</t>
   </si>
@@ -126,9 +126,6 @@
   </si>
   <si>
     <t>both</t>
-  </si>
-  <si>
-    <t>&gt; have to rerun as LVOF formula was incorrect</t>
   </si>
   <si>
     <t>summer</t>
@@ -1020,10 +1017,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A17" dT="2026-05-27T21:41:37.20" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9CE96C07-E110-41BE-B453-65310D0A2128}">
+  <threadedComment ref="A21" dT="2026-05-27T21:41:37.20" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9CE96C07-E110-41BE-B453-65310D0A2128}">
     <text>Summer is the summer hot weekdays + high weekends.</text>
   </threadedComment>
-  <threadedComment ref="A18" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+  <threadedComment ref="A22" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
     <text>Winter is low winter weekdays + low weekends</text>
   </threadedComment>
 </ThreadedComments>
@@ -1031,15 +1028,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:U27"/>
+  <dimension ref="A1:T30"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="3" max="3" width="14.23046875" customWidth="1"/>
+    <col min="5" max="5" width="10.3046875" customWidth="1"/>
+    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.53515625" customWidth="1"/>
+    <col min="9" max="9" width="9.07421875" customWidth="1"/>
+    <col min="20" max="20" width="7.84375" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="2" spans="1:21" x14ac:dyDescent="0.4">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="2" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1089,7 +1094,7 @@
         <v>15</v>
       </c>
       <c r="Q2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="R2" t="s">
         <v>17</v>
@@ -1101,196 +1106,119 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>20</v>
       </c>
       <c r="B3" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>103692.5996</v>
+        <v>111737.917851103</v>
       </c>
       <c r="E3">
-        <v>282180.92219999997</v>
+        <v>282179.67125484499</v>
       </c>
       <c r="F3">
-        <v>0.79822753599999996</v>
+        <v>0.826742406143402</v>
       </c>
       <c r="G3">
-        <v>17807.339960000001</v>
+        <v>18663.290146715601</v>
       </c>
       <c r="H3">
-        <v>4786.7821690000001</v>
+        <v>4963.6224309139197</v>
       </c>
       <c r="I3">
-        <v>2570.2005570000001</v>
+        <v>2666.4923762402</v>
       </c>
       <c r="J3">
-        <v>25164.322690000001</v>
+        <v>26293.4049538697</v>
       </c>
       <c r="K3">
-        <v>48812.876550000001</v>
+        <v>50843.184012302001</v>
       </c>
       <c r="L3">
-        <v>9846.8091789999999</v>
+        <v>15303.798393478701</v>
       </c>
       <c r="M3">
-        <v>18876.280470000002</v>
+        <v>19297.530491452799</v>
       </c>
       <c r="N3">
-        <v>992.31070790000001</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
       <c r="P3">
-        <v>225244.5821</v>
+        <v>233289.900377985</v>
       </c>
       <c r="Q3">
-        <v>1086.928874</v>
+        <v>1127.0837800240299</v>
       </c>
       <c r="R3">
-        <v>160.26157760000001</v>
-      </c>
-      <c r="S3">
-        <v>6.9678946799999997</v>
-      </c>
-      <c r="T3">
-        <v>466.95526849999999</v>
-      </c>
-      <c r="U3" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A4" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
+      <c r="B4" t="s">
         <v>23</v>
       </c>
-      <c r="B4" t="s">
-        <v>21</v>
-      </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4">
-        <v>112836.8172</v>
+        <v>120897.164660582</v>
       </c>
       <c r="E4">
-        <v>282179.67129999999</v>
+        <v>282179.67125255102</v>
       </c>
       <c r="F4">
-        <v>0.83063673100000002</v>
+        <v>0.85920132414667005</v>
       </c>
       <c r="G4">
-        <v>20374.552169999999</v>
+        <v>21103.178564432201</v>
       </c>
       <c r="H4">
-        <v>4898.9862890000004</v>
+        <v>5044.5785543711099</v>
       </c>
       <c r="I4">
-        <v>9033.9920129999991</v>
+        <v>9304.8946454247507</v>
       </c>
       <c r="J4">
-        <v>34307.530469999998</v>
+        <v>35452.651764228103</v>
       </c>
       <c r="K4">
-        <v>48813.007669999999</v>
+        <v>50843.1840118412</v>
       </c>
       <c r="L4">
-        <v>9847.699482</v>
+        <v>15303.7983932269</v>
       </c>
       <c r="M4">
-        <v>18876.268899999999</v>
+        <v>19297.530491286099</v>
       </c>
       <c r="N4">
-        <v>992.31070790000001</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
       <c r="P4">
-        <v>234388.79980000001</v>
+        <v>242449.147187464</v>
       </c>
       <c r="Q4">
-        <v>1094.554862</v>
+        <v>1127.0837796179201</v>
       </c>
       <c r="R4">
-        <v>20.456524869999999</v>
-      </c>
-      <c r="S4">
-        <v>2.5570656089999999</v>
-      </c>
-      <c r="T4">
-        <v>3211.2873840000002</v>
-      </c>
-    </row>
-    <row r="5" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5">
-        <v>111442.0141</v>
-      </c>
-      <c r="E5">
-        <v>282179.67119999998</v>
-      </c>
-      <c r="F5">
-        <v>0.82569376999999999</v>
-      </c>
-      <c r="G5">
-        <v>17692.481769999999</v>
-      </c>
-      <c r="H5">
-        <v>4757.593132</v>
-      </c>
-      <c r="I5">
-        <v>2555.1155720000002</v>
-      </c>
-      <c r="J5">
-        <v>25005.190470000001</v>
-      </c>
-      <c r="K5">
-        <v>50843.184009999997</v>
-      </c>
-      <c r="L5">
-        <v>15303.79839</v>
-      </c>
-      <c r="M5">
-        <v>19297.530490000001</v>
-      </c>
-      <c r="N5">
-        <v>992.31070790000001</v>
-      </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
-      <c r="P5">
-        <v>232993.99660000001</v>
-      </c>
-      <c r="Q5">
-        <v>1080.3009549999999</v>
-      </c>
-      <c r="R5">
-        <v>359.38311010000001</v>
-      </c>
-      <c r="S5">
-        <v>10.268088860000001</v>
-      </c>
-      <c r="T5">
-        <v>208.67458189999999</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1301,862 +1229,818 @@
         <v>0</v>
       </c>
       <c r="D6">
-        <v>137194.4558</v>
+        <v>111179.352715972</v>
       </c>
       <c r="E6">
-        <v>374196.25630000001</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F6">
-        <v>0.69147254700000005</v>
+        <v>0.82476293995957695</v>
       </c>
       <c r="G6">
-        <v>23651.266039999999</v>
+        <v>18266.8157113575</v>
       </c>
       <c r="H6">
-        <v>6338.5673459999998</v>
+        <v>4858.1774967593901</v>
       </c>
       <c r="I6">
-        <v>3404.7859779999999</v>
+        <v>2609.8466266994801</v>
       </c>
       <c r="J6">
-        <v>33394.619359999997</v>
+        <v>25734.839834816299</v>
       </c>
       <c r="K6">
-        <v>64727.042860000001</v>
+        <v>50843.184005923897</v>
       </c>
       <c r="L6">
-        <v>13049.5375</v>
+        <v>15303.798385783701</v>
       </c>
       <c r="M6">
-        <v>25030.945339999998</v>
+        <v>19297.530489448302</v>
       </c>
       <c r="N6">
-        <v>992.31070790000001</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
       <c r="P6">
-        <v>258746.43830000001</v>
+        <v>232731.33524285399</v>
       </c>
       <c r="Q6">
-        <v>1439.29087</v>
+        <v>1103.1405255510299</v>
       </c>
       <c r="R6">
         <v>0</v>
       </c>
-      <c r="S6">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:21" x14ac:dyDescent="0.4">
+    </row>
+    <row r="7" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C7">
         <v>0</v>
       </c>
       <c r="D7">
-        <v>111441.1241</v>
+        <v>103268.55989110901</v>
       </c>
       <c r="E7">
-        <v>282179.67129999999</v>
+        <v>282179.79409919202</v>
       </c>
       <c r="F7">
-        <v>0.82569061600000004</v>
+        <v>0.79672799796204397</v>
       </c>
       <c r="G7">
-        <v>17691.850109999999</v>
+        <v>18267.443429751202</v>
       </c>
       <c r="H7">
-        <v>4757.4251000000004</v>
+        <v>4858.6111494831202</v>
       </c>
       <c r="I7">
-        <v>2555.0253269999998</v>
+        <v>2610.0795879488901</v>
       </c>
       <c r="J7">
-        <v>25004.30054</v>
+        <v>25736.1341671833</v>
       </c>
       <c r="K7">
-        <v>50843.184009999997</v>
+        <v>48811.852007574802</v>
       </c>
       <c r="L7">
-        <v>15303.79839</v>
+        <v>9844.5408077047105</v>
       </c>
       <c r="M7">
-        <v>19297.530490000001</v>
+        <v>18876.032908646699</v>
       </c>
       <c r="N7">
-        <v>992.31070790000001</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
       <c r="P7">
-        <v>232993.1067</v>
+        <v>224820.542417991</v>
       </c>
       <c r="Q7">
-        <v>1080.2628</v>
+        <v>1103.23899455419</v>
       </c>
       <c r="R7">
-        <v>360.71821890000001</v>
-      </c>
-      <c r="S7">
-        <v>10.306234829999999</v>
-      </c>
-      <c r="T7">
-        <v>207.90469189999999</v>
-      </c>
-    </row>
-    <row r="8" spans="1:21" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C8">
         <v>0</v>
       </c>
       <c r="D8">
-        <v>120218.63830000001</v>
+        <v>103268.55989110901</v>
       </c>
       <c r="E8">
-        <v>282179.67119999998</v>
+        <v>282179.79409919202</v>
       </c>
       <c r="F8">
-        <v>0.856796734</v>
+        <v>0.79672799796204397</v>
       </c>
       <c r="G8">
-        <v>20036.014340000002</v>
+        <v>18267.443429751202</v>
       </c>
       <c r="H8">
-        <v>4832.3564850000002</v>
+        <v>4858.6111494831202</v>
       </c>
       <c r="I8">
-        <v>8913.4439079999993</v>
+        <v>2610.0795879488901</v>
       </c>
       <c r="J8">
-        <v>33781.814729999998</v>
+        <v>25736.1341671833</v>
       </c>
       <c r="K8">
-        <v>50843.184009999997</v>
+        <v>48811.852007574802</v>
       </c>
       <c r="L8">
-        <v>15303.79839</v>
+        <v>9844.5408077047105</v>
       </c>
       <c r="M8">
-        <v>19297.530490000001</v>
+        <v>18876.032908646699</v>
       </c>
       <c r="N8">
-        <v>992.31070790000001</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O8">
         <v>0</v>
       </c>
       <c r="P8">
-        <v>241770.6208</v>
+        <v>224820.542417991</v>
       </c>
       <c r="Q8">
-        <v>1079.6681140000001</v>
+        <v>1103.23899455419</v>
       </c>
       <c r="R8">
-        <v>863.44253030000004</v>
-      </c>
-      <c r="S8">
-        <v>9.5938058920000007</v>
-      </c>
-      <c r="T8">
-        <v>76.690102300000007</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A10" t="s">
+        <v>22</v>
+      </c>
+      <c r="B10" t="s">
         <v>25</v>
       </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9">
-        <v>148899.34179999999</v>
-      </c>
-      <c r="E9">
-        <v>374122.73599999998</v>
-      </c>
-      <c r="F9">
-        <v>0.72289464999999997</v>
-      </c>
-      <c r="G9">
-        <v>26811.872899999998</v>
-      </c>
-      <c r="H9">
-        <v>6422.7654039999998</v>
-      </c>
-      <c r="I9">
-        <v>11835.53282</v>
-      </c>
-      <c r="J9">
-        <v>45070.171119999999</v>
-      </c>
-      <c r="K9">
-        <v>64727.04277</v>
-      </c>
-      <c r="L9">
-        <v>13081.150960000001</v>
-      </c>
-      <c r="M9">
-        <v>25028.66619</v>
-      </c>
-      <c r="N9">
-        <v>992.31070790000001</v>
-      </c>
-      <c r="O9">
-        <v>0</v>
-      </c>
-      <c r="P9">
-        <v>270451.32429999998</v>
-      </c>
-      <c r="Q9">
-        <v>1435.0048529999999</v>
-      </c>
-      <c r="R9">
-        <v>0</v>
-      </c>
-      <c r="S9">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" t="s">
-        <v>26</v>
-      </c>
       <c r="C10">
         <v>0</v>
       </c>
       <c r="D10">
-        <v>120217.3988</v>
+        <v>120133.22940371701</v>
       </c>
       <c r="E10">
-        <v>282179.67119999998</v>
+        <v>282181.81222384499</v>
       </c>
       <c r="F10">
-        <v>0.85679234199999998</v>
+        <v>0.85648756036366303</v>
       </c>
       <c r="G10">
-        <v>20035.275740000001</v>
+        <v>20646.853340244099</v>
       </c>
       <c r="H10">
-        <v>4832.1803879999998</v>
+        <v>4935.5483613883198</v>
       </c>
       <c r="I10">
-        <v>8913.1190900000001</v>
+        <v>9103.7847909659795</v>
       </c>
       <c r="J10">
-        <v>33780.575219999999</v>
+        <v>34686.186492598397</v>
       </c>
       <c r="K10">
-        <v>50843.184009999997</v>
+        <v>50844.052885348698</v>
       </c>
       <c r="L10">
-        <v>15303.79839</v>
+        <v>15305.212873121</v>
       </c>
       <c r="M10">
-        <v>19297.530490000001</v>
+        <v>19297.777152649</v>
       </c>
       <c r="N10">
-        <v>992.31070790000001</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O10">
         <v>0</v>
       </c>
       <c r="P10">
-        <v>241769.38130000001</v>
+        <v>241685.21193059901</v>
       </c>
       <c r="Q10">
-        <v>1079.6287689999999</v>
+        <v>1102.72373433861</v>
       </c>
       <c r="R10">
-        <v>866.96784479999997</v>
-      </c>
-      <c r="S10">
-        <v>9.6329760540000002</v>
-      </c>
-      <c r="T10">
-        <v>76.379690299999993</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A11" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B11" t="s">
         <v>24</v>
       </c>
       <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>112735.91652453299</v>
+      </c>
+      <c r="E11">
+        <v>282179.67125392298</v>
+      </c>
+      <c r="F11">
+        <v>0.83027915515780504</v>
+      </c>
+      <c r="G11">
+        <v>20960.382547718</v>
+      </c>
+      <c r="H11">
+        <v>5010.4440999274602</v>
+      </c>
+      <c r="I11">
+        <v>9241.9323985477895</v>
+      </c>
+      <c r="J11">
+        <v>35212.7590461933</v>
+      </c>
+      <c r="K11">
+        <v>48809.459899526402</v>
+      </c>
+      <c r="L11">
+        <v>9838.1648407904995</v>
+      </c>
+      <c r="M11">
+        <v>18875.532738023201</v>
+      </c>
+      <c r="N11">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O11">
+        <v>0</v>
+      </c>
+      <c r="P11">
+        <v>234287.89905141501</v>
+      </c>
+      <c r="Q11">
+        <v>1119.4572971447301</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>112735.91652453299</v>
+      </c>
+      <c r="E12">
+        <v>282179.67125392298</v>
+      </c>
+      <c r="F12">
+        <v>0.83027915515780504</v>
+      </c>
+      <c r="G12">
+        <v>20960.382547718</v>
+      </c>
+      <c r="H12">
+        <v>5010.4440999274602</v>
+      </c>
+      <c r="I12">
+        <v>9241.9323985477895</v>
+      </c>
+      <c r="J12">
+        <v>35212.7590461933</v>
+      </c>
+      <c r="K12">
+        <v>48809.459899526402</v>
+      </c>
+      <c r="L12">
+        <v>9838.1648407904995</v>
+      </c>
+      <c r="M12">
+        <v>18875.532738023201</v>
+      </c>
+      <c r="N12">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O12">
+        <v>0</v>
+      </c>
+      <c r="P12">
+        <v>234287.89905141501</v>
+      </c>
+      <c r="Q12">
+        <v>1119.4572971447301</v>
+      </c>
+      <c r="R12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A14" t="s">
+        <v>20</v>
+      </c>
+      <c r="B14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C14">
         <v>2</v>
       </c>
-      <c r="D11">
-        <v>111441.11810000001</v>
-      </c>
-      <c r="E11">
-        <v>282179.67119999998</v>
-      </c>
-      <c r="F11">
-        <v>0.82569059499999997</v>
-      </c>
-      <c r="G11">
-        <v>17691.84577</v>
-      </c>
-      <c r="H11">
-        <v>4757.4239850000004</v>
-      </c>
-      <c r="I11">
-        <v>2555.0247060000002</v>
-      </c>
-      <c r="J11">
-        <v>25004.294460000001</v>
-      </c>
-      <c r="K11">
-        <v>50843.184009999997</v>
-      </c>
-      <c r="L11">
-        <v>15303.79839</v>
-      </c>
-      <c r="M11">
-        <v>19297.530490000001</v>
-      </c>
-      <c r="N11">
-        <v>992.31070790000001</v>
-      </c>
-      <c r="O11">
-        <v>0</v>
-      </c>
-      <c r="P11">
-        <v>232993.10060000001</v>
-      </c>
-      <c r="Q11">
-        <v>1080.262547</v>
-      </c>
-      <c r="R11">
-        <v>2069.5658520000002</v>
-      </c>
-      <c r="S11">
-        <v>12.542823350000001</v>
-      </c>
-      <c r="T11">
-        <v>4.9104200000000002E-4</v>
-      </c>
-    </row>
-    <row r="12" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
+    </row>
+    <row r="15" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A15" t="s">
+        <v>22</v>
+      </c>
+      <c r="B15" t="s">
         <v>23</v>
       </c>
-      <c r="B12" t="s">
-        <v>24</v>
-      </c>
-      <c r="C12">
+      <c r="C15">
         <v>2</v>
       </c>
-      <c r="D12">
-        <v>118535.91039999999</v>
-      </c>
-      <c r="E12">
-        <v>282179.67119999998</v>
-      </c>
-      <c r="F12">
-        <v>0.85083341400000001</v>
-      </c>
-      <c r="G12">
-        <v>19552.055189999999</v>
-      </c>
-      <c r="H12">
-        <v>6487.5388240000002</v>
-      </c>
-      <c r="I12">
-        <v>6025.9340460000003</v>
-      </c>
-      <c r="J12">
-        <v>32065.528060000001</v>
-      </c>
-      <c r="K12">
-        <v>50847.613210000003</v>
-      </c>
-      <c r="L12">
-        <v>15315.701870000001</v>
-      </c>
-      <c r="M12">
-        <v>19298.449550000001</v>
-      </c>
-      <c r="N12">
-        <v>1008.617701</v>
-      </c>
-      <c r="O12">
-        <v>0</v>
-      </c>
-      <c r="P12">
-        <v>240087.89290000001</v>
-      </c>
-      <c r="Q12">
-        <v>1449.4768389999999</v>
-      </c>
-      <c r="R12">
-        <v>27623.63321</v>
-      </c>
-      <c r="S12">
-        <v>317.5130254</v>
-      </c>
-      <c r="T12">
-        <v>0.68036269900000002</v>
-      </c>
-    </row>
-    <row r="16" spans="1:21" x14ac:dyDescent="0.4">
-      <c r="A16" s="1" t="s">
-        <v>28</v>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A16" t="s">
+        <v>20</v>
+      </c>
+      <c r="B16" t="s">
+        <v>21</v>
+      </c>
+      <c r="C16">
+        <v>4</v>
+      </c>
+      <c r="D16">
+        <v>103263.067623782</v>
+      </c>
+      <c r="E16">
+        <v>282179.67123287701</v>
+      </c>
+      <c r="F16">
+        <v>0.79670888114802996</v>
+      </c>
+      <c r="G16">
+        <v>18270.343045682599</v>
+      </c>
+      <c r="H16">
+        <v>4859.1187222275803</v>
+      </c>
+      <c r="I16">
+        <v>2610.3522592715499</v>
+      </c>
+      <c r="J16">
+        <v>25739.814027181699</v>
+      </c>
+      <c r="K16">
+        <v>48809.484574716203</v>
+      </c>
+      <c r="L16">
+        <v>9838.23116441202</v>
+      </c>
+      <c r="M16">
+        <v>18875.537857472798</v>
+      </c>
+      <c r="N16">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16">
+        <v>224815.050150664</v>
+      </c>
+      <c r="Q16">
+        <v>1103.3542485400801</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+      <c r="S16">
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <v>0</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A17" t="s">
+        <v>22</v>
+      </c>
+      <c r="B17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C17">
+        <v>4</v>
+      </c>
+      <c r="D17">
+        <v>108527.711286153</v>
+      </c>
+      <c r="E17">
+        <v>282179.67123319401</v>
+      </c>
+      <c r="F17">
+        <v>0.81536594329254797</v>
+      </c>
+      <c r="G17">
+        <v>19470.284119269101</v>
+      </c>
+      <c r="H17">
+        <v>5251.7861497213999</v>
+      </c>
+      <c r="I17">
+        <v>4921.3210739687102</v>
+      </c>
+      <c r="J17">
+        <v>29643.391342959199</v>
+      </c>
+      <c r="K17">
+        <v>49158.923944860697</v>
+      </c>
+      <c r="L17">
+        <v>10777.3494715455</v>
+      </c>
+      <c r="M17">
+        <v>18948.046526787599</v>
+      </c>
+      <c r="N17">
+        <v>1008.6177006503</v>
+      </c>
+      <c r="O17">
+        <v>0</v>
+      </c>
+      <c r="P17">
+        <v>230079.69381303401</v>
+      </c>
+      <c r="Q17">
+        <v>1173.3790798621201</v>
+      </c>
+      <c r="R17">
+        <v>12990.682952859001</v>
+      </c>
+      <c r="S17">
+        <v>463.95296260210699</v>
+      </c>
+      <c r="T17">
+        <v>1.63318791126541</v>
+      </c>
+    </row>
+    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A20" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
+        <v>22</v>
+      </c>
+      <c r="B21" t="s">
         <v>23</v>
       </c>
-      <c r="B17" t="s">
-        <v>24</v>
-      </c>
-      <c r="C17">
-        <v>0</v>
-      </c>
-      <c r="D17">
-        <v>177048.079214225</v>
-      </c>
-      <c r="E17">
-        <v>282179.697150969</v>
-      </c>
-      <c r="F17">
-        <v>1.0581911624256699</v>
-      </c>
-      <c r="G17">
-        <v>79845.342667291203</v>
-      </c>
-      <c r="H17">
-        <v>6222.1442638440503</v>
-      </c>
-      <c r="I17">
-        <v>4534.7814140862702</v>
-      </c>
-      <c r="J17">
-        <f>SUM(G17:I17)</f>
-        <v>90602.268345221528</v>
-      </c>
-      <c r="K17">
-        <v>50847.265569999399</v>
-      </c>
-      <c r="L17">
-        <v>15307.856370494001</v>
-      </c>
-      <c r="M17">
-        <v>19298.378220313502</v>
-      </c>
-      <c r="N17">
-        <v>992.31070819735999</v>
-      </c>
-      <c r="O17">
-        <v>0</v>
-      </c>
-      <c r="P17">
-        <v>298600.06174110703</v>
-      </c>
-      <c r="Q17">
-        <v>987.15586819601197</v>
-      </c>
-      <c r="R17">
-        <v>15618.4724861042</v>
-      </c>
-      <c r="S17">
-        <v>92.967098131572797</v>
-      </c>
-      <c r="T17">
-        <v>-2.5456367562447402</v>
-      </c>
-    </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A18" t="s">
+      <c r="C21">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A22" t="s">
         <v>20</v>
       </c>
-      <c r="B18" t="s">
-        <v>24</v>
-      </c>
-      <c r="C18">
-        <v>0</v>
-      </c>
-      <c r="D18">
-        <v>114550.946983783</v>
-      </c>
-      <c r="E18">
-        <v>282179.671291181</v>
-      </c>
-      <c r="F18">
-        <v>0.83671133512318097</v>
-      </c>
-      <c r="G18">
-        <v>21079.803315233199</v>
-      </c>
-      <c r="H18">
-        <v>6217.0342487801199</v>
-      </c>
-      <c r="I18">
-        <v>817.27332915015802</v>
-      </c>
-      <c r="J18">
-        <f>SUM(G18:I18)</f>
-        <v>28114.110893163477</v>
-      </c>
-      <c r="K18">
-        <v>50843.189627163199</v>
-      </c>
-      <c r="L18">
-        <v>15303.8040979052</v>
-      </c>
-      <c r="M18">
-        <v>19297.531657665499</v>
-      </c>
-      <c r="N18">
-        <v>992.31070788561601</v>
-      </c>
-      <c r="O18">
-        <v>0</v>
-      </c>
-      <c r="P18">
-        <v>236102.92951066399</v>
-      </c>
-      <c r="Q18">
-        <v>986.72714338313494</v>
-      </c>
-      <c r="R18">
-        <v>15669.8633517084</v>
-      </c>
-      <c r="S18">
-        <v>93.272996141121894</v>
-      </c>
-      <c r="T18">
-        <v>-0.19839357341549399</v>
-      </c>
-    </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A19" t="s">
+      <c r="B22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A23" t="s">
         <v>20</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B23" t="s">
         <v>21</v>
       </c>
-      <c r="C19">
+      <c r="C23">
         <v>4</v>
       </c>
-      <c r="D19">
+      <c r="D23">
         <v>108960.613539453</v>
       </c>
-      <c r="E19">
+      <c r="E23">
         <v>282179.67123287701</v>
       </c>
-      <c r="F19">
+      <c r="F23">
         <v>0.81690008021909599</v>
       </c>
-      <c r="G19">
+      <c r="G23">
         <v>23571.632136721099</v>
       </c>
-      <c r="H19">
+      <c r="H23">
         <v>6951.9409028971204</v>
       </c>
-      <c r="I19">
+      <c r="I23">
         <v>913.88179307768496</v>
       </c>
-      <c r="J19">
-        <f>SUM(G19:I19)</f>
+      <c r="J23">
+        <f>SUM(G23:I23)</f>
         <v>31437.454832695905</v>
       </c>
-      <c r="K19">
+      <c r="K23">
         <v>48809.460212750702</v>
       </c>
-      <c r="L19">
+      <c r="L23">
         <v>9838.1656916422507</v>
       </c>
-      <c r="M19">
+      <c r="M23">
         <v>18875.532802364902</v>
       </c>
-      <c r="N19">
+      <c r="N23">
         <v>992.31070788530405</v>
       </c>
-      <c r="O19">
-        <v>0</v>
-      </c>
-      <c r="P19">
+      <c r="O23">
+        <v>0</v>
+      </c>
+      <c r="P23">
         <v>230512.59606633501</v>
       </c>
-      <c r="Q19">
+      <c r="Q23">
         <v>1103.3673370121001</v>
       </c>
-      <c r="R19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A20" t="s">
-        <v>23</v>
-      </c>
-      <c r="B20" t="s">
+      <c r="R23">
+        <v>0</v>
+      </c>
+      <c r="S23">
+        <v>0</v>
+      </c>
+      <c r="T23">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B24" t="s">
         <v>21</v>
       </c>
-      <c r="C20">
+      <c r="C24">
         <v>4</v>
       </c>
-      <c r="D20">
+      <c r="D24">
         <v>113598.307758221</v>
       </c>
-      <c r="E20">
+      <c r="E24">
         <v>282179.67123287398</v>
       </c>
-      <c r="F20">
+      <c r="F24">
         <v>0.83333533297315499</v>
       </c>
-      <c r="G20">
+      <c r="G24">
         <v>21005.263452339499</v>
       </c>
-      <c r="H20">
+      <c r="H24">
         <v>9419.1929847336105</v>
       </c>
-      <c r="I20">
-        <v>0</v>
-      </c>
-      <c r="J20">
-        <f>SUM(G20:I20)</f>
+      <c r="I24">
+        <v>0</v>
+      </c>
+      <c r="J24">
+        <f>SUM(G24:I24)</f>
         <v>30424.45643707311</v>
       </c>
-      <c r="K20">
+      <c r="K24">
         <v>48819.627456497903</v>
       </c>
-      <c r="L20">
+      <c r="L24">
         <v>14784.690159207899</v>
       </c>
-      <c r="M20">
+      <c r="M24">
         <v>19569.533705442402</v>
       </c>
-      <c r="N20">
+      <c r="N24">
         <v>1040.9289460857101</v>
       </c>
-      <c r="O20">
-        <v>0</v>
-      </c>
-      <c r="P20">
+      <c r="O24">
+        <v>0</v>
+      </c>
+      <c r="P24">
         <v>235150.29028510299</v>
       </c>
-      <c r="Q20">
+      <c r="Q24">
         <v>1494.95371016114</v>
       </c>
-      <c r="R20">
+      <c r="R24">
         <v>40078.803663142098</v>
       </c>
-      <c r="S20">
+      <c r="S24">
         <v>910.88190143504903</v>
       </c>
-      <c r="T20">
+      <c r="T24">
         <v>0.51068072492979899</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A24" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A25" t="s">
-        <v>0</v>
-      </c>
-      <c r="B25" t="s">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A27" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="28" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A28" t="s">
+        <v>0</v>
+      </c>
+      <c r="B28" t="s">
         <v>1</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C28" t="s">
         <v>2</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D28" t="s">
         <v>3</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E28" t="s">
         <v>4</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F28" t="s">
         <v>5</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G28" t="s">
         <v>6</v>
       </c>
-      <c r="H25" t="s">
+      <c r="H28" t="s">
         <v>7</v>
       </c>
-      <c r="I25" t="s">
+      <c r="I28" t="s">
         <v>8</v>
       </c>
-      <c r="J25" t="s">
+      <c r="J28" t="s">
         <v>9</v>
       </c>
-      <c r="K25" t="s">
+      <c r="K28" t="s">
         <v>10</v>
       </c>
-      <c r="L25" t="s">
+      <c r="L28" t="s">
         <v>11</v>
       </c>
-      <c r="M25" t="s">
+      <c r="M28" t="s">
         <v>12</v>
       </c>
-      <c r="N25" t="s">
+      <c r="N28" t="s">
         <v>13</v>
       </c>
-      <c r="O25" t="s">
+      <c r="O28" t="s">
         <v>14</v>
       </c>
-      <c r="P25" t="s">
+      <c r="P28" t="s">
         <v>15</v>
       </c>
-      <c r="Q25" t="s">
+      <c r="Q28" t="s">
         <v>16</v>
       </c>
-      <c r="R25" t="s">
+      <c r="R28" t="s">
         <v>17</v>
       </c>
-      <c r="S25" t="s">
+      <c r="S28" t="s">
         <v>18</v>
       </c>
-      <c r="T25" t="s">
+      <c r="T28" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A26" t="s">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A29" t="s">
         <v>20</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B29" t="s">
         <v>21</v>
       </c>
-      <c r="C26">
+      <c r="C29">
         <v>4</v>
       </c>
-      <c r="D26">
+      <c r="D29">
         <v>29525.427309999999</v>
       </c>
-      <c r="E26">
+      <c r="E29">
         <v>80391.755990000005</v>
       </c>
-      <c r="F26">
+      <c r="F29">
         <v>0.79280104200000001</v>
       </c>
-      <c r="G26">
+      <c r="G29">
         <v>5050.6365619999997</v>
       </c>
-      <c r="H26">
+      <c r="H29">
         <v>4678.3390820000004</v>
       </c>
-      <c r="I26">
+      <c r="I29">
         <v>2508.6600360000002</v>
       </c>
-      <c r="J26">
+      <c r="J29">
         <v>12237.635679999999</v>
       </c>
-      <c r="K26">
+      <c r="K29">
         <v>13920</v>
       </c>
-      <c r="L26">
+      <c r="L29">
         <v>2841.544922</v>
       </c>
-      <c r="M26">
+      <c r="M29">
         <v>5380.5444360000001</v>
       </c>
-      <c r="N26">
+      <c r="N29">
         <v>279.27307350000001</v>
       </c>
-      <c r="O26">
-        <v>0</v>
-      </c>
-      <c r="P26">
+      <c r="O29">
+        <v>0</v>
+      </c>
+      <c r="P29">
         <v>63734.6679</v>
       </c>
-      <c r="Q26">
+      <c r="Q29">
         <v>1078.4492829999999</v>
       </c>
-      <c r="R26">
+      <c r="R29">
         <v>624.70352849999995</v>
       </c>
-      <c r="S26">
+      <c r="S29">
         <v>13.014656840000001</v>
       </c>
-      <c r="T26">
+      <c r="T29">
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A27" t="s">
-        <v>23</v>
-      </c>
-      <c r="B27" t="s">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A30" t="s">
+        <v>22</v>
+      </c>
+      <c r="B30" t="s">
         <v>21</v>
       </c>
-      <c r="C27">
+      <c r="C30">
         <v>4</v>
       </c>
-      <c r="D27">
+      <c r="D30">
         <v>30655.78772</v>
       </c>
-      <c r="E27">
+      <c r="E30">
         <v>79415.835619999998</v>
       </c>
-      <c r="F27">
+      <c r="F30">
         <v>0.81677700399999997</v>
       </c>
-      <c r="G27">
+      <c r="G30">
         <v>5129.9926729999997</v>
       </c>
-      <c r="H27">
+      <c r="H30">
         <v>5254.1641179999997</v>
       </c>
-      <c r="I27">
+      <c r="I30">
         <v>4834.2260249999999</v>
       </c>
-      <c r="J27">
+      <c r="J30">
         <v>15218.382820000001</v>
       </c>
-      <c r="K27">
+      <c r="K30">
         <v>13875.1543</v>
       </c>
-      <c r="L27">
+      <c r="L30">
         <v>3140.6678670000001</v>
       </c>
-      <c r="M27">
+      <c r="M30">
         <v>5340.9854210000003</v>
       </c>
-      <c r="N27">
+      <c r="N30">
         <v>286.5902719</v>
       </c>
-      <c r="O27">
-        <v>0</v>
-      </c>
-      <c r="P27">
+      <c r="O30">
+        <v>0</v>
+      </c>
+      <c r="P30">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q27">
+      <c r="Q30">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R27">
+      <c r="R30">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S27">
+      <c r="S30">
         <v>452.7322633</v>
       </c>
-      <c r="T27">
+      <c r="T30">
         <v>5.8154128590000003</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Testing 2 flexible skids
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FAC0585A-C9E4-4D65-BA13-A6B2D40A7502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46208FB6-8308-47A6-882A-B9FBF922CF41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57495" yWindow="8550" windowWidth="14610" windowHeight="15585" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
   </authors>
   <commentList>
-    <comment ref="A21" authorId="0" shapeId="0" xr:uid="{9CE96C07-E110-41BE-B453-65310D0A2128}">
+    <comment ref="A27" authorId="0" shapeId="0" xr:uid="{9CE96C07-E110-41BE-B453-65310D0A2128}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -47,7 +47,7 @@
     Summer is the summer hot weekdays + high weekends.</t>
       </text>
     </comment>
-    <comment ref="A22" authorId="1" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A28" authorId="1" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -60,7 +60,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="30">
   <si>
     <t>Season</t>
   </si>
@@ -633,9 +633,10 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1017,10 +1018,10 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A21" dT="2026-05-27T21:41:37.20" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9CE96C07-E110-41BE-B453-65310D0A2128}">
+  <threadedComment ref="A27" dT="2026-05-27T21:41:37.20" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9CE96C07-E110-41BE-B453-65310D0A2128}">
     <text>Summer is the summer hot weekdays + high weekends.</text>
   </threadedComment>
-  <threadedComment ref="A22" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+  <threadedComment ref="A28" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
     <text>Winter is low winter weekdays + low weekends</text>
   </threadedComment>
 </ThreadedComments>
@@ -1028,7 +1029,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:T30"/>
+  <dimension ref="A1:T36"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="3" max="3" width="14.23046875" customWidth="1"/>
@@ -1161,6 +1162,12 @@
       <c r="R3">
         <v>0</v>
       </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>0</v>
+      </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
@@ -1217,43 +1224,49 @@
       <c r="R4">
         <v>0</v>
       </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
     </row>
     <row r="6" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C6">
         <v>0</v>
       </c>
       <c r="D6">
-        <v>111179.352715972</v>
+        <v>111142.758477303</v>
       </c>
       <c r="E6">
         <v>282179.67123287602</v>
       </c>
       <c r="F6">
-        <v>0.82476293995957695</v>
+        <v>0.82463325578173197</v>
       </c>
       <c r="G6">
-        <v>18266.8157113575</v>
+        <v>18240.8407502021</v>
       </c>
       <c r="H6">
-        <v>4858.1774967593901</v>
+        <v>4851.2693328072801</v>
       </c>
       <c r="I6">
-        <v>2609.8466266994801</v>
+        <v>2606.1355131391001</v>
       </c>
       <c r="J6">
-        <v>25734.839834816299</v>
+        <v>25698.245596148499</v>
       </c>
       <c r="K6">
-        <v>50843.184005923897</v>
+        <v>50843.1840059237</v>
       </c>
       <c r="L6">
-        <v>15303.798385783701</v>
+        <v>15303.7983857831</v>
       </c>
       <c r="M6">
         <v>19297.530489448302</v>
@@ -1265,18 +1278,24 @@
         <v>0</v>
       </c>
       <c r="P6">
-        <v>232731.33524285399</v>
+        <v>232694.74100418499</v>
       </c>
       <c r="Q6">
-        <v>1103.1405255510299</v>
+        <v>1101.5718970651201</v>
       </c>
       <c r="R6">
+        <v>0</v>
+      </c>
+      <c r="S6">
+        <v>0</v>
+      </c>
+      <c r="T6">
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B7" t="s">
         <v>24</v>
@@ -1285,34 +1304,34 @@
         <v>0</v>
       </c>
       <c r="D7">
-        <v>103268.55989110901</v>
+        <v>120105.62640119799</v>
       </c>
       <c r="E7">
-        <v>282179.79409919202</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F7">
-        <v>0.79672799796204397</v>
+        <v>0.85639623815652299</v>
       </c>
       <c r="G7">
-        <v>18267.443429751202</v>
+        <v>20632.008189972999</v>
       </c>
       <c r="H7">
-        <v>4858.6111494831202</v>
+        <v>4931.94871395263</v>
       </c>
       <c r="I7">
-        <v>2610.0795879488901</v>
+        <v>9097.1451203198394</v>
       </c>
       <c r="J7">
-        <v>25736.1341671833</v>
+        <v>34661.102024245498</v>
       </c>
       <c r="K7">
-        <v>48811.852007574802</v>
+        <v>50843.186957348102</v>
       </c>
       <c r="L7">
-        <v>9844.5408077047105</v>
+        <v>15303.8063177357</v>
       </c>
       <c r="M7">
-        <v>18876.032908646699</v>
+        <v>19297.531101868899</v>
       </c>
       <c r="N7">
         <v>992.31070788530405</v>
@@ -1321,68 +1340,80 @@
         <v>0</v>
       </c>
       <c r="P7">
-        <v>224820.542417991</v>
+        <v>241657.60892808001</v>
       </c>
       <c r="Q7">
-        <v>1103.23899455419</v>
+        <v>1101.9194839550801</v>
       </c>
       <c r="R7">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A8" t="s">
+      <c r="S7">
+        <v>0</v>
+      </c>
+      <c r="T7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A9" t="s">
         <v>20</v>
       </c>
-      <c r="B8" t="s">
-        <v>21</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8">
-        <v>103268.55989110901</v>
-      </c>
-      <c r="E8">
-        <v>282179.79409919202</v>
-      </c>
-      <c r="F8">
-        <v>0.79672799796204397</v>
-      </c>
-      <c r="G8">
-        <v>18267.443429751202</v>
-      </c>
-      <c r="H8">
-        <v>4858.6111494831202</v>
-      </c>
-      <c r="I8">
-        <v>2610.0795879488901</v>
-      </c>
-      <c r="J8">
-        <v>25736.1341671833</v>
-      </c>
-      <c r="K8">
-        <v>48811.852007574802</v>
-      </c>
-      <c r="L8">
-        <v>9844.5408077047105</v>
-      </c>
-      <c r="M8">
-        <v>18876.032908646699</v>
-      </c>
-      <c r="N8">
+      <c r="B9" t="s">
+        <v>25</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>111179.352715972</v>
+      </c>
+      <c r="E9">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F9">
+        <v>0.82476293995957695</v>
+      </c>
+      <c r="G9">
+        <v>18266.8157113575</v>
+      </c>
+      <c r="H9">
+        <v>4858.1774967593901</v>
+      </c>
+      <c r="I9">
+        <v>2609.8466266994801</v>
+      </c>
+      <c r="J9">
+        <v>25734.839834816299</v>
+      </c>
+      <c r="K9">
+        <v>50843.184005923897</v>
+      </c>
+      <c r="L9">
+        <v>15303.798385783701</v>
+      </c>
+      <c r="M9">
+        <v>19297.530489448302</v>
+      </c>
+      <c r="N9">
         <v>992.31070788530405</v>
       </c>
-      <c r="O8">
-        <v>0</v>
-      </c>
-      <c r="P8">
-        <v>224820.542417991</v>
-      </c>
-      <c r="Q8">
-        <v>1103.23899455419</v>
-      </c>
-      <c r="R8">
+      <c r="O9">
+        <v>0</v>
+      </c>
+      <c r="P9">
+        <v>232731.33524285399</v>
+      </c>
+      <c r="Q9">
+        <v>1103.1405255510299</v>
+      </c>
+      <c r="R9">
+        <v>0</v>
+      </c>
+      <c r="S9">
+        <v>0</v>
+      </c>
+      <c r="T9">
         <v>0</v>
       </c>
     </row>
@@ -1441,60 +1472,10 @@
       <c r="R10">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A11" t="s">
-        <v>22</v>
-      </c>
-      <c r="B11" t="s">
-        <v>24</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11">
-        <v>112735.91652453299</v>
-      </c>
-      <c r="E11">
-        <v>282179.67125392298</v>
-      </c>
-      <c r="F11">
-        <v>0.83027915515780504</v>
-      </c>
-      <c r="G11">
-        <v>20960.382547718</v>
-      </c>
-      <c r="H11">
-        <v>5010.4440999274602</v>
-      </c>
-      <c r="I11">
-        <v>9241.9323985477895</v>
-      </c>
-      <c r="J11">
-        <v>35212.7590461933</v>
-      </c>
-      <c r="K11">
-        <v>48809.459899526402</v>
-      </c>
-      <c r="L11">
-        <v>9838.1648407904995</v>
-      </c>
-      <c r="M11">
-        <v>18875.532738023201</v>
-      </c>
-      <c r="N11">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O11">
-        <v>0</v>
-      </c>
-      <c r="P11">
-        <v>234287.89905141501</v>
-      </c>
-      <c r="Q11">
-        <v>1119.4572971447301</v>
-      </c>
-      <c r="R11">
+      <c r="S10">
+        <v>0</v>
+      </c>
+      <c r="T10">
         <v>0</v>
       </c>
     </row>
@@ -1509,34 +1490,34 @@
         <v>0</v>
       </c>
       <c r="D12">
-        <v>112735.91652453299</v>
+        <v>120105.62640119799</v>
       </c>
       <c r="E12">
-        <v>282179.67125392298</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F12">
-        <v>0.83027915515780504</v>
+        <v>0.85639623815652299</v>
       </c>
       <c r="G12">
-        <v>20960.382547718</v>
+        <v>20632.008189972999</v>
       </c>
       <c r="H12">
-        <v>5010.4440999274602</v>
+        <v>4931.94871395263</v>
       </c>
       <c r="I12">
-        <v>9241.9323985477895</v>
+        <v>9097.1451203198394</v>
       </c>
       <c r="J12">
-        <v>35212.7590461933</v>
+        <v>34661.102024245498</v>
       </c>
       <c r="K12">
-        <v>48809.459899526402</v>
+        <v>50843.186957348102</v>
       </c>
       <c r="L12">
-        <v>9838.1648407904995</v>
+        <v>15303.8063177357</v>
       </c>
       <c r="M12">
-        <v>18875.532738023201</v>
+        <v>19297.531101868899</v>
       </c>
       <c r="N12">
         <v>992.31070788530405</v>
@@ -1545,29 +1526,86 @@
         <v>0</v>
       </c>
       <c r="P12">
-        <v>234287.89905141501</v>
+        <v>241657.60892808001</v>
       </c>
       <c r="Q12">
-        <v>1119.4572971447301</v>
+        <v>1101.9194839550801</v>
       </c>
       <c r="R12">
         <v>0</v>
       </c>
-    </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A14" t="s">
+      <c r="S12">
+        <v>0</v>
+      </c>
+      <c r="T12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A13" t="s">
         <v>20</v>
       </c>
-      <c r="B14" t="s">
-        <v>23</v>
-      </c>
-      <c r="C14">
-        <v>2</v>
+      <c r="B13" t="s">
+        <v>21</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>111142.758477303</v>
+      </c>
+      <c r="E13">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F13">
+        <v>0.82463325578173197</v>
+      </c>
+      <c r="G13">
+        <v>18240.8407502021</v>
+      </c>
+      <c r="H13">
+        <v>4851.2693328072801</v>
+      </c>
+      <c r="I13">
+        <v>2606.1355131391001</v>
+      </c>
+      <c r="J13">
+        <v>25698.245596148499</v>
+      </c>
+      <c r="K13">
+        <v>50843.1840059237</v>
+      </c>
+      <c r="L13">
+        <v>15303.7983857831</v>
+      </c>
+      <c r="M13">
+        <v>19297.530489448302</v>
+      </c>
+      <c r="N13">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O13">
+        <v>0</v>
+      </c>
+      <c r="P13">
+        <v>232694.74100418499</v>
+      </c>
+      <c r="Q13">
+        <v>1101.5718970651201</v>
+      </c>
+      <c r="R13">
+        <v>0</v>
+      </c>
+      <c r="S13">
+        <v>0</v>
+      </c>
+      <c r="T13">
+        <v>0</v>
       </c>
     </row>
     <row r="15" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B15" t="s">
         <v>23</v>
@@ -1578,158 +1616,102 @@
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
+        <v>22</v>
+      </c>
+      <c r="B16" t="s">
+        <v>23</v>
+      </c>
+      <c r="C16">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A18" t="s">
         <v>20</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B18" t="s">
         <v>21</v>
       </c>
-      <c r="C16">
+      <c r="C18">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A19" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" t="s">
+        <v>21</v>
+      </c>
+      <c r="C19">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A22" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B22" t="s">
+        <v>21</v>
+      </c>
+      <c r="C22">
         <v>4</v>
       </c>
-      <c r="D16">
+      <c r="D22">
         <v>103263.067623782</v>
       </c>
-      <c r="E16">
+      <c r="E22">
         <v>282179.67123287701</v>
       </c>
-      <c r="F16">
+      <c r="F22">
         <v>0.79670888114802996</v>
       </c>
-      <c r="G16">
+      <c r="G22">
         <v>18270.343045682599</v>
       </c>
-      <c r="H16">
+      <c r="H22">
         <v>4859.1187222275803</v>
       </c>
-      <c r="I16">
+      <c r="I22">
         <v>2610.3522592715499</v>
       </c>
-      <c r="J16">
+      <c r="J22">
         <v>25739.814027181699</v>
       </c>
-      <c r="K16">
+      <c r="K22">
         <v>48809.484574716203</v>
       </c>
-      <c r="L16">
+      <c r="L22">
         <v>9838.23116441202</v>
       </c>
-      <c r="M16">
+      <c r="M22">
         <v>18875.537857472798</v>
       </c>
-      <c r="N16">
+      <c r="N22">
         <v>992.31070788530405</v>
       </c>
-      <c r="O16">
-        <v>0</v>
-      </c>
-      <c r="P16">
+      <c r="O22">
+        <v>0</v>
+      </c>
+      <c r="P22">
         <v>224815.050150664</v>
       </c>
-      <c r="Q16">
+      <c r="Q22">
         <v>1103.3542485400801</v>
       </c>
-      <c r="R16">
-        <v>0</v>
-      </c>
-      <c r="S16">
-        <v>0</v>
-      </c>
-      <c r="T16">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A17" t="s">
+      <c r="R22">
+        <v>0</v>
+      </c>
+      <c r="S22">
+        <v>0</v>
+      </c>
+      <c r="T22">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A23" s="2" t="s">
         <v>22</v>
-      </c>
-      <c r="B17" t="s">
-        <v>21</v>
-      </c>
-      <c r="C17">
-        <v>4</v>
-      </c>
-      <c r="D17">
-        <v>108527.711286153</v>
-      </c>
-      <c r="E17">
-        <v>282179.67123319401</v>
-      </c>
-      <c r="F17">
-        <v>0.81536594329254797</v>
-      </c>
-      <c r="G17">
-        <v>19470.284119269101</v>
-      </c>
-      <c r="H17">
-        <v>5251.7861497213999</v>
-      </c>
-      <c r="I17">
-        <v>4921.3210739687102</v>
-      </c>
-      <c r="J17">
-        <v>29643.391342959199</v>
-      </c>
-      <c r="K17">
-        <v>49158.923944860697</v>
-      </c>
-      <c r="L17">
-        <v>10777.3494715455</v>
-      </c>
-      <c r="M17">
-        <v>18948.046526787599</v>
-      </c>
-      <c r="N17">
-        <v>1008.6177006503</v>
-      </c>
-      <c r="O17">
-        <v>0</v>
-      </c>
-      <c r="P17">
-        <v>230079.69381303401</v>
-      </c>
-      <c r="Q17">
-        <v>1173.3790798621201</v>
-      </c>
-      <c r="R17">
-        <v>12990.682952859001</v>
-      </c>
-      <c r="S17">
-        <v>463.95296260210699</v>
-      </c>
-      <c r="T17">
-        <v>1.63318791126541</v>
-      </c>
-    </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A20" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A21" t="s">
-        <v>22</v>
-      </c>
-      <c r="B21" t="s">
-        <v>23</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A22" t="s">
-        <v>20</v>
-      </c>
-      <c r="B22" t="s">
-        <v>23</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A23" t="s">
-        <v>20</v>
       </c>
       <c r="B23" t="s">
         <v>21</v>
@@ -1738,190 +1720,86 @@
         <v>4</v>
       </c>
       <c r="D23">
-        <v>108960.613539453</v>
+        <v>108527.711286153</v>
       </c>
       <c r="E23">
-        <v>282179.67123287701</v>
+        <v>282179.67123319401</v>
       </c>
       <c r="F23">
-        <v>0.81690008021909599</v>
+        <v>0.81536594329254797</v>
       </c>
       <c r="G23">
-        <v>23571.632136721099</v>
+        <v>19470.284119269101</v>
       </c>
       <c r="H23">
-        <v>6951.9409028971204</v>
+        <v>5251.7861497213999</v>
       </c>
       <c r="I23">
-        <v>913.88179307768496</v>
+        <v>4921.3210739687102</v>
       </c>
       <c r="J23">
-        <f>SUM(G23:I23)</f>
-        <v>31437.454832695905</v>
+        <v>29643.391342959199</v>
       </c>
       <c r="K23">
-        <v>48809.460212750702</v>
+        <v>49158.923944860697</v>
       </c>
       <c r="L23">
-        <v>9838.1656916422507</v>
+        <v>10777.3494715455</v>
       </c>
       <c r="M23">
-        <v>18875.532802364902</v>
+        <v>18948.046526787599</v>
       </c>
       <c r="N23">
-        <v>992.31070788530405</v>
+        <v>1008.6177006503</v>
       </c>
       <c r="O23">
         <v>0</v>
       </c>
       <c r="P23">
-        <v>230512.59606633501</v>
+        <v>230079.69381303401</v>
       </c>
       <c r="Q23">
-        <v>1103.3673370121001</v>
+        <v>1173.3790798621201</v>
       </c>
       <c r="R23">
-        <v>0</v>
+        <v>12990.682952859001</v>
       </c>
       <c r="S23">
-        <v>0</v>
+        <v>463.95296260210699</v>
       </c>
       <c r="T23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A24" t="s">
+        <v>1.63318791126541</v>
+      </c>
+    </row>
+    <row r="26" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A26" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A27" t="s">
         <v>22</v>
       </c>
-      <c r="B24" t="s">
-        <v>21</v>
-      </c>
-      <c r="C24">
-        <v>4</v>
-      </c>
-      <c r="D24">
-        <v>113598.307758221</v>
-      </c>
-      <c r="E24">
-        <v>282179.67123287398</v>
-      </c>
-      <c r="F24">
-        <v>0.83333533297315499</v>
-      </c>
-      <c r="G24">
-        <v>21005.263452339499</v>
-      </c>
-      <c r="H24">
-        <v>9419.1929847336105</v>
-      </c>
-      <c r="I24">
-        <v>0</v>
-      </c>
-      <c r="J24">
-        <f>SUM(G24:I24)</f>
-        <v>30424.45643707311</v>
-      </c>
-      <c r="K24">
-        <v>48819.627456497903</v>
-      </c>
-      <c r="L24">
-        <v>14784.690159207899</v>
-      </c>
-      <c r="M24">
-        <v>19569.533705442402</v>
-      </c>
-      <c r="N24">
-        <v>1040.9289460857101</v>
-      </c>
-      <c r="O24">
-        <v>0</v>
-      </c>
-      <c r="P24">
-        <v>235150.29028510299</v>
-      </c>
-      <c r="Q24">
-        <v>1494.95371016114</v>
-      </c>
-      <c r="R24">
-        <v>40078.803663142098</v>
-      </c>
-      <c r="S24">
-        <v>910.88190143504903</v>
-      </c>
-      <c r="T24">
-        <v>0.51068072492979899</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A27" s="1" t="s">
-        <v>26</v>
+      <c r="B27" t="s">
+        <v>23</v>
+      </c>
+      <c r="C27">
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="B28" t="s">
-        <v>1</v>
-      </c>
-      <c r="C28" t="s">
-        <v>2</v>
-      </c>
-      <c r="D28" t="s">
-        <v>3</v>
-      </c>
-      <c r="E28" t="s">
-        <v>4</v>
-      </c>
-      <c r="F28" t="s">
-        <v>5</v>
-      </c>
-      <c r="G28" t="s">
-        <v>6</v>
-      </c>
-      <c r="H28" t="s">
-        <v>7</v>
-      </c>
-      <c r="I28" t="s">
-        <v>8</v>
-      </c>
-      <c r="J28" t="s">
-        <v>9</v>
-      </c>
-      <c r="K28" t="s">
-        <v>10</v>
-      </c>
-      <c r="L28" t="s">
-        <v>11</v>
-      </c>
-      <c r="M28" t="s">
-        <v>12</v>
-      </c>
-      <c r="N28" t="s">
-        <v>13</v>
-      </c>
-      <c r="O28" t="s">
-        <v>14</v>
-      </c>
-      <c r="P28" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q28" t="s">
-        <v>16</v>
-      </c>
-      <c r="R28" t="s">
-        <v>17</v>
-      </c>
-      <c r="S28" t="s">
-        <v>18</v>
-      </c>
-      <c r="T28" t="s">
-        <v>19</v>
+        <v>23</v>
+      </c>
+      <c r="C28">
+        <v>0</v>
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A29" t="s">
+      <c r="A29" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B29" t="s">
@@ -1931,59 +1809,60 @@
         <v>4</v>
       </c>
       <c r="D29">
-        <v>29525.427309999999</v>
+        <v>108960.613539453</v>
       </c>
       <c r="E29">
-        <v>80391.755990000005</v>
+        <v>282179.67123287701</v>
       </c>
       <c r="F29">
-        <v>0.79280104200000001</v>
+        <v>0.81690008021909599</v>
       </c>
       <c r="G29">
-        <v>5050.6365619999997</v>
+        <v>23571.632136721099</v>
       </c>
       <c r="H29">
-        <v>4678.3390820000004</v>
+        <v>6951.9409028971204</v>
       </c>
       <c r="I29">
-        <v>2508.6600360000002</v>
+        <v>913.88179307768496</v>
       </c>
       <c r="J29">
-        <v>12237.635679999999</v>
+        <f>SUM(G29:I29)</f>
+        <v>31437.454832695905</v>
       </c>
       <c r="K29">
-        <v>13920</v>
+        <v>48809.460212750702</v>
       </c>
       <c r="L29">
-        <v>2841.544922</v>
+        <v>9838.1656916422507</v>
       </c>
       <c r="M29">
-        <v>5380.5444360000001</v>
+        <v>18875.532802364902</v>
       </c>
       <c r="N29">
-        <v>279.27307350000001</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O29">
         <v>0</v>
       </c>
       <c r="P29">
-        <v>63734.6679</v>
+        <v>230512.59606633501</v>
       </c>
       <c r="Q29">
-        <v>1078.4492829999999</v>
+        <v>1103.3673370121001</v>
       </c>
       <c r="R29">
-        <v>624.70352849999995</v>
+        <v>0</v>
       </c>
       <c r="S29">
-        <v>13.014656840000001</v>
+        <v>0</v>
       </c>
       <c r="T29">
-        <v>27.514184579999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A30" t="s">
+      <c r="A30" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B30" t="s">
@@ -1993,60 +1872,253 @@
         <v>4</v>
       </c>
       <c r="D30">
+        <v>113598.307758221</v>
+      </c>
+      <c r="E30">
+        <v>282179.67123287398</v>
+      </c>
+      <c r="F30">
+        <v>0.83333533297315499</v>
+      </c>
+      <c r="G30">
+        <v>21005.263452339499</v>
+      </c>
+      <c r="H30">
+        <v>9419.1929847336105</v>
+      </c>
+      <c r="I30">
+        <v>0</v>
+      </c>
+      <c r="J30">
+        <f>SUM(G30:I30)</f>
+        <v>30424.45643707311</v>
+      </c>
+      <c r="K30">
+        <v>48819.627456497903</v>
+      </c>
+      <c r="L30">
+        <v>14784.690159207899</v>
+      </c>
+      <c r="M30">
+        <v>19569.533705442402</v>
+      </c>
+      <c r="N30">
+        <v>1040.9289460857101</v>
+      </c>
+      <c r="O30">
+        <v>0</v>
+      </c>
+      <c r="P30">
+        <v>235150.29028510299</v>
+      </c>
+      <c r="Q30">
+        <v>1494.95371016114</v>
+      </c>
+      <c r="R30">
+        <v>40078.803663142098</v>
+      </c>
+      <c r="S30">
+        <v>910.88190143504903</v>
+      </c>
+      <c r="T30">
+        <v>0.51068072492979899</v>
+      </c>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A33" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A34" t="s">
+        <v>0</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1</v>
+      </c>
+      <c r="C34" t="s">
+        <v>2</v>
+      </c>
+      <c r="D34" t="s">
+        <v>3</v>
+      </c>
+      <c r="E34" t="s">
+        <v>4</v>
+      </c>
+      <c r="F34" t="s">
+        <v>5</v>
+      </c>
+      <c r="G34" t="s">
+        <v>6</v>
+      </c>
+      <c r="H34" t="s">
+        <v>7</v>
+      </c>
+      <c r="I34" t="s">
+        <v>8</v>
+      </c>
+      <c r="J34" t="s">
+        <v>9</v>
+      </c>
+      <c r="K34" t="s">
+        <v>10</v>
+      </c>
+      <c r="L34" t="s">
+        <v>11</v>
+      </c>
+      <c r="M34" t="s">
+        <v>12</v>
+      </c>
+      <c r="N34" t="s">
+        <v>13</v>
+      </c>
+      <c r="O34" t="s">
+        <v>14</v>
+      </c>
+      <c r="P34" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>16</v>
+      </c>
+      <c r="R34" t="s">
+        <v>17</v>
+      </c>
+      <c r="S34" t="s">
+        <v>18</v>
+      </c>
+      <c r="T34" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A35" t="s">
+        <v>20</v>
+      </c>
+      <c r="B35" t="s">
+        <v>21</v>
+      </c>
+      <c r="C35">
+        <v>4</v>
+      </c>
+      <c r="D35">
+        <v>29525.427309999999</v>
+      </c>
+      <c r="E35">
+        <v>80391.755990000005</v>
+      </c>
+      <c r="F35">
+        <v>0.79280104200000001</v>
+      </c>
+      <c r="G35">
+        <v>5050.6365619999997</v>
+      </c>
+      <c r="H35">
+        <v>4678.3390820000004</v>
+      </c>
+      <c r="I35">
+        <v>2508.6600360000002</v>
+      </c>
+      <c r="J35">
+        <v>12237.635679999999</v>
+      </c>
+      <c r="K35">
+        <v>13920</v>
+      </c>
+      <c r="L35">
+        <v>2841.544922</v>
+      </c>
+      <c r="M35">
+        <v>5380.5444360000001</v>
+      </c>
+      <c r="N35">
+        <v>279.27307350000001</v>
+      </c>
+      <c r="O35">
+        <v>0</v>
+      </c>
+      <c r="P35">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q35">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R35">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S35">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T35">
+        <v>27.514184579999998</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A36" t="s">
+        <v>22</v>
+      </c>
+      <c r="B36" t="s">
+        <v>21</v>
+      </c>
+      <c r="C36">
+        <v>4</v>
+      </c>
+      <c r="D36">
         <v>30655.78772</v>
       </c>
-      <c r="E30">
+      <c r="E36">
         <v>79415.835619999998</v>
       </c>
-      <c r="F30">
+      <c r="F36">
         <v>0.81677700399999997</v>
       </c>
-      <c r="G30">
+      <c r="G36">
         <v>5129.9926729999997</v>
       </c>
-      <c r="H30">
+      <c r="H36">
         <v>5254.1641179999997</v>
       </c>
-      <c r="I30">
+      <c r="I36">
         <v>4834.2260249999999</v>
       </c>
-      <c r="J30">
+      <c r="J36">
         <v>15218.382820000001</v>
       </c>
-      <c r="K30">
+      <c r="K36">
         <v>13875.1543</v>
       </c>
-      <c r="L30">
+      <c r="L36">
         <v>3140.6678670000001</v>
       </c>
-      <c r="M30">
+      <c r="M36">
         <v>5340.9854210000003</v>
       </c>
-      <c r="N30">
+      <c r="N36">
         <v>286.5902719</v>
       </c>
-      <c r="O30">
-        <v>0</v>
-      </c>
-      <c r="P30">
+      <c r="O36">
+        <v>0</v>
+      </c>
+      <c r="P36">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q30">
+      <c r="Q36">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R30">
+      <c r="R36">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S30">
+      <c r="S36">
         <v>452.7322633</v>
       </c>
-      <c r="T30">
+      <c r="T36">
         <v>5.8154128590000003</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
Summer w/ 2 flex trains and smaller MIP gap
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46208FB6-8308-47A6-882A-B9FBF922CF41}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F689B85-74EF-4482-8A79-E9A59BAFD73B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -35,11 +35,20 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={ABAC2AC6-7A74-4F44-BF4E-754717C772A0}</author>
     <author>tc={9CE96C07-E110-41BE-B453-65310D0A2128}</author>
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
   </authors>
   <commentList>
-    <comment ref="A27" authorId="0" shapeId="0" xr:uid="{9CE96C07-E110-41BE-B453-65310D0A2128}">
+    <comment ref="A24" authorId="0" shapeId="0" xr:uid="{ABAC2AC6-7A74-4F44-BF4E-754717C772A0}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Have to re-run with fixed uf recovery and the 2nd order surrogate</t>
+      </text>
+    </comment>
+    <comment ref="A28" authorId="1" shapeId="0" xr:uid="{9CE96C07-E110-41BE-B453-65310D0A2128}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -47,7 +56,7 @@
     Summer is the summer hot weekdays + high weekends.</t>
       </text>
     </comment>
-    <comment ref="A28" authorId="1" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A29" authorId="2" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -60,7 +69,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="30">
   <si>
     <t>Season</t>
   </si>
@@ -156,7 +165,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -290,6 +299,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1018,10 +1033,13 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A27" dT="2026-05-27T21:41:37.20" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9CE96C07-E110-41BE-B453-65310D0A2128}">
+  <threadedComment ref="A24" dT="2026-05-28T22:11:07.28" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{ABAC2AC6-7A74-4F44-BF4E-754717C772A0}">
+    <text>Have to re-run with fixed uf recovery and the 2nd order surrogate</text>
+  </threadedComment>
+  <threadedComment ref="A28" dT="2026-05-27T21:41:37.20" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9CE96C07-E110-41BE-B453-65310D0A2128}">
     <text>Summer is the summer hot weekdays + high weekends.</text>
   </threadedComment>
-  <threadedComment ref="A28" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+  <threadedComment ref="A29" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
     <text>Winter is low winter weekdays + low weekends</text>
   </threadedComment>
 </ThreadedComments>
@@ -1029,10 +1047,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:T36"/>
+  <dimension ref="A1:T37"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="3" max="3" width="14.23046875" customWidth="1"/>
+    <col min="3" max="3" width="12.4609375" customWidth="1"/>
     <col min="5" max="5" width="10.3046875" customWidth="1"/>
     <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.53515625" customWidth="1"/>
@@ -1611,7 +1629,7 @@
         <v>23</v>
       </c>
       <c r="C15">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.4">
@@ -1622,7 +1640,7 @@
         <v>23</v>
       </c>
       <c r="C16">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.4">
@@ -1630,10 +1648,55 @@
         <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C18">
         <v>2</v>
+      </c>
+      <c r="D18">
+        <v>111737.917851103</v>
+      </c>
+      <c r="E18">
+        <v>282179.67125484499</v>
+      </c>
+      <c r="F18">
+        <v>0.826742406143402</v>
+      </c>
+      <c r="G18">
+        <v>18663.290146715601</v>
+      </c>
+      <c r="H18">
+        <v>4963.6224309139197</v>
+      </c>
+      <c r="I18">
+        <v>2666.4923762402</v>
+      </c>
+      <c r="J18">
+        <v>26293.4049538697</v>
+      </c>
+      <c r="K18">
+        <v>50843.184012302001</v>
+      </c>
+      <c r="L18">
+        <v>15303.798393478701</v>
+      </c>
+      <c r="M18">
+        <v>19297.530491452799</v>
+      </c>
+      <c r="N18">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O18">
+        <v>0</v>
+      </c>
+      <c r="P18">
+        <v>233289.900377985</v>
+      </c>
+      <c r="Q18">
+        <v>1127.0837800240299</v>
+      </c>
+      <c r="R18">
+        <v>0</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.4">
@@ -1641,155 +1704,211 @@
         <v>22</v>
       </c>
       <c r="B19" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C19">
         <v>2</v>
       </c>
     </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A21" t="s">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
+        <v>21</v>
+      </c>
+      <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21">
+        <v>111737.92287843001</v>
+      </c>
+      <c r="E21">
+        <v>282179.67125484499</v>
+      </c>
+      <c r="F21">
+        <v>0.82674242395945297</v>
+      </c>
+      <c r="G21">
+        <v>18663.290416404601</v>
+      </c>
+      <c r="H21">
+        <v>4963.6225077490999</v>
+      </c>
+      <c r="I21">
+        <v>2666.4924108713899</v>
+      </c>
+      <c r="J21">
+        <v>26293.405335025102</v>
+      </c>
+      <c r="K21">
+        <v>50843.185205157402</v>
+      </c>
+      <c r="L21">
+        <v>15303.8015992776</v>
+      </c>
+      <c r="M21">
+        <v>19297.530738970301</v>
+      </c>
+      <c r="N21">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O21">
+        <v>0</v>
+      </c>
+      <c r="P21">
+        <v>233289.90540531199</v>
+      </c>
+      <c r="Q21">
+        <v>1127.08379747136</v>
+      </c>
+      <c r="R21">
+        <v>0</v>
+      </c>
+    </row>
     <row r="22" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A22" s="2" t="s">
-        <v>20</v>
+      <c r="A22" t="s">
+        <v>22</v>
       </c>
       <c r="B22" t="s">
         <v>21</v>
       </c>
       <c r="C22">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A24" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24">
         <v>4</v>
       </c>
-      <c r="D22">
+      <c r="D24">
         <v>103263.067623782</v>
       </c>
-      <c r="E22">
+      <c r="E24">
         <v>282179.67123287701</v>
       </c>
-      <c r="F22">
+      <c r="F24">
         <v>0.79670888114802996</v>
       </c>
-      <c r="G22">
+      <c r="G24">
         <v>18270.343045682599</v>
       </c>
-      <c r="H22">
+      <c r="H24">
         <v>4859.1187222275803</v>
       </c>
-      <c r="I22">
+      <c r="I24">
         <v>2610.3522592715499</v>
       </c>
-      <c r="J22">
+      <c r="J24">
         <v>25739.814027181699</v>
       </c>
-      <c r="K22">
+      <c r="K24">
         <v>48809.484574716203</v>
       </c>
-      <c r="L22">
+      <c r="L24">
         <v>9838.23116441202</v>
       </c>
-      <c r="M22">
+      <c r="M24">
         <v>18875.537857472798</v>
       </c>
-      <c r="N22">
+      <c r="N24">
         <v>992.31070788530405</v>
       </c>
-      <c r="O22">
-        <v>0</v>
-      </c>
-      <c r="P22">
+      <c r="O24">
+        <v>0</v>
+      </c>
+      <c r="P24">
         <v>224815.050150664</v>
       </c>
-      <c r="Q22">
+      <c r="Q24">
         <v>1103.3542485400801</v>
       </c>
-      <c r="R22">
-        <v>0</v>
-      </c>
-      <c r="S22">
-        <v>0</v>
-      </c>
-      <c r="T22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A23" s="2" t="s">
+      <c r="R24">
+        <v>0</v>
+      </c>
+      <c r="S24">
+        <v>0</v>
+      </c>
+      <c r="T24">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A25" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B25" t="s">
         <v>21</v>
       </c>
-      <c r="C23">
+      <c r="C25">
         <v>4</v>
       </c>
-      <c r="D23">
+      <c r="D25">
         <v>108527.711286153</v>
       </c>
-      <c r="E23">
+      <c r="E25">
         <v>282179.67123319401</v>
       </c>
-      <c r="F23">
+      <c r="F25">
         <v>0.81536594329254797</v>
       </c>
-      <c r="G23">
+      <c r="G25">
         <v>19470.284119269101</v>
       </c>
-      <c r="H23">
+      <c r="H25">
         <v>5251.7861497213999</v>
       </c>
-      <c r="I23">
+      <c r="I25">
         <v>4921.3210739687102</v>
       </c>
-      <c r="J23">
+      <c r="J25">
         <v>29643.391342959199</v>
       </c>
-      <c r="K23">
+      <c r="K25">
         <v>49158.923944860697</v>
       </c>
-      <c r="L23">
+      <c r="L25">
         <v>10777.3494715455</v>
       </c>
-      <c r="M23">
+      <c r="M25">
         <v>18948.046526787599</v>
       </c>
-      <c r="N23">
+      <c r="N25">
         <v>1008.6177006503</v>
       </c>
-      <c r="O23">
-        <v>0</v>
-      </c>
-      <c r="P23">
+      <c r="O25">
+        <v>0</v>
+      </c>
+      <c r="P25">
         <v>230079.69381303401</v>
       </c>
-      <c r="Q23">
+      <c r="Q25">
         <v>1173.3790798621201</v>
       </c>
-      <c r="R23">
+      <c r="R25">
         <v>12990.682952859001</v>
       </c>
-      <c r="S23">
+      <c r="S25">
         <v>463.95296260210699</v>
       </c>
-      <c r="T23">
+      <c r="T25">
         <v>1.63318791126541</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A26" s="1" t="s">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A27" s="1" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A27" t="s">
-        <v>22</v>
-      </c>
-      <c r="B27" t="s">
-        <v>23</v>
-      </c>
-      <c r="C27">
-        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B28" t="s">
         <v>23</v>
@@ -1799,71 +1918,19 @@
       </c>
     </row>
     <row r="29" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A29" s="2" t="s">
+      <c r="A29" t="s">
         <v>20</v>
       </c>
       <c r="B29" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C29">
-        <v>4</v>
-      </c>
-      <c r="D29">
-        <v>108960.613539453</v>
-      </c>
-      <c r="E29">
-        <v>282179.67123287701</v>
-      </c>
-      <c r="F29">
-        <v>0.81690008021909599</v>
-      </c>
-      <c r="G29">
-        <v>23571.632136721099</v>
-      </c>
-      <c r="H29">
-        <v>6951.9409028971204</v>
-      </c>
-      <c r="I29">
-        <v>913.88179307768496</v>
-      </c>
-      <c r="J29">
-        <f>SUM(G29:I29)</f>
-        <v>31437.454832695905</v>
-      </c>
-      <c r="K29">
-        <v>48809.460212750702</v>
-      </c>
-      <c r="L29">
-        <v>9838.1656916422507</v>
-      </c>
-      <c r="M29">
-        <v>18875.532802364902</v>
-      </c>
-      <c r="N29">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O29">
-        <v>0</v>
-      </c>
-      <c r="P29">
-        <v>230512.59606633501</v>
-      </c>
-      <c r="Q29">
-        <v>1103.3673370121001</v>
-      </c>
-      <c r="R29">
-        <v>0</v>
-      </c>
-      <c r="S29">
-        <v>0</v>
-      </c>
-      <c r="T29">
         <v>0</v>
       </c>
     </row>
     <row r="30" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B30" t="s">
         <v>21</v>
@@ -1872,190 +1939,191 @@
         <v>4</v>
       </c>
       <c r="D30">
-        <v>113598.307758221</v>
+        <v>108960.613539453</v>
       </c>
       <c r="E30">
-        <v>282179.67123287398</v>
+        <v>282179.67123287701</v>
       </c>
       <c r="F30">
-        <v>0.83333533297315499</v>
+        <v>0.81690008021909599</v>
       </c>
       <c r="G30">
-        <v>21005.263452339499</v>
+        <v>23571.632136721099</v>
       </c>
       <c r="H30">
-        <v>9419.1929847336105</v>
+        <v>6951.9409028971204</v>
       </c>
       <c r="I30">
-        <v>0</v>
+        <v>913.88179307768496</v>
       </c>
       <c r="J30">
         <f>SUM(G30:I30)</f>
+        <v>31437.454832695905</v>
+      </c>
+      <c r="K30">
+        <v>48809.460212750702</v>
+      </c>
+      <c r="L30">
+        <v>9838.1656916422507</v>
+      </c>
+      <c r="M30">
+        <v>18875.532802364902</v>
+      </c>
+      <c r="N30">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O30">
+        <v>0</v>
+      </c>
+      <c r="P30">
+        <v>230512.59606633501</v>
+      </c>
+      <c r="Q30">
+        <v>1103.3673370121001</v>
+      </c>
+      <c r="R30">
+        <v>0</v>
+      </c>
+      <c r="S30">
+        <v>0</v>
+      </c>
+      <c r="T30">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A31" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B31" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31">
+        <v>4</v>
+      </c>
+      <c r="D31">
+        <v>113598.307758221</v>
+      </c>
+      <c r="E31">
+        <v>282179.67123287398</v>
+      </c>
+      <c r="F31">
+        <v>0.83333533297315499</v>
+      </c>
+      <c r="G31">
+        <v>21005.263452339499</v>
+      </c>
+      <c r="H31">
+        <v>9419.1929847336105</v>
+      </c>
+      <c r="I31">
+        <v>0</v>
+      </c>
+      <c r="J31">
+        <f>SUM(G31:I31)</f>
         <v>30424.45643707311</v>
       </c>
-      <c r="K30">
+      <c r="K31">
         <v>48819.627456497903</v>
       </c>
-      <c r="L30">
+      <c r="L31">
         <v>14784.690159207899</v>
       </c>
-      <c r="M30">
+      <c r="M31">
         <v>19569.533705442402</v>
       </c>
-      <c r="N30">
+      <c r="N31">
         <v>1040.9289460857101</v>
       </c>
-      <c r="O30">
-        <v>0</v>
-      </c>
-      <c r="P30">
+      <c r="O31">
+        <v>0</v>
+      </c>
+      <c r="P31">
         <v>235150.29028510299</v>
       </c>
-      <c r="Q30">
+      <c r="Q31">
         <v>1494.95371016114</v>
       </c>
-      <c r="R30">
+      <c r="R31">
         <v>40078.803663142098</v>
       </c>
-      <c r="S30">
+      <c r="S31">
         <v>910.88190143504903</v>
       </c>
-      <c r="T30">
+      <c r="T31">
         <v>0.51068072492979899</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A33" s="1" t="s">
+    <row r="34" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A34" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A34" t="s">
-        <v>0</v>
-      </c>
-      <c r="B34" t="s">
+    <row r="35" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A35" t="s">
+        <v>0</v>
+      </c>
+      <c r="B35" t="s">
         <v>1</v>
       </c>
-      <c r="C34" t="s">
+      <c r="C35" t="s">
         <v>2</v>
       </c>
-      <c r="D34" t="s">
+      <c r="D35" t="s">
         <v>3</v>
       </c>
-      <c r="E34" t="s">
+      <c r="E35" t="s">
         <v>4</v>
       </c>
-      <c r="F34" t="s">
+      <c r="F35" t="s">
         <v>5</v>
       </c>
-      <c r="G34" t="s">
+      <c r="G35" t="s">
         <v>6</v>
       </c>
-      <c r="H34" t="s">
+      <c r="H35" t="s">
         <v>7</v>
       </c>
-      <c r="I34" t="s">
+      <c r="I35" t="s">
         <v>8</v>
       </c>
-      <c r="J34" t="s">
+      <c r="J35" t="s">
         <v>9</v>
       </c>
-      <c r="K34" t="s">
+      <c r="K35" t="s">
         <v>10</v>
       </c>
-      <c r="L34" t="s">
+      <c r="L35" t="s">
         <v>11</v>
       </c>
-      <c r="M34" t="s">
+      <c r="M35" t="s">
         <v>12</v>
       </c>
-      <c r="N34" t="s">
+      <c r="N35" t="s">
         <v>13</v>
       </c>
-      <c r="O34" t="s">
+      <c r="O35" t="s">
         <v>14</v>
       </c>
-      <c r="P34" t="s">
+      <c r="P35" t="s">
         <v>15</v>
       </c>
-      <c r="Q34" t="s">
+      <c r="Q35" t="s">
         <v>16</v>
       </c>
-      <c r="R34" t="s">
+      <c r="R35" t="s">
         <v>17</v>
       </c>
-      <c r="S34" t="s">
+      <c r="S35" t="s">
         <v>18</v>
       </c>
-      <c r="T34" t="s">
+      <c r="T35" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A35" t="s">
+    <row r="36" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A36" s="2" t="s">
         <v>20</v>
-      </c>
-      <c r="B35" t="s">
-        <v>21</v>
-      </c>
-      <c r="C35">
-        <v>4</v>
-      </c>
-      <c r="D35">
-        <v>29525.427309999999</v>
-      </c>
-      <c r="E35">
-        <v>80391.755990000005</v>
-      </c>
-      <c r="F35">
-        <v>0.79280104200000001</v>
-      </c>
-      <c r="G35">
-        <v>5050.6365619999997</v>
-      </c>
-      <c r="H35">
-        <v>4678.3390820000004</v>
-      </c>
-      <c r="I35">
-        <v>2508.6600360000002</v>
-      </c>
-      <c r="J35">
-        <v>12237.635679999999</v>
-      </c>
-      <c r="K35">
-        <v>13920</v>
-      </c>
-      <c r="L35">
-        <v>2841.544922</v>
-      </c>
-      <c r="M35">
-        <v>5380.5444360000001</v>
-      </c>
-      <c r="N35">
-        <v>279.27307350000001</v>
-      </c>
-      <c r="O35">
-        <v>0</v>
-      </c>
-      <c r="P35">
-        <v>63734.6679</v>
-      </c>
-      <c r="Q35">
-        <v>1078.4492829999999</v>
-      </c>
-      <c r="R35">
-        <v>624.70352849999995</v>
-      </c>
-      <c r="S35">
-        <v>13.014656840000001</v>
-      </c>
-      <c r="T35">
-        <v>27.514184579999998</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A36" t="s">
-        <v>22</v>
       </c>
       <c r="B36" t="s">
         <v>21</v>
@@ -2064,54 +2132,116 @@
         <v>4</v>
       </c>
       <c r="D36">
+        <v>29525.427309999999</v>
+      </c>
+      <c r="E36">
+        <v>80391.755990000005</v>
+      </c>
+      <c r="F36">
+        <v>0.79280104200000001</v>
+      </c>
+      <c r="G36">
+        <v>5050.6365619999997</v>
+      </c>
+      <c r="H36">
+        <v>4678.3390820000004</v>
+      </c>
+      <c r="I36">
+        <v>2508.6600360000002</v>
+      </c>
+      <c r="J36">
+        <v>12237.635679999999</v>
+      </c>
+      <c r="K36">
+        <v>13920</v>
+      </c>
+      <c r="L36">
+        <v>2841.544922</v>
+      </c>
+      <c r="M36">
+        <v>5380.5444360000001</v>
+      </c>
+      <c r="N36">
+        <v>279.27307350000001</v>
+      </c>
+      <c r="O36">
+        <v>0</v>
+      </c>
+      <c r="P36">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q36">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R36">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S36">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T36">
+        <v>27.514184579999998</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A37" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B37" t="s">
+        <v>21</v>
+      </c>
+      <c r="C37">
+        <v>4</v>
+      </c>
+      <c r="D37">
         <v>30655.78772</v>
       </c>
-      <c r="E36">
+      <c r="E37">
         <v>79415.835619999998</v>
       </c>
-      <c r="F36">
+      <c r="F37">
         <v>0.81677700399999997</v>
       </c>
-      <c r="G36">
+      <c r="G37">
         <v>5129.9926729999997</v>
       </c>
-      <c r="H36">
+      <c r="H37">
         <v>5254.1641179999997</v>
       </c>
-      <c r="I36">
+      <c r="I37">
         <v>4834.2260249999999</v>
       </c>
-      <c r="J36">
+      <c r="J37">
         <v>15218.382820000001</v>
       </c>
-      <c r="K36">
+      <c r="K37">
         <v>13875.1543</v>
       </c>
-      <c r="L36">
+      <c r="L37">
         <v>3140.6678670000001</v>
       </c>
-      <c r="M36">
+      <c r="M37">
         <v>5340.9854210000003</v>
       </c>
-      <c r="N36">
+      <c r="N37">
         <v>286.5902719</v>
       </c>
-      <c r="O36">
-        <v>0</v>
-      </c>
-      <c r="P36">
+      <c r="O37">
+        <v>0</v>
+      </c>
+      <c r="P37">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q36">
+      <c r="Q37">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R36">
+      <c r="R37">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S36">
+      <c r="S37">
         <v>452.7322633</v>
       </c>
-      <c r="T36">
+      <c r="T37">
         <v>5.8154128590000003</v>
       </c>
     </row>

</xml_diff>

<commit_message>
flow and both for 2 trains
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F689B85-74EF-4482-8A79-E9A59BAFD73B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A42202-C387-4414-A65D-31F46AB4A59C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9780" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-86" yWindow="0" windowWidth="16629" windowHeight="17880" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -35,12 +35,21 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={059B2785-9A39-4C22-958C-B8BAB93BD95A}</author>
     <author>tc={ABAC2AC6-7A74-4F44-BF4E-754717C772A0}</author>
     <author>tc={9CE96C07-E110-41BE-B453-65310D0A2128}</author>
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
   </authors>
   <commentList>
-    <comment ref="A24" authorId="0" shapeId="0" xr:uid="{ABAC2AC6-7A74-4F44-BF4E-754717C772A0}">
+    <comment ref="A19" authorId="0" shapeId="0" xr:uid="{059B2785-9A39-4C22-958C-B8BAB93BD95A}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Flex_type = rr has same solution</t>
+      </text>
+    </comment>
+    <comment ref="A24" authorId="1" shapeId="0" xr:uid="{ABAC2AC6-7A74-4F44-BF4E-754717C772A0}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -48,7 +57,7 @@
     Have to re-run with fixed uf recovery and the 2nd order surrogate</t>
       </text>
     </comment>
-    <comment ref="A28" authorId="1" shapeId="0" xr:uid="{9CE96C07-E110-41BE-B453-65310D0A2128}">
+    <comment ref="A28" authorId="2" shapeId="0" xr:uid="{9CE96C07-E110-41BE-B453-65310D0A2128}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -56,7 +65,7 @@
     Summer is the summer hot weekdays + high weekends.</t>
       </text>
     </comment>
-    <comment ref="A29" authorId="2" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A29" authorId="3" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -1033,6 +1042,9 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="A19" dT="2026-05-29T21:01:16.53" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{059B2785-9A39-4C22-958C-B8BAB93BD95A}">
+    <text>Flex_type = rr has same solution</text>
+  </threadedComment>
   <threadedComment ref="A24" dT="2026-05-28T22:11:07.28" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{ABAC2AC6-7A74-4F44-BF4E-754717C772A0}">
     <text>Have to re-run with fixed uf recovery and the 2nd order surrogate</text>
   </threadedComment>
@@ -1709,6 +1721,57 @@
       <c r="C19">
         <v>2</v>
       </c>
+      <c r="D19">
+        <v>118366.61344104999</v>
+      </c>
+      <c r="E19">
+        <v>282322.94999999902</v>
+      </c>
+      <c r="F19">
+        <v>0.84980195895491895</v>
+      </c>
+      <c r="G19">
+        <v>20300.730727046899</v>
+      </c>
+      <c r="H19">
+        <v>6562.4436275804401</v>
+      </c>
+      <c r="I19">
+        <v>6015.5411364260799</v>
+      </c>
+      <c r="J19">
+        <v>32878.715491053401</v>
+      </c>
+      <c r="K19">
+        <v>50869.000000000102</v>
+      </c>
+      <c r="L19">
+        <v>15311.5689999966</v>
+      </c>
+      <c r="M19">
+        <v>19307.328949999701</v>
+      </c>
+      <c r="N19">
+        <v>999.49269129581296</v>
+      </c>
+      <c r="O19">
+        <v>0</v>
+      </c>
+      <c r="P19">
+        <v>239918.595967931</v>
+      </c>
+      <c r="Q19">
+        <v>1466.2124273779</v>
+      </c>
+      <c r="R19">
+        <v>16513.412838507898</v>
+      </c>
+      <c r="S19">
+        <v>351.34920932995601</v>
+      </c>
+      <c r="T19">
+        <v>1.0883139285619701</v>
+      </c>
     </row>
     <row r="21" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A21" t="s">

</xml_diff>

<commit_message>
running for 4 flexible trains
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73A42202-C387-4414-A65D-31F46AB4A59C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3DD61BE-730F-4810-8CF1-521B0F0E811A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-86" yWindow="0" windowWidth="16629" windowHeight="17880" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -174,7 +174,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -308,12 +308,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1060,22 +1054,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:T37"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="12.4609375" customWidth="1"/>
-    <col min="5" max="5" width="10.3046875" customWidth="1"/>
-    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.53515625" customWidth="1"/>
-    <col min="9" max="9" width="9.07421875" customWidth="1"/>
-    <col min="20" max="20" width="7.84375" customWidth="1"/>
+    <col min="3" max="3" width="12.453125" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.54296875" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1137,7 +1131,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1199,7 +1193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1261,7 +1255,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1323,7 +1317,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -1385,7 +1379,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1447,7 +1441,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1509,7 +1503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1571,7 +1565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -1633,7 +1627,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1643,8 +1637,53 @@
       <c r="C15">
         <v>1</v>
       </c>
-    </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="D15">
+        <v>112765.52483279799</v>
+      </c>
+      <c r="E15">
+        <v>282322.94999999902</v>
+      </c>
+      <c r="F15">
+        <v>0.82996266282879405</v>
+      </c>
+      <c r="G15">
+        <v>18232.263309167702</v>
+      </c>
+      <c r="H15">
+        <v>6458.86539103209</v>
+      </c>
+      <c r="I15">
+        <v>2586.49818260132</v>
+      </c>
+      <c r="J15">
+        <v>27277.626882801102</v>
+      </c>
+      <c r="K15">
+        <v>50868.999999997599</v>
+      </c>
+      <c r="L15">
+        <v>15311.568999999699</v>
+      </c>
+      <c r="M15">
+        <v>19307.328949999501</v>
+      </c>
+      <c r="N15">
+        <v>994.09650999907501</v>
+      </c>
+      <c r="O15">
+        <v>0</v>
+      </c>
+      <c r="P15">
+        <v>234317.507359679</v>
+      </c>
+      <c r="Q15">
+        <v>1466.60679969635</v>
+      </c>
+      <c r="R15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1654,8 +1693,53 @@
       <c r="C16">
         <v>1</v>
       </c>
-    </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="D16">
+        <v>121661.732552156</v>
+      </c>
+      <c r="E16">
+        <v>282322.94999999902</v>
+      </c>
+      <c r="F16">
+        <v>0.86147341220059803</v>
+      </c>
+      <c r="G16">
+        <v>20583.8776149273</v>
+      </c>
+      <c r="H16">
+        <v>6564.2083881818999</v>
+      </c>
+      <c r="I16">
+        <v>9025.7485990471305</v>
+      </c>
+      <c r="J16">
+        <v>36173.834602156297</v>
+      </c>
+      <c r="K16">
+        <v>50869</v>
+      </c>
+      <c r="L16">
+        <v>15311.569</v>
+      </c>
+      <c r="M16">
+        <v>19307.328949999999</v>
+      </c>
+      <c r="N16">
+        <v>994.09650999907501</v>
+      </c>
+      <c r="O16">
+        <v>0</v>
+      </c>
+      <c r="P16">
+        <v>243213.715079038</v>
+      </c>
+      <c r="Q16">
+        <v>1466.6067124359399</v>
+      </c>
+      <c r="R16">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1711,7 +1795,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -1722,34 +1806,34 @@
         <v>2</v>
       </c>
       <c r="D19">
-        <v>118366.61344104999</v>
+        <v>118393.04078958899</v>
       </c>
       <c r="E19">
-        <v>282322.94999999902</v>
+        <v>282322.95</v>
       </c>
       <c r="F19">
-        <v>0.84980195895491895</v>
+        <v>0.84989556575712399</v>
       </c>
       <c r="G19">
-        <v>20300.730727046899</v>
+        <v>20322.3387120884</v>
       </c>
       <c r="H19">
-        <v>6562.4436275804401</v>
+        <v>6565.6354226596604</v>
       </c>
       <c r="I19">
-        <v>6015.5411364260799</v>
+        <v>6017.1687048407903</v>
       </c>
       <c r="J19">
-        <v>32878.715491053401</v>
+        <v>32905.142839588902</v>
       </c>
       <c r="K19">
         <v>50869.000000000102</v>
       </c>
       <c r="L19">
-        <v>15311.5689999966</v>
+        <v>15311.568999999899</v>
       </c>
       <c r="M19">
-        <v>19307.328949999701</v>
+        <v>19307.328949999999</v>
       </c>
       <c r="N19">
         <v>999.49269129581296</v>
@@ -1758,22 +1842,22 @@
         <v>0</v>
       </c>
       <c r="P19">
-        <v>239918.595967931</v>
+        <v>239945.02331647</v>
       </c>
       <c r="Q19">
-        <v>1466.2124273779</v>
+        <v>1466.9255534444001</v>
       </c>
       <c r="R19">
-        <v>16513.412838507898</v>
+        <v>22473.732168664301</v>
       </c>
       <c r="S19">
-        <v>351.34920932995601</v>
+        <v>351.15206513537998</v>
       </c>
       <c r="T19">
-        <v>1.0883139285619701</v>
-      </c>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
+        <v>0.79850332454920403</v>
+      </c>
+    </row>
+    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -1829,7 +1913,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1839,8 +1923,59 @@
       <c r="C22">
         <v>2</v>
       </c>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="D22">
+        <v>111145.74490869101</v>
+      </c>
+      <c r="E22">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F22">
+        <v>0.824643839220908</v>
+      </c>
+      <c r="G22">
+        <v>18242.859043300999</v>
+      </c>
+      <c r="H22">
+        <v>4851.8098358536599</v>
+      </c>
+      <c r="I22">
+        <v>2606.42587512207</v>
+      </c>
+      <c r="J22">
+        <v>25701.094754276801</v>
+      </c>
+      <c r="K22">
+        <v>50843.219249379203</v>
+      </c>
+      <c r="L22">
+        <v>15303.8931025696</v>
+      </c>
+      <c r="M22">
+        <v>19297.537802465198</v>
+      </c>
+      <c r="N22">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O22">
+        <v>0</v>
+      </c>
+      <c r="P22">
+        <v>232697.72743557199</v>
+      </c>
+      <c r="Q22">
+        <v>1101.6946284421099</v>
+      </c>
+      <c r="R22">
+        <v>0</v>
+      </c>
+      <c r="S22">
+        <v>487.22587310308802</v>
+      </c>
+      <c r="T22">
+        <v>1.75628458077399</v>
+      </c>
+    </row>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -1902,7 +2037,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>22</v>
       </c>
@@ -1964,12 +2099,12 @@
         <v>1.63318791126541</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -1980,7 +2115,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>20</v>
       </c>
@@ -1991,7 +2126,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2054,7 +2189,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>22</v>
       </c>
@@ -2117,12 +2252,12 @@
         <v>0.51068072492979899</v>
       </c>
     </row>
-    <row r="34" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>0</v>
       </c>
@@ -2184,7 +2319,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>20</v>
       </c>
@@ -2246,7 +2381,7 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="37" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>22</v>
       </c>

</xml_diff>

<commit_message>
Baseline weeks for RTP
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3DD61BE-730F-4810-8CF1-521B0F0E811A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC0C4A69-FF19-43A2-9DEB-ED14130D8A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -78,7 +78,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="31">
   <si>
     <t>Season</t>
   </si>
@@ -168,6 +168,9 @@
   </si>
   <si>
     <t>Maximum Power</t>
+  </si>
+  <si>
+    <t>New, not sure feed and flow are different…</t>
   </si>
 </sst>
 </file>
@@ -1053,13 +1056,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:T37"/>
+  <dimension ref="A1:T39"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="12.453125" customWidth="1"/>
     <col min="5" max="5" width="10.26953125" customWidth="1"/>
     <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.54296875" customWidth="1"/>
+    <col min="7" max="7" width="15.26953125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.08984375" customWidth="1"/>
     <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
@@ -2191,255 +2194,308 @@
     </row>
     <row r="31" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D31">
+        <v>116833.749486644</v>
+      </c>
+      <c r="E31">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F31">
+        <v>0.84480122530439805</v>
+      </c>
+      <c r="G31">
+        <v>23535.478746437901</v>
+      </c>
+      <c r="H31">
+        <v>6941.2778055266899</v>
+      </c>
+      <c r="I31">
+        <v>912.48005352310201</v>
+      </c>
+      <c r="J31">
+        <v>31389.236605487698</v>
+      </c>
+      <c r="K31">
+        <v>50843.184005923998</v>
+      </c>
+      <c r="L31">
+        <v>15303.798385784499</v>
+      </c>
+      <c r="M31">
+        <v>19297.5304894484</v>
+      </c>
+      <c r="N31">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O31">
+        <v>0</v>
+      </c>
+      <c r="P31">
+        <v>238385.73201352599</v>
+      </c>
+      <c r="Q31">
+        <v>1101.67495873487</v>
+      </c>
+      <c r="R31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A32" s="2"/>
+    </row>
+    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A33" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B33" t="s">
         <v>21</v>
       </c>
-      <c r="C31">
+      <c r="C33">
         <v>4</v>
       </c>
-      <c r="D31">
+      <c r="D33">
         <v>113598.307758221</v>
       </c>
-      <c r="E31">
+      <c r="E33">
         <v>282179.67123287398</v>
       </c>
-      <c r="F31">
+      <c r="F33">
         <v>0.83333533297315499</v>
       </c>
-      <c r="G31">
+      <c r="G33">
         <v>21005.263452339499</v>
       </c>
-      <c r="H31">
+      <c r="H33">
         <v>9419.1929847336105</v>
       </c>
-      <c r="I31">
-        <v>0</v>
-      </c>
-      <c r="J31">
-        <f>SUM(G31:I31)</f>
+      <c r="I33">
+        <v>0</v>
+      </c>
+      <c r="J33">
+        <f>SUM(G33:I33)</f>
         <v>30424.45643707311</v>
       </c>
-      <c r="K31">
+      <c r="K33">
         <v>48819.627456497903</v>
       </c>
-      <c r="L31">
+      <c r="L33">
         <v>14784.690159207899</v>
       </c>
-      <c r="M31">
+      <c r="M33">
         <v>19569.533705442402</v>
       </c>
-      <c r="N31">
+      <c r="N33">
         <v>1040.9289460857101</v>
       </c>
-      <c r="O31">
-        <v>0</v>
-      </c>
-      <c r="P31">
+      <c r="O33">
+        <v>0</v>
+      </c>
+      <c r="P33">
         <v>235150.29028510299</v>
       </c>
-      <c r="Q31">
+      <c r="Q33">
         <v>1494.95371016114</v>
       </c>
-      <c r="R31">
+      <c r="R33">
         <v>40078.803663142098</v>
       </c>
-      <c r="S31">
+      <c r="S33">
         <v>910.88190143504903</v>
       </c>
-      <c r="T31">
+      <c r="T33">
         <v>0.51068072492979899</v>
       </c>
     </row>
-    <row r="34" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A34" s="1" t="s">
+    <row r="36" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A36" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="35" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A35" t="s">
-        <v>0</v>
-      </c>
-      <c r="B35" t="s">
+    <row r="37" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>0</v>
+      </c>
+      <c r="B37" t="s">
         <v>1</v>
       </c>
-      <c r="C35" t="s">
+      <c r="C37" t="s">
         <v>2</v>
       </c>
-      <c r="D35" t="s">
+      <c r="D37" t="s">
         <v>3</v>
       </c>
-      <c r="E35" t="s">
+      <c r="E37" t="s">
         <v>4</v>
       </c>
-      <c r="F35" t="s">
+      <c r="F37" t="s">
         <v>5</v>
       </c>
-      <c r="G35" t="s">
+      <c r="G37" t="s">
         <v>6</v>
       </c>
-      <c r="H35" t="s">
+      <c r="H37" t="s">
         <v>7</v>
       </c>
-      <c r="I35" t="s">
+      <c r="I37" t="s">
         <v>8</v>
       </c>
-      <c r="J35" t="s">
+      <c r="J37" t="s">
         <v>9</v>
       </c>
-      <c r="K35" t="s">
+      <c r="K37" t="s">
         <v>10</v>
       </c>
-      <c r="L35" t="s">
+      <c r="L37" t="s">
         <v>11</v>
       </c>
-      <c r="M35" t="s">
+      <c r="M37" t="s">
         <v>12</v>
       </c>
-      <c r="N35" t="s">
+      <c r="N37" t="s">
         <v>13</v>
       </c>
-      <c r="O35" t="s">
+      <c r="O37" t="s">
         <v>14</v>
       </c>
-      <c r="P35" t="s">
+      <c r="P37" t="s">
         <v>15</v>
       </c>
-      <c r="Q35" t="s">
+      <c r="Q37" t="s">
         <v>16</v>
       </c>
-      <c r="R35" t="s">
+      <c r="R37" t="s">
         <v>17</v>
       </c>
-      <c r="S35" t="s">
+      <c r="S37" t="s">
         <v>18</v>
       </c>
-      <c r="T35" t="s">
+      <c r="T37" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="36" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A36" s="2" t="s">
+    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B36" t="s">
+      <c r="B38" t="s">
         <v>21</v>
       </c>
-      <c r="C36">
+      <c r="C38">
         <v>4</v>
       </c>
-      <c r="D36">
+      <c r="D38">
         <v>29525.427309999999</v>
       </c>
-      <c r="E36">
+      <c r="E38">
         <v>80391.755990000005</v>
       </c>
-      <c r="F36">
+      <c r="F38">
         <v>0.79280104200000001</v>
       </c>
-      <c r="G36">
+      <c r="G38">
         <v>5050.6365619999997</v>
       </c>
-      <c r="H36">
+      <c r="H38">
         <v>4678.3390820000004</v>
       </c>
-      <c r="I36">
+      <c r="I38">
         <v>2508.6600360000002</v>
       </c>
-      <c r="J36">
+      <c r="J38">
         <v>12237.635679999999</v>
       </c>
-      <c r="K36">
+      <c r="K38">
         <v>13920</v>
       </c>
-      <c r="L36">
+      <c r="L38">
         <v>2841.544922</v>
       </c>
-      <c r="M36">
+      <c r="M38">
         <v>5380.5444360000001</v>
       </c>
-      <c r="N36">
+      <c r="N38">
         <v>279.27307350000001</v>
       </c>
-      <c r="O36">
-        <v>0</v>
-      </c>
-      <c r="P36">
+      <c r="O38">
+        <v>0</v>
+      </c>
+      <c r="P38">
         <v>63734.6679</v>
       </c>
-      <c r="Q36">
+      <c r="Q38">
         <v>1078.4492829999999</v>
       </c>
-      <c r="R36">
+      <c r="R38">
         <v>624.70352849999995</v>
       </c>
-      <c r="S36">
+      <c r="S38">
         <v>13.014656840000001</v>
       </c>
-      <c r="T36">
+      <c r="T38">
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="37" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A37" s="2" t="s">
+    <row r="39" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A39" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B37" t="s">
+      <c r="B39" t="s">
         <v>21</v>
       </c>
-      <c r="C37">
+      <c r="C39">
         <v>4</v>
       </c>
-      <c r="D37">
+      <c r="D39">
         <v>30655.78772</v>
       </c>
-      <c r="E37">
+      <c r="E39">
         <v>79415.835619999998</v>
       </c>
-      <c r="F37">
+      <c r="F39">
         <v>0.81677700399999997</v>
       </c>
-      <c r="G37">
+      <c r="G39">
         <v>5129.9926729999997</v>
       </c>
-      <c r="H37">
+      <c r="H39">
         <v>5254.1641179999997</v>
       </c>
-      <c r="I37">
+      <c r="I39">
         <v>4834.2260249999999</v>
       </c>
-      <c r="J37">
+      <c r="J39">
         <v>15218.382820000001</v>
       </c>
-      <c r="K37">
+      <c r="K39">
         <v>13875.1543</v>
       </c>
-      <c r="L37">
+      <c r="L39">
         <v>3140.6678670000001</v>
       </c>
-      <c r="M37">
+      <c r="M39">
         <v>5340.9854210000003</v>
       </c>
-      <c r="N37">
+      <c r="N39">
         <v>286.5902719</v>
       </c>
-      <c r="O37">
-        <v>0</v>
-      </c>
-      <c r="P37">
+      <c r="O39">
+        <v>0</v>
+      </c>
+      <c r="P39">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q37">
+      <c r="Q39">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R37">
+      <c r="R39">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S37">
+      <c r="S39">
         <v>452.7322633</v>
       </c>
-      <c r="T37">
+      <c r="T39">
         <v>5.8154128590000003</v>
       </c>
     </row>

</xml_diff>

<commit_message>
RTP baseline but with both flexible
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC0C4A69-FF19-43A2-9DEB-ED14130D8A44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B0FB9A-F158-4610-9094-FF54D891DF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -1057,22 +1057,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:T39"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="3" max="3" width="12.453125" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.08984375" customWidth="1"/>
-    <col min="20" max="20" width="7.81640625" customWidth="1"/>
+    <col min="3" max="3" width="12.4609375" customWidth="1"/>
+    <col min="5" max="5" width="10.23046875" customWidth="1"/>
+    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.23046875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.07421875" customWidth="1"/>
+    <col min="20" max="20" width="7.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1134,7 +1134,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1196,7 +1196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1258,7 +1258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1320,7 +1320,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -1382,7 +1382,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1444,7 +1444,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1506,7 +1506,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1568,7 +1568,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -1630,7 +1630,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1686,7 +1686,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1742,7 +1742,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1798,7 +1798,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -1860,7 +1860,7 @@
         <v>0.79850332454920403</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -1916,7 +1916,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1978,7 +1978,7 @@
         <v>1.75628458077399</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -2040,7 +2040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A25" s="2" t="s">
         <v>22</v>
       </c>
@@ -2102,12 +2102,12 @@
         <v>1.63318791126541</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -2117,8 +2117,59 @@
       <c r="C28">
         <v>0</v>
       </c>
-    </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="D28">
+        <v>155096.37936009499</v>
+      </c>
+      <c r="E28">
+        <v>374203.2</v>
+      </c>
+      <c r="F28">
+        <v>0.73929982930925298</v>
+      </c>
+      <c r="G28">
+        <v>31331.647259594902</v>
+      </c>
+      <c r="H28">
+        <v>9240.58822328104</v>
+      </c>
+      <c r="I28">
+        <v>1214.7406677558599</v>
+      </c>
+      <c r="J28">
+        <v>41786.976150631803</v>
+      </c>
+      <c r="K28">
+        <v>67424.000002429399</v>
+      </c>
+      <c r="L28">
+        <v>20294.624006529499</v>
+      </c>
+      <c r="M28">
+        <v>25590.779200504101</v>
+      </c>
+      <c r="N28">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O28">
+        <v>0</v>
+      </c>
+      <c r="P28">
+        <v>276648.361886976</v>
+      </c>
+      <c r="Q28">
+        <v>1466.6067163402599</v>
+      </c>
+      <c r="R28">
+        <v>0</v>
+      </c>
+      <c r="S28">
+        <v>0</v>
+      </c>
+      <c r="T28">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>20</v>
       </c>
@@ -2128,8 +2179,59 @@
       <c r="C29">
         <v>0</v>
       </c>
-    </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="D29">
+        <v>247948.64160389101</v>
+      </c>
+      <c r="E29">
+        <v>374203.2</v>
+      </c>
+      <c r="F29">
+        <v>0.98743309552342695</v>
+      </c>
+      <c r="G29">
+        <v>118659.96685142</v>
+      </c>
+      <c r="H29">
+        <v>9240.5882208594503</v>
+      </c>
+      <c r="I29">
+        <v>6738.6833231561404</v>
+      </c>
+      <c r="J29">
+        <v>134639.23839543501</v>
+      </c>
+      <c r="K29">
+        <v>67424.000002171</v>
+      </c>
+      <c r="L29">
+        <v>20294.624005833801</v>
+      </c>
+      <c r="M29">
+        <v>25590.779200450401</v>
+      </c>
+      <c r="N29">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O29">
+        <v>0</v>
+      </c>
+      <c r="P29">
+        <v>369500.62413077202</v>
+      </c>
+      <c r="Q29">
+        <v>1466.60671595592</v>
+      </c>
+      <c r="R29">
+        <v>0</v>
+      </c>
+      <c r="S29">
+        <v>0</v>
+      </c>
+      <c r="T29">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
@@ -2192,7 +2294,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A31" s="2" t="s">
         <v>30</v>
       </c>
@@ -2241,11 +2343,17 @@
       <c r="R31">
         <v>0</v>
       </c>
-    </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="S31">
+        <v>0</v>
+      </c>
+      <c r="T31">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A32" s="2"/>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A33" s="2" t="s">
         <v>22</v>
       </c>
@@ -2308,12 +2416,12 @@
         <v>0.51068072492979899</v>
       </c>
     </row>
-    <row r="36" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
       <c r="A36" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="37" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>0</v>
       </c>
@@ -2375,7 +2483,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
       <c r="A38" s="2" t="s">
         <v>20</v>
       </c>
@@ -2437,7 +2545,7 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="39" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
       <c r="A39" s="2" t="s">
         <v>22</v>
       </c>

</xml_diff>

<commit_message>
Re-adding the first four days limitation
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5B0FB9A-F158-4610-9094-FF54D891DF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A3E3C7-C3D9-4112-85AA-AACC7D8922DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="68505" yWindow="8550" windowWidth="18000" windowHeight="15585" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -39,6 +39,7 @@
     <author>tc={ABAC2AC6-7A74-4F44-BF4E-754717C772A0}</author>
     <author>tc={9CE96C07-E110-41BE-B453-65310D0A2128}</author>
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
+    <author>tc={44AB14B7-66C1-445B-8271-3F9869928B60}</author>
   </authors>
   <commentList>
     <comment ref="A19" authorId="0" shapeId="0" xr:uid="{059B2785-9A39-4C22-958C-B8BAB93BD95A}">
@@ -73,12 +74,20 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
+    <comment ref="T30" authorId="4" shapeId="0" xr:uid="{44AB14B7-66C1-445B-8271-3F9869928B60}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    The whole baseline for this might be corrupted</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="31">
   <si>
     <t>Season</t>
   </si>
@@ -177,7 +186,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -311,6 +320,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1051,12 +1066,15 @@
   <threadedComment ref="A29" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
     <text>Winter is low winter weekdays + low weekends</text>
   </threadedComment>
+  <threadedComment ref="T30" dT="2026-06-01T20:16:04.04" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{44AB14B7-66C1-445B-8271-3F9869928B60}">
+    <text>The whole baseline for this might be corrupted</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:T39"/>
+  <dimension ref="A1:W42"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="3" max="3" width="12.4609375" customWidth="1"/>
@@ -1742,7 +1760,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1798,7 +1816,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -1860,7 +1878,7 @@
         <v>0.79850332454920403</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -1916,7 +1934,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1978,7 +1996,7 @@
         <v>1.75628458077399</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -2040,7 +2058,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A25" s="2" t="s">
         <v>22</v>
       </c>
@@ -2102,12 +2120,12 @@
         <v>1.63318791126541</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -2169,7 +2187,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.4">
       <c r="A29" t="s">
         <v>20</v>
       </c>
@@ -2231,46 +2249,45 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A30" s="2" t="s">
-        <v>20</v>
+    <row r="30" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A30" t="s">
+        <v>22</v>
       </c>
       <c r="B30" t="s">
         <v>21</v>
       </c>
       <c r="C30">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D30">
-        <v>108960.613539453</v>
+        <v>171865.08676903401</v>
       </c>
       <c r="E30">
-        <v>282179.67123287701</v>
+        <v>282179.67634316301</v>
       </c>
       <c r="F30">
-        <v>0.81690008021909599</v>
+        <v>1.0398235376068901</v>
       </c>
       <c r="G30">
-        <v>23571.632136721099</v>
+        <v>74067.572494025299</v>
       </c>
       <c r="H30">
-        <v>6951.9409028971204</v>
+        <v>7441.88027751749</v>
       </c>
       <c r="I30">
-        <v>913.88179307768496</v>
+        <v>4044.9309060690198</v>
       </c>
       <c r="J30">
-        <f>SUM(G30:I30)</f>
-        <v>31437.454832695905</v>
+        <v>85554.383677611797</v>
       </c>
       <c r="K30">
-        <v>48809.460212750702</v>
+        <v>51065.569692514699</v>
       </c>
       <c r="L30">
-        <v>9838.1656916422507</v>
+        <v>15901.4577210732</v>
       </c>
       <c r="M30">
-        <v>18875.532802364902</v>
+        <v>19343.675677834799</v>
       </c>
       <c r="N30">
         <v>992.31070788530405</v>
@@ -2279,54 +2296,60 @@
         <v>0</v>
       </c>
       <c r="P30">
-        <v>230512.59606633501</v>
+        <v>293417.06929591601</v>
       </c>
       <c r="Q30">
-        <v>1103.3673370121001</v>
+        <v>1181.12736261847</v>
       </c>
       <c r="R30">
-        <v>0</v>
+        <v>7149.8947939583104</v>
       </c>
       <c r="S30">
-        <v>0</v>
+        <v>210.29102335171501</v>
       </c>
       <c r="T30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A31" s="2" t="s">
-        <v>30</v>
+        <v>-4.8547669539218203</v>
+      </c>
+    </row>
+    <row r="31" spans="1:23" x14ac:dyDescent="0.4">
+      <c r="A31" t="s">
+        <v>20</v>
+      </c>
+      <c r="B31" t="s">
+        <v>21</v>
+      </c>
+      <c r="C31">
+        <v>0</v>
       </c>
       <c r="D31">
-        <v>116833.749486644</v>
+        <v>117032.41959359701</v>
       </c>
       <c r="E31">
-        <v>282179.67123287602</v>
+        <v>282179.67123286898</v>
       </c>
       <c r="F31">
-        <v>0.84480122530439805</v>
+        <v>0.845505280653571</v>
       </c>
       <c r="G31">
-        <v>23535.478746437901</v>
+        <v>23683.129427060001</v>
       </c>
       <c r="H31">
-        <v>6941.2778055266899</v>
+        <v>6986.3695969997798</v>
       </c>
       <c r="I31">
-        <v>912.48005352310201</v>
+        <v>918.40768838365295</v>
       </c>
       <c r="J31">
-        <v>31389.236605487698</v>
+        <v>31587.906712443499</v>
       </c>
       <c r="K31">
-        <v>50843.184005923998</v>
+        <v>50843.1840059237</v>
       </c>
       <c r="L31">
-        <v>15303.798385784499</v>
+        <v>15303.7983857823</v>
       </c>
       <c r="M31">
-        <v>19297.5304894484</v>
+        <v>19297.530489448101</v>
       </c>
       <c r="N31">
         <v>992.31070788530405</v>
@@ -2335,27 +2358,33 @@
         <v>0</v>
       </c>
       <c r="P31">
-        <v>238385.73201352599</v>
+        <v>238584.402120479</v>
       </c>
       <c r="Q31">
-        <v>1101.67495873487</v>
+        <v>1108.83163779344</v>
       </c>
       <c r="R31">
         <v>0</v>
       </c>
       <c r="S31">
-        <v>0</v>
+        <v>230512.59606633501</v>
       </c>
       <c r="T31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A32" s="2"/>
+        <v>1103.3673370121001</v>
+      </c>
+      <c r="U31">
+        <v>0</v>
+      </c>
+      <c r="V31">
+        <v>0</v>
+      </c>
+      <c r="W31">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A33" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B33" t="s">
         <v>21</v>
@@ -2364,248 +2393,312 @@
         <v>4</v>
       </c>
       <c r="D33">
-        <v>113598.307758221</v>
+        <v>108960.613539453</v>
       </c>
       <c r="E33">
-        <v>282179.67123287398</v>
+        <v>282179.67123287701</v>
       </c>
       <c r="F33">
-        <v>0.83333533297315499</v>
+        <v>0.81690008021909599</v>
       </c>
       <c r="G33">
-        <v>21005.263452339499</v>
+        <v>23571.632136721099</v>
       </c>
       <c r="H33">
-        <v>9419.1929847336105</v>
+        <v>6951.9409028971204</v>
       </c>
       <c r="I33">
-        <v>0</v>
+        <v>913.88179307768496</v>
       </c>
       <c r="J33">
         <f>SUM(G33:I33)</f>
+        <v>31437.454832695905</v>
+      </c>
+      <c r="K33">
+        <v>48809.460212750702</v>
+      </c>
+      <c r="L33">
+        <v>9838.1656916422507</v>
+      </c>
+      <c r="M33">
+        <v>18875.532802364902</v>
+      </c>
+      <c r="N33">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O33">
+        <v>0</v>
+      </c>
+      <c r="P33">
+        <v>238385.73201352599</v>
+      </c>
+      <c r="Q33">
+        <v>1101.67495873487</v>
+      </c>
+      <c r="R33">
+        <v>0</v>
+      </c>
+      <c r="S33">
+        <v>0</v>
+      </c>
+      <c r="T33">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A34" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D34">
+        <v>116833.749486644</v>
+      </c>
+      <c r="E34">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F34">
+        <v>0.84480122530439805</v>
+      </c>
+      <c r="G34">
+        <v>23535.478746437901</v>
+      </c>
+      <c r="H34">
+        <v>6941.2778055266899</v>
+      </c>
+      <c r="I34">
+        <v>912.48005352310201</v>
+      </c>
+      <c r="J34">
+        <v>31389.236605487698</v>
+      </c>
+      <c r="K34">
+        <v>50843.184005923998</v>
+      </c>
+      <c r="L34">
+        <v>15303.798385784499</v>
+      </c>
+      <c r="M34">
+        <v>19297.5304894484</v>
+      </c>
+      <c r="N34">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O34">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A35" s="2"/>
+      <c r="P35">
+        <v>235150.29028510299</v>
+      </c>
+      <c r="Q35">
+        <v>1494.95371016114</v>
+      </c>
+      <c r="R35">
+        <v>40078.803663142098</v>
+      </c>
+      <c r="S35">
+        <v>910.88190143504903</v>
+      </c>
+      <c r="T35">
+        <v>0.51068072492979899</v>
+      </c>
+    </row>
+    <row r="36" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A36" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B36" t="s">
+        <v>21</v>
+      </c>
+      <c r="C36">
+        <v>4</v>
+      </c>
+      <c r="D36">
+        <v>113598.307758221</v>
+      </c>
+      <c r="E36">
+        <v>282179.67123287398</v>
+      </c>
+      <c r="F36">
+        <v>0.83333533297315499</v>
+      </c>
+      <c r="G36">
+        <v>21005.263452339499</v>
+      </c>
+      <c r="H36">
+        <v>9419.1929847336105</v>
+      </c>
+      <c r="I36">
+        <v>0</v>
+      </c>
+      <c r="J36">
+        <f>SUM(G36:I36)</f>
         <v>30424.45643707311</v>
       </c>
-      <c r="K33">
+      <c r="K36">
         <v>48819.627456497903</v>
       </c>
-      <c r="L33">
+      <c r="L36">
         <v>14784.690159207899</v>
       </c>
-      <c r="M33">
+      <c r="M36">
         <v>19569.533705442402</v>
       </c>
-      <c r="N33">
+      <c r="N36">
         <v>1040.9289460857101</v>
       </c>
-      <c r="O33">
-        <v>0</v>
-      </c>
-      <c r="P33">
-        <v>235150.29028510299</v>
-      </c>
-      <c r="Q33">
-        <v>1494.95371016114</v>
-      </c>
-      <c r="R33">
-        <v>40078.803663142098</v>
-      </c>
-      <c r="S33">
-        <v>910.88190143504903</v>
-      </c>
-      <c r="T33">
-        <v>0.51068072492979899</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A36" s="1" t="s">
+      <c r="O36">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.4"/>
+    <row r="39" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A39" s="1" t="s">
         <v>26</v>
       </c>
-    </row>
-    <row r="37" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A37" t="s">
-        <v>0</v>
-      </c>
-      <c r="B37" t="s">
+      <c r="P39" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q39" t="s">
+        <v>16</v>
+      </c>
+      <c r="R39" t="s">
+        <v>17</v>
+      </c>
+      <c r="S39" t="s">
+        <v>18</v>
+      </c>
+      <c r="T39" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="40" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A40" t="s">
+        <v>0</v>
+      </c>
+      <c r="B40" t="s">
         <v>1</v>
       </c>
-      <c r="C37" t="s">
+      <c r="C40" t="s">
         <v>2</v>
       </c>
-      <c r="D37" t="s">
+      <c r="D40" t="s">
         <v>3</v>
       </c>
-      <c r="E37" t="s">
+      <c r="E40" t="s">
         <v>4</v>
       </c>
-      <c r="F37" t="s">
+      <c r="F40" t="s">
         <v>5</v>
       </c>
-      <c r="G37" t="s">
+      <c r="G40" t="s">
         <v>6</v>
       </c>
-      <c r="H37" t="s">
+      <c r="H40" t="s">
         <v>7</v>
       </c>
-      <c r="I37" t="s">
+      <c r="I40" t="s">
         <v>8</v>
       </c>
-      <c r="J37" t="s">
+      <c r="J40" t="s">
         <v>9</v>
       </c>
-      <c r="K37" t="s">
+      <c r="K40" t="s">
         <v>10</v>
       </c>
-      <c r="L37" t="s">
+      <c r="L40" t="s">
         <v>11</v>
       </c>
-      <c r="M37" t="s">
+      <c r="M40" t="s">
         <v>12</v>
       </c>
-      <c r="N37" t="s">
+      <c r="N40" t="s">
         <v>13</v>
       </c>
-      <c r="O37" t="s">
+      <c r="O40" t="s">
         <v>14</v>
       </c>
-      <c r="P37" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q37" t="s">
-        <v>16</v>
-      </c>
-      <c r="R37" t="s">
-        <v>17</v>
-      </c>
-      <c r="S37" t="s">
-        <v>18</v>
-      </c>
-      <c r="T37" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A38" s="2" t="s">
+      <c r="P40">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q40">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R40">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S40">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T40">
+        <v>27.514184579999998</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A41" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B38" t="s">
+      <c r="B41" t="s">
         <v>21</v>
       </c>
-      <c r="C38">
+      <c r="C41">
         <v>4</v>
       </c>
-      <c r="D38">
+      <c r="D41">
         <v>29525.427309999999</v>
       </c>
-      <c r="E38">
+      <c r="E41">
         <v>80391.755990000005</v>
       </c>
-      <c r="F38">
+      <c r="F41">
         <v>0.79280104200000001</v>
       </c>
-      <c r="G38">
+      <c r="G41">
         <v>5050.6365619999997</v>
       </c>
-      <c r="H38">
+      <c r="H41">
         <v>4678.3390820000004</v>
       </c>
-      <c r="I38">
+      <c r="I41">
         <v>2508.6600360000002</v>
       </c>
-      <c r="J38">
+      <c r="J41">
         <v>12237.635679999999</v>
       </c>
-      <c r="K38">
+      <c r="K41">
         <v>13920</v>
       </c>
-      <c r="L38">
+      <c r="L41">
         <v>2841.544922</v>
       </c>
-      <c r="M38">
+      <c r="M41">
         <v>5380.5444360000001</v>
       </c>
-      <c r="N38">
+      <c r="N41">
         <v>279.27307350000001</v>
       </c>
-      <c r="O38">
-        <v>0</v>
-      </c>
-      <c r="P38">
-        <v>63734.6679</v>
-      </c>
-      <c r="Q38">
-        <v>1078.4492829999999</v>
-      </c>
-      <c r="R38">
-        <v>624.70352849999995</v>
-      </c>
-      <c r="S38">
-        <v>13.014656840000001</v>
-      </c>
-      <c r="T38">
-        <v>27.514184579999998</v>
-      </c>
-    </row>
-    <row r="39" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A39" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B39" t="s">
-        <v>21</v>
-      </c>
-      <c r="C39">
-        <v>4</v>
-      </c>
-      <c r="D39">
-        <v>30655.78772</v>
-      </c>
-      <c r="E39">
-        <v>79415.835619999998</v>
-      </c>
-      <c r="F39">
-        <v>0.81677700399999997</v>
-      </c>
-      <c r="G39">
-        <v>5129.9926729999997</v>
-      </c>
-      <c r="H39">
-        <v>5254.1641179999997</v>
-      </c>
-      <c r="I39">
-        <v>4834.2260249999999</v>
-      </c>
-      <c r="J39">
-        <v>15218.382820000001</v>
-      </c>
-      <c r="K39">
-        <v>13875.1543</v>
-      </c>
-      <c r="L39">
-        <v>3140.6678670000001</v>
-      </c>
-      <c r="M39">
-        <v>5340.9854210000003</v>
-      </c>
-      <c r="N39">
-        <v>286.5902719</v>
-      </c>
-      <c r="O39">
-        <v>0</v>
-      </c>
-      <c r="P39">
+      <c r="O41">
+        <v>0</v>
+      </c>
+      <c r="P41">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q39">
+      <c r="Q41">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R39">
+      <c r="R41">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S39">
+      <c r="S41">
         <v>452.7322633</v>
       </c>
-      <c r="T39">
+      <c r="T41">
         <v>5.8154128590000003</v>
       </c>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A42" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
defining a baseline flow_type with three trains on at steady state
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52A3E3C7-C3D9-4112-85AA-AACC7D8922DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{925D20A0-3156-44FB-965B-1164F5A14466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="68505" yWindow="8550" windowWidth="18000" windowHeight="15585" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -40,6 +40,7 @@
     <author>tc={9CE96C07-E110-41BE-B453-65310D0A2128}</author>
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
     <author>tc={44AB14B7-66C1-445B-8271-3F9869928B60}</author>
+    <author>tc={7EE5B16F-BA75-491F-B2FC-64121BCB8031}</author>
   </authors>
   <commentList>
     <comment ref="A19" authorId="0" shapeId="0" xr:uid="{059B2785-9A39-4C22-958C-B8BAB93BD95A}">
@@ -82,12 +83,20 @@
     The whole baseline for this might be corrupted</t>
       </text>
     </comment>
+    <comment ref="P35" authorId="5" shapeId="0" xr:uid="{7EE5B16F-BA75-491F-B2FC-64121BCB8031}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Idk which case these values go with</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="30">
   <si>
     <t>Season</t>
   </si>
@@ -177,9 +186,6 @@
   </si>
   <si>
     <t>Maximum Power</t>
-  </si>
-  <si>
-    <t>New, not sure feed and flow are different…</t>
   </si>
 </sst>
 </file>
@@ -1069,28 +1075,31 @@
   <threadedComment ref="T30" dT="2026-06-01T20:16:04.04" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{44AB14B7-66C1-445B-8271-3F9869928B60}">
     <text>The whole baseline for this might be corrupted</text>
   </threadedComment>
+  <threadedComment ref="P35" dT="2026-06-02T14:10:33.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7EE5B16F-BA75-491F-B2FC-64121BCB8031}">
+    <text>Idk which case these values go with</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:W42"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="3" max="3" width="12.4609375" customWidth="1"/>
-    <col min="5" max="5" width="10.23046875" customWidth="1"/>
-    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.23046875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.07421875" customWidth="1"/>
-    <col min="20" max="20" width="7.84375" customWidth="1"/>
+    <col min="3" max="3" width="12.453125" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.26953125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1152,7 +1161,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1214,7 +1223,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1276,7 +1285,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1338,7 +1347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -1400,7 +1409,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1462,7 +1471,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1524,7 +1533,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -1586,7 +1595,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>20</v>
       </c>
@@ -1648,7 +1657,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1704,7 +1713,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1760,7 +1769,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1816,7 +1825,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>22</v>
       </c>
@@ -1878,7 +1887,7 @@
         <v>0.79850332454920403</v>
       </c>
     </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -1934,7 +1943,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:23" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>22</v>
       </c>
@@ -1996,7 +2005,7 @@
         <v>1.75628458077399</v>
       </c>
     </row>
-    <row r="24" spans="1:23" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>20</v>
       </c>
@@ -2058,7 +2067,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:23" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>22</v>
       </c>
@@ -2120,12 +2129,12 @@
         <v>1.63318791126541</v>
       </c>
     </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -2187,7 +2196,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>20</v>
       </c>
@@ -2249,7 +2258,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:23" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>22</v>
       </c>
@@ -2311,7 +2320,7 @@
         <v>-4.8547669539218203</v>
       </c>
     </row>
-    <row r="31" spans="1:23" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:23" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>20</v>
       </c>
@@ -2382,7 +2391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>20</v>
       </c>
@@ -2393,35 +2402,34 @@
         <v>4</v>
       </c>
       <c r="D33">
-        <v>108960.613539453</v>
+        <v>116833.749486644</v>
       </c>
       <c r="E33">
-        <v>282179.67123287701</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F33">
-        <v>0.81690008021909599</v>
+        <v>0.84480122530439805</v>
       </c>
       <c r="G33">
-        <v>23571.632136721099</v>
+        <v>23535.478746437901</v>
       </c>
       <c r="H33">
-        <v>6951.9409028971204</v>
+        <v>6941.2778055266899</v>
       </c>
       <c r="I33">
-        <v>913.88179307768496</v>
+        <v>912.48005352310201</v>
       </c>
       <c r="J33">
-        <f>SUM(G33:I33)</f>
-        <v>31437.454832695905</v>
+        <v>31389.236605487698</v>
       </c>
       <c r="K33">
-        <v>48809.460212750702</v>
+        <v>50843.184005923998</v>
       </c>
       <c r="L33">
-        <v>9838.1656916422507</v>
+        <v>15303.798385784499</v>
       </c>
       <c r="M33">
-        <v>18875.532802364902</v>
+        <v>19297.5304894484</v>
       </c>
       <c r="N33">
         <v>992.31070788530405</v>
@@ -2429,64 +2437,11 @@
       <c r="O33">
         <v>0</v>
       </c>
-      <c r="P33">
-        <v>238385.73201352599</v>
-      </c>
-      <c r="Q33">
-        <v>1101.67495873487</v>
-      </c>
-      <c r="R33">
-        <v>0</v>
-      </c>
-      <c r="S33">
-        <v>0</v>
-      </c>
-      <c r="T33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A34" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="D34">
-        <v>116833.749486644</v>
-      </c>
-      <c r="E34">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F34">
-        <v>0.84480122530439805</v>
-      </c>
-      <c r="G34">
-        <v>23535.478746437901</v>
-      </c>
-      <c r="H34">
-        <v>6941.2778055266899</v>
-      </c>
-      <c r="I34">
-        <v>912.48005352310201</v>
-      </c>
-      <c r="J34">
-        <v>31389.236605487698</v>
-      </c>
-      <c r="K34">
-        <v>50843.184005923998</v>
-      </c>
-      <c r="L34">
-        <v>15303.798385784499</v>
-      </c>
-      <c r="M34">
-        <v>19297.5304894484</v>
-      </c>
-      <c r="N34">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.4">
+    </row>
+    <row r="34" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A34" s="2"/>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A35" s="2"/>
       <c r="P35">
         <v>235150.29028510299</v>
@@ -2504,7 +2459,7 @@
         <v>0.51068072492979899</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>22</v>
       </c>
@@ -2552,8 +2507,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.4"/>
-    <row r="39" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="39" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="1" t="s">
         <v>26</v>
       </c>
@@ -2573,7 +2528,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="40" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>0</v>
       </c>
@@ -2635,7 +2590,7 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="41" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>20</v>
       </c>
@@ -2697,7 +2652,7 @@
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A42" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
running with recovery change with fast script
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{925D20A0-3156-44FB-965B-1164F5A14466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FC9F4BC7-E19E-4A12-BA8A-BD09F0B8E2B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="28695" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -41,6 +41,7 @@
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
     <author>tc={44AB14B7-66C1-445B-8271-3F9869928B60}</author>
     <author>tc={7EE5B16F-BA75-491F-B2FC-64121BCB8031}</author>
+    <author>tc={7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}</author>
   </authors>
   <commentList>
     <comment ref="A19" authorId="0" shapeId="0" xr:uid="{059B2785-9A39-4C22-958C-B8BAB93BD95A}">
@@ -83,7 +84,7 @@
     The whole baseline for this might be corrupted</t>
       </text>
     </comment>
-    <comment ref="P35" authorId="5" shapeId="0" xr:uid="{7EE5B16F-BA75-491F-B2FC-64121BCB8031}">
+    <comment ref="P34" authorId="5" shapeId="0" xr:uid="{7EE5B16F-BA75-491F-B2FC-64121BCB8031}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -91,12 +92,20 @@
     Idk which case these values go with</t>
       </text>
     </comment>
+    <comment ref="A36" authorId="6" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Result from the fast solve</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="31">
   <si>
     <t>Season</t>
   </si>
@@ -186,6 +195,9 @@
   </si>
   <si>
     <t>Maximum Power</t>
+  </si>
+  <si>
+    <t>Simple DR</t>
   </si>
 </sst>
 </file>
@@ -328,10 +340,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="33">
@@ -675,10 +687,11 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1075,15 +1088,18 @@
   <threadedComment ref="T30" dT="2026-06-01T20:16:04.04" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{44AB14B7-66C1-445B-8271-3F9869928B60}">
     <text>The whole baseline for this might be corrupted</text>
   </threadedComment>
-  <threadedComment ref="P35" dT="2026-06-02T14:10:33.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7EE5B16F-BA75-491F-B2FC-64121BCB8031}">
+  <threadedComment ref="P34" dT="2026-06-02T14:10:33.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7EE5B16F-BA75-491F-B2FC-64121BCB8031}">
     <text>Idk which case these values go with</text>
+  </threadedComment>
+  <threadedComment ref="A36" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <text>Result from the fast solve</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:W42"/>
+  <dimension ref="A1:W44"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="3" max="3" width="12.453125" customWidth="1"/>
@@ -2392,7 +2408,7 @@
       </c>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A33" s="2" t="s">
+      <c r="A33" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B33" t="s">
@@ -2440,27 +2456,72 @@
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A34" s="2"/>
+      <c r="P34">
+        <v>235150.29028510299</v>
+      </c>
+      <c r="Q34">
+        <v>1494.95371016114</v>
+      </c>
+      <c r="R34">
+        <v>40078.803663142098</v>
+      </c>
+      <c r="S34">
+        <v>910.88190143504903</v>
+      </c>
+      <c r="T34">
+        <v>0.51068072492979899</v>
+      </c>
     </row>
     <row r="35" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A35" s="2"/>
-      <c r="P35">
-        <v>235150.29028510299</v>
-      </c>
-      <c r="Q35">
-        <v>1494.95371016114</v>
-      </c>
-      <c r="R35">
-        <v>40078.803663142098</v>
-      </c>
-      <c r="S35">
-        <v>910.88190143504903</v>
-      </c>
-      <c r="T35">
-        <v>0.51068072492979899</v>
+      <c r="A35" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B35" t="s">
+        <v>21</v>
+      </c>
+      <c r="C35">
+        <v>4</v>
+      </c>
+      <c r="D35">
+        <v>113598.307758221</v>
+      </c>
+      <c r="E35">
+        <v>282179.67123287398</v>
+      </c>
+      <c r="F35">
+        <v>0.83333533297315499</v>
+      </c>
+      <c r="G35">
+        <v>21005.263452339499</v>
+      </c>
+      <c r="H35">
+        <v>9419.1929847336105</v>
+      </c>
+      <c r="I35">
+        <v>0</v>
+      </c>
+      <c r="J35">
+        <f>SUM(G35:I35)</f>
+        <v>30424.45643707311</v>
+      </c>
+      <c r="K35">
+        <v>48819.627456497903</v>
+      </c>
+      <c r="L35">
+        <v>14784.690159207899</v>
+      </c>
+      <c r="M35">
+        <v>19569.533705442402</v>
+      </c>
+      <c r="N35">
+        <v>1040.9289460857101</v>
+      </c>
+      <c r="O35">
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A36" s="2" t="s">
+      <c r="A36" t="s">
         <v>22</v>
       </c>
       <c r="B36" t="s">
@@ -2470,190 +2531,333 @@
         <v>4</v>
       </c>
       <c r="D36">
-        <v>113598.307758221</v>
+        <v>108493.492202382</v>
       </c>
       <c r="E36">
-        <v>282179.67123287398</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F36">
-        <v>0.83333533297315499</v>
+        <v>0.81524467628787201</v>
       </c>
       <c r="G36">
-        <v>21005.263452339499</v>
+        <v>19433.390629510399</v>
       </c>
       <c r="H36">
-        <v>9419.1929847336105</v>
+        <v>5222.6561863913303</v>
       </c>
       <c r="I36">
-        <v>0</v>
+        <v>4899.46807259245</v>
       </c>
       <c r="J36">
-        <f>SUM(G36:I36)</f>
-        <v>30424.45643707311</v>
+        <v>29555.514888494199</v>
       </c>
       <c r="K36">
-        <v>48819.627456497903</v>
+        <v>49172.699906497</v>
       </c>
       <c r="L36">
-        <v>14784.690159207899</v>
+        <v>10814.372368574401</v>
       </c>
       <c r="M36">
-        <v>19569.533705442402</v>
+        <v>18950.9050388172</v>
       </c>
       <c r="N36">
-        <v>1040.9289460857101</v>
+        <v>1008.6177006503</v>
       </c>
       <c r="O36">
         <v>0</v>
       </c>
-    </row>
-    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.35"/>
+      <c r="P36">
+        <v>230045.47472926401</v>
+      </c>
+      <c r="Q36">
+        <v>1166.87072431198</v>
+      </c>
+      <c r="R36">
+        <v>13047.3855631853</v>
+      </c>
+      <c r="S36">
+        <v>465.97805582804898</v>
+      </c>
+      <c r="T36">
+        <v>1.6328254200035199</v>
+      </c>
+    </row>
+    <row r="37" spans="1:20" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="38" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+      <c r="A38" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="P38" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q38" t="s">
+        <v>16</v>
+      </c>
+      <c r="R38" t="s">
+        <v>17</v>
+      </c>
+      <c r="S38" t="s">
+        <v>18</v>
+      </c>
+      <c r="T38" t="s">
+        <v>19</v>
+      </c>
+    </row>
     <row r="39" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A39" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="P39" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q39" t="s">
-        <v>16</v>
-      </c>
-      <c r="R39" t="s">
-        <v>17</v>
-      </c>
-      <c r="S39" t="s">
-        <v>18</v>
-      </c>
-      <c r="T39" t="s">
-        <v>19</v>
+      <c r="A39" t="s">
+        <v>0</v>
+      </c>
+      <c r="B39" t="s">
+        <v>1</v>
+      </c>
+      <c r="C39" t="s">
+        <v>2</v>
+      </c>
+      <c r="D39" t="s">
+        <v>3</v>
+      </c>
+      <c r="E39" t="s">
+        <v>4</v>
+      </c>
+      <c r="F39" t="s">
+        <v>5</v>
+      </c>
+      <c r="G39" t="s">
+        <v>6</v>
+      </c>
+      <c r="H39" t="s">
+        <v>7</v>
+      </c>
+      <c r="I39" t="s">
+        <v>8</v>
+      </c>
+      <c r="J39" t="s">
+        <v>9</v>
+      </c>
+      <c r="K39" t="s">
+        <v>10</v>
+      </c>
+      <c r="L39" t="s">
+        <v>11</v>
+      </c>
+      <c r="M39" t="s">
+        <v>12</v>
+      </c>
+      <c r="N39" t="s">
+        <v>13</v>
+      </c>
+      <c r="O39" t="s">
+        <v>14</v>
+      </c>
+      <c r="P39">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q39">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R39">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S39">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T39">
+        <v>27.514184579999998</v>
       </c>
     </row>
     <row r="40" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A40" t="s">
-        <v>0</v>
+      <c r="A40" s="2" t="s">
+        <v>20</v>
       </c>
       <c r="B40" t="s">
-        <v>1</v>
-      </c>
-      <c r="C40" t="s">
+        <v>21</v>
+      </c>
+      <c r="C40">
+        <v>4</v>
+      </c>
+      <c r="D40">
+        <v>29525.427309999999</v>
+      </c>
+      <c r="E40">
+        <v>80391.755990000005</v>
+      </c>
+      <c r="F40">
+        <v>0.79280104200000001</v>
+      </c>
+      <c r="G40">
+        <v>5050.6365619999997</v>
+      </c>
+      <c r="H40">
+        <v>4678.3390820000004</v>
+      </c>
+      <c r="I40">
+        <v>2508.6600360000002</v>
+      </c>
+      <c r="J40">
+        <v>12237.635679999999</v>
+      </c>
+      <c r="K40">
+        <v>13920</v>
+      </c>
+      <c r="L40">
+        <v>2841.544922</v>
+      </c>
+      <c r="M40">
+        <v>5380.5444360000001</v>
+      </c>
+      <c r="N40">
+        <v>279.27307350000001</v>
+      </c>
+      <c r="O40">
+        <v>0</v>
+      </c>
+      <c r="P40">
+        <v>64865.028310000002</v>
+      </c>
+      <c r="Q40">
+        <v>1191.7509680000001</v>
+      </c>
+      <c r="R40">
+        <v>7243.7162129999997</v>
+      </c>
+      <c r="S40">
+        <v>452.7322633</v>
+      </c>
+      <c r="T40">
+        <v>5.8154128590000003</v>
+      </c>
+    </row>
+    <row r="41" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A41" s="2"/>
+    </row>
+    <row r="42" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A42" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A43" t="s">
+        <v>22</v>
+      </c>
+      <c r="B43" t="s">
+        <v>25</v>
+      </c>
+      <c r="C43">
         <v>2</v>
       </c>
-      <c r="D40" t="s">
-        <v>3</v>
-      </c>
-      <c r="E40" t="s">
+      <c r="D43">
+        <v>115472.147206908</v>
+      </c>
+      <c r="E43">
+        <v>282495</v>
+      </c>
+      <c r="F43">
+        <v>0.83903831831993503</v>
+      </c>
+      <c r="G43">
+        <v>20221.889710343999</v>
+      </c>
+      <c r="H43">
+        <v>6553.7440767980397</v>
+      </c>
+      <c r="I43">
+        <v>6160.4249909476703</v>
+      </c>
+      <c r="J43">
+        <v>32936.058778089697</v>
+      </c>
+      <c r="K43">
+        <v>50939.5611113743</v>
+      </c>
+      <c r="L43">
+        <v>15427.2204868183</v>
+      </c>
+      <c r="M43">
+        <v>19327.3039306102</v>
+      </c>
+      <c r="N43">
+        <v>1004.9477757237401</v>
+      </c>
+      <c r="O43">
+        <v>3157.9970999842499</v>
+      </c>
+      <c r="P43">
+        <v>237024.12973379</v>
+      </c>
+      <c r="Q43">
+        <v>1464.2687322859999</v>
+      </c>
+      <c r="R43">
+        <v>8672.9882445954008</v>
+      </c>
+      <c r="S43">
+        <v>346.91952978381602</v>
+      </c>
+      <c r="T43">
+        <v>2.4302910949698302</v>
+      </c>
+    </row>
+    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>22</v>
+      </c>
+      <c r="B44" t="s">
+        <v>25</v>
+      </c>
+      <c r="C44">
         <v>4</v>
       </c>
-      <c r="F40" t="s">
-        <v>5</v>
-      </c>
-      <c r="G40" t="s">
-        <v>6</v>
-      </c>
-      <c r="H40" t="s">
-        <v>7</v>
-      </c>
-      <c r="I40" t="s">
-        <v>8</v>
-      </c>
-      <c r="J40" t="s">
-        <v>9</v>
-      </c>
-      <c r="K40" t="s">
-        <v>10</v>
-      </c>
-      <c r="L40" t="s">
-        <v>11</v>
-      </c>
-      <c r="M40" t="s">
-        <v>12</v>
-      </c>
-      <c r="N40" t="s">
-        <v>13</v>
-      </c>
-      <c r="O40" t="s">
-        <v>14</v>
-      </c>
-      <c r="P40">
-        <v>63734.6679</v>
-      </c>
-      <c r="Q40">
-        <v>1078.4492829999999</v>
-      </c>
-      <c r="R40">
-        <v>624.70352849999995</v>
-      </c>
-      <c r="S40">
-        <v>13.014656840000001</v>
-      </c>
-      <c r="T40">
-        <v>27.514184579999998</v>
-      </c>
-    </row>
-    <row r="41" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
-      <c r="A41" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B41" t="s">
-        <v>21</v>
-      </c>
-      <c r="C41">
-        <v>4</v>
-      </c>
-      <c r="D41">
-        <v>29525.427309999999</v>
-      </c>
-      <c r="E41">
-        <v>80391.755990000005</v>
-      </c>
-      <c r="F41">
-        <v>0.79280104200000001</v>
-      </c>
-      <c r="G41">
-        <v>5050.6365619999997</v>
-      </c>
-      <c r="H41">
-        <v>4678.3390820000004</v>
-      </c>
-      <c r="I41">
-        <v>2508.6600360000002</v>
-      </c>
-      <c r="J41">
-        <v>12237.635679999999</v>
-      </c>
-      <c r="K41">
-        <v>13920</v>
-      </c>
-      <c r="L41">
-        <v>2841.544922</v>
-      </c>
-      <c r="M41">
-        <v>5380.5444360000001</v>
-      </c>
-      <c r="N41">
-        <v>279.27307350000001</v>
-      </c>
-      <c r="O41">
-        <v>0</v>
-      </c>
-      <c r="P41">
-        <v>64865.028310000002</v>
-      </c>
-      <c r="Q41">
-        <v>1191.7509680000001</v>
-      </c>
-      <c r="R41">
-        <v>7243.7162129999997</v>
-      </c>
-      <c r="S41">
-        <v>452.7322633</v>
-      </c>
-      <c r="T41">
-        <v>5.8154128590000003</v>
-      </c>
-    </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A42" s="2"/>
+      <c r="D44">
+        <v>108958.027502652</v>
+      </c>
+      <c r="E44">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F44">
+        <v>0.81689091571482797</v>
+      </c>
+      <c r="G44">
+        <v>20285.098342207999</v>
+      </c>
+      <c r="H44">
+        <v>6552.6722224723899</v>
+      </c>
+      <c r="I44">
+        <v>6068.9240568166097</v>
+      </c>
+      <c r="J44">
+        <v>32906.694621497001</v>
+      </c>
+      <c r="K44">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="L44">
+        <v>16378.7983857829</v>
+      </c>
+      <c r="M44">
+        <v>19449.350489448301</v>
+      </c>
+      <c r="N44">
+        <v>1004.9477757237401</v>
+      </c>
+      <c r="O44">
+        <v>10620</v>
+      </c>
+      <c r="P44">
+        <v>230510.010029533</v>
+      </c>
+      <c r="Q44">
+        <v>1464.02925348484</v>
+      </c>
+      <c r="R44">
+        <v>26064.489084194902</v>
+      </c>
+      <c r="S44">
+        <v>407.257641940545</v>
+      </c>
+      <c r="T44">
+        <v>1.09609872121186</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Redo 2 trains w/ TOU 8
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21C63577-EE39-4007-A62E-9DA6AC8354C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69EAC33E-64CC-47E7-A221-3F702E7D312E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="9740" yWindow="0" windowWidth="9550" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -96,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="32">
   <si>
     <t>Season</t>
   </si>
@@ -189,6 +189,9 @@
   </si>
   <si>
     <t>Simple DR</t>
+  </si>
+  <si>
+    <t>TOU 8</t>
   </si>
 </sst>
 </file>
@@ -1088,7 +1091,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:W44"/>
+  <dimension ref="A1:W49"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.6328125" customWidth="1"/>
@@ -2033,7 +2036,7 @@
       <c r="G23" s="4"/>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A24" s="2" t="s">
+      <c r="A24" s="3" t="s">
         <v>20</v>
       </c>
       <c r="B24" t="s">
@@ -2095,7 +2098,7 @@
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="3" t="s">
         <v>22</v>
       </c>
       <c r="B25" t="s">
@@ -2166,7 +2169,7 @@
       <c r="G27" s="4"/>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A28" t="s">
+      <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B28" t="s">
@@ -2228,7 +2231,7 @@
       </c>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A29" t="s">
+      <c r="A29" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B29" t="s">
@@ -2680,155 +2683,345 @@
       </c>
     </row>
     <row r="40" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="G40" s="4"/>
+      <c r="A40" s="1" t="s">
+        <v>31</v>
+      </c>
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A41" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G41" s="4"/>
-      <c r="P41" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q41" t="s">
-        <v>16</v>
-      </c>
-      <c r="R41" t="s">
-        <v>17</v>
-      </c>
-      <c r="S41" t="s">
-        <v>18</v>
-      </c>
-      <c r="T41" t="s">
-        <v>19</v>
+      <c r="A41" t="s">
+        <v>20</v>
+      </c>
+      <c r="B41" t="s">
+        <v>21</v>
+      </c>
+      <c r="C41">
+        <v>2</v>
+      </c>
+      <c r="D41">
+        <v>115714.10508262301</v>
+      </c>
+      <c r="E41">
+        <v>282179.67125387199</v>
+      </c>
+      <c r="F41">
+        <v>0.840833383054163</v>
+      </c>
+      <c r="G41">
+        <v>20578.507216446698</v>
+      </c>
+      <c r="H41">
+        <v>7102.57515066207</v>
+      </c>
+      <c r="I41">
+        <v>2588.5052959285099</v>
+      </c>
+      <c r="J41">
+        <v>30269.587663037299</v>
+      </c>
+      <c r="K41">
+        <v>50843.185173268597</v>
+      </c>
+      <c r="L41">
+        <v>15303.8015139941</v>
+      </c>
+      <c r="M41">
+        <v>19297.530732323401</v>
+      </c>
+      <c r="N41">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O41">
+        <v>0</v>
+      </c>
+      <c r="P41">
+        <v>237266.08760950499</v>
+      </c>
+      <c r="Q41">
+        <v>1127.2750356983099</v>
+      </c>
+      <c r="R41">
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="B42" t="s">
-        <v>1</v>
-      </c>
-      <c r="C42" t="s">
-        <v>2</v>
-      </c>
-      <c r="D42" t="s">
-        <v>3</v>
-      </c>
-      <c r="E42" t="s">
+        <v>21</v>
+      </c>
+      <c r="C42">
         <v>4</v>
       </c>
-      <c r="F42" t="s">
-        <v>5</v>
-      </c>
-      <c r="G42" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H42" t="s">
-        <v>7</v>
-      </c>
-      <c r="I42" t="s">
-        <v>8</v>
-      </c>
-      <c r="J42" t="s">
-        <v>9</v>
-      </c>
-      <c r="K42" t="s">
-        <v>10</v>
-      </c>
-      <c r="L42" t="s">
-        <v>11</v>
-      </c>
-      <c r="M42" t="s">
-        <v>12</v>
-      </c>
-      <c r="N42" t="s">
-        <v>13</v>
-      </c>
-      <c r="O42" t="s">
-        <v>14</v>
+      <c r="D42">
+        <v>115714.10508261999</v>
+      </c>
+      <c r="E42">
+        <v>282179.671253876</v>
+      </c>
+      <c r="F42">
+        <v>0.84083338305413902</v>
+      </c>
+      <c r="G42">
+        <v>20578.5072164468</v>
+      </c>
+      <c r="H42">
+        <v>7102.5751506616798</v>
+      </c>
+      <c r="I42">
+        <v>2588.50529592865</v>
+      </c>
+      <c r="J42">
+        <v>30269.587663037099</v>
+      </c>
+      <c r="K42">
+        <v>50843.185173268197</v>
+      </c>
+      <c r="L42">
+        <v>15303.8015139912</v>
+      </c>
+      <c r="M42">
+        <v>19297.530732323299</v>
+      </c>
+      <c r="N42">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O42">
+        <v>0</v>
       </c>
       <c r="P42">
-        <v>63734.6679</v>
+        <v>237266.087609501</v>
       </c>
       <c r="Q42">
-        <v>1078.4492829999999</v>
+        <v>1127.2750356983499</v>
       </c>
       <c r="R42">
-        <v>624.70352849999995</v>
-      </c>
-      <c r="S42">
-        <v>13.014656840000001</v>
-      </c>
-      <c r="T42">
-        <v>27.514184579999998</v>
+        <v>0</v>
       </c>
     </row>
     <row r="43" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A43" s="2" t="s">
-        <v>20</v>
+      <c r="A43" t="s">
+        <v>22</v>
       </c>
       <c r="B43" t="s">
         <v>21</v>
       </c>
       <c r="C43">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A44" t="s">
+        <v>22</v>
+      </c>
+      <c r="B44" t="s">
+        <v>21</v>
+      </c>
+      <c r="C44">
         <v>4</v>
       </c>
-      <c r="D43">
+      <c r="D44">
+        <v>120375.156660901</v>
+      </c>
+      <c r="E44">
+        <v>282179.671232878</v>
+      </c>
+      <c r="F44">
+        <v>0.857351410648304</v>
+      </c>
+      <c r="G44">
+        <v>21285.1004075495</v>
+      </c>
+      <c r="H44">
+        <v>7426.32532798384</v>
+      </c>
+      <c r="I44">
+        <v>5046.79446201879</v>
+      </c>
+      <c r="J44">
+        <v>33758.220197552102</v>
+      </c>
+      <c r="K44">
+        <v>51144.191344099498</v>
+      </c>
+      <c r="L44">
+        <v>16112.7556071296</v>
+      </c>
+      <c r="M44">
+        <v>19359.989512119799</v>
+      </c>
+      <c r="N44">
+        <v>1006.77939378399</v>
+      </c>
+      <c r="O44">
+        <v>0</v>
+      </c>
+      <c r="P44">
+        <v>241927.13918778201</v>
+      </c>
+      <c r="Q44">
+        <v>1178.65858109644</v>
+      </c>
+      <c r="R44">
+        <v>12586.325853030899</v>
+      </c>
+      <c r="S44">
+        <v>466.16021677892502</v>
+      </c>
+      <c r="T44">
+        <v>1.3585822738026401</v>
+      </c>
+    </row>
+    <row r="45" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="G45" s="4"/>
+    </row>
+    <row r="46" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A46" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G46" s="4"/>
+      <c r="P46" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q46" t="s">
+        <v>16</v>
+      </c>
+      <c r="R46" t="s">
+        <v>17</v>
+      </c>
+      <c r="S46" t="s">
+        <v>18</v>
+      </c>
+      <c r="T46" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A47" t="s">
+        <v>0</v>
+      </c>
+      <c r="B47" t="s">
+        <v>1</v>
+      </c>
+      <c r="C47" t="s">
+        <v>2</v>
+      </c>
+      <c r="D47" t="s">
+        <v>3</v>
+      </c>
+      <c r="E47" t="s">
+        <v>4</v>
+      </c>
+      <c r="F47" t="s">
+        <v>5</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H47" t="s">
+        <v>7</v>
+      </c>
+      <c r="I47" t="s">
+        <v>8</v>
+      </c>
+      <c r="J47" t="s">
+        <v>9</v>
+      </c>
+      <c r="K47" t="s">
+        <v>10</v>
+      </c>
+      <c r="L47" t="s">
+        <v>11</v>
+      </c>
+      <c r="M47" t="s">
+        <v>12</v>
+      </c>
+      <c r="N47" t="s">
+        <v>13</v>
+      </c>
+      <c r="O47" t="s">
+        <v>14</v>
+      </c>
+      <c r="P47">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q47">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R47">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S47">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T47">
+        <v>27.514184579999998</v>
+      </c>
+    </row>
+    <row r="48" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A48" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B48" t="s">
+        <v>21</v>
+      </c>
+      <c r="C48">
+        <v>4</v>
+      </c>
+      <c r="D48">
         <v>29525.427309999999</v>
       </c>
-      <c r="E43">
+      <c r="E48">
         <v>80391.755990000005</v>
       </c>
-      <c r="F43">
+      <c r="F48">
         <v>0.79280104200000001</v>
       </c>
-      <c r="G43" s="4">
+      <c r="G48" s="4">
         <v>5050.6365619999997</v>
       </c>
-      <c r="H43">
+      <c r="H48">
         <v>4678.3390820000004</v>
       </c>
-      <c r="I43">
+      <c r="I48">
         <v>2508.6600360000002</v>
       </c>
-      <c r="J43">
+      <c r="J48">
         <v>12237.635679999999</v>
       </c>
-      <c r="K43">
+      <c r="K48">
         <v>13920</v>
       </c>
-      <c r="L43">
+      <c r="L48">
         <v>2841.544922</v>
       </c>
-      <c r="M43">
+      <c r="M48">
         <v>5380.5444360000001</v>
       </c>
-      <c r="N43">
+      <c r="N48">
         <v>279.27307350000001</v>
       </c>
-      <c r="O43">
-        <v>0</v>
-      </c>
-      <c r="P43">
+      <c r="O48">
+        <v>0</v>
+      </c>
+      <c r="P48">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q43">
+      <c r="Q48">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R43">
+      <c r="R48">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S43">
+      <c r="S48">
         <v>452.7322633</v>
       </c>
-      <c r="T43">
+      <c r="T48">
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A44" s="2"/>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
+      <c r="A49" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Ipopt results for a summer and winter week
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69EAC33E-64CC-47E7-A221-3F702E7D312E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7682F503-1E77-4599-87A9-53F403D37CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9740" yWindow="0" windowWidth="9550" windowHeight="10170" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="-19310" yWindow="10680" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1091,7 +1092,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:W49"/>
+  <dimension ref="A1:W50"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.6328125" customWidth="1"/>
@@ -2745,74 +2746,69 @@
     </row>
     <row r="42" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B42" t="s">
         <v>21</v>
       </c>
       <c r="C42">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D42">
-        <v>115714.10508261999</v>
+        <v>120628.41082793</v>
       </c>
       <c r="E42">
-        <v>282179.671253876</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F42">
-        <v>0.84083338305413902</v>
+        <v>0.85824890324911396</v>
       </c>
       <c r="G42">
-        <v>20578.5072164468</v>
+        <v>20824.7129679639</v>
       </c>
       <c r="H42">
-        <v>7102.5751506616798</v>
+        <v>7456.39074483072</v>
       </c>
       <c r="I42">
-        <v>2588.50529592865</v>
+        <v>5114.4587365303096</v>
       </c>
       <c r="J42">
-        <v>30269.587663037099</v>
+        <v>33395.562449324898</v>
       </c>
       <c r="K42">
-        <v>50843.185173268197</v>
+        <v>51302.320205525801</v>
       </c>
       <c r="L42">
-        <v>15303.8015139912</v>
+        <v>16537.7269222135</v>
       </c>
       <c r="M42">
-        <v>19297.530732323299</v>
+        <v>19392.801250865799</v>
       </c>
       <c r="N42">
-        <v>992.31070788530405</v>
+        <v>1004.9477757237401</v>
       </c>
       <c r="O42">
         <v>0</v>
       </c>
       <c r="P42">
-        <v>237266.087609501</v>
+        <v>242180.39335481101</v>
       </c>
       <c r="Q42">
-        <v>1127.2750356983499</v>
+        <v>1183.4303612998101</v>
       </c>
       <c r="R42">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A43" t="s">
-        <v>22</v>
-      </c>
-      <c r="B43" t="s">
-        <v>21</v>
-      </c>
-      <c r="C43">
-        <v>2</v>
+        <v>15931.1957490451</v>
+      </c>
+      <c r="S42">
+        <v>346.33034237054602</v>
+      </c>
+      <c r="T42">
+        <v>1.0959871186973</v>
       </c>
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B44" t="s">
         <v>21</v>
@@ -2821,207 +2817,263 @@
         <v>4</v>
       </c>
       <c r="D44">
+        <v>115714.10508261999</v>
+      </c>
+      <c r="E44">
+        <v>282179.671253876</v>
+      </c>
+      <c r="F44">
+        <v>0.84083338305413902</v>
+      </c>
+      <c r="G44">
+        <v>20578.5072164468</v>
+      </c>
+      <c r="H44">
+        <v>7102.5751506616798</v>
+      </c>
+      <c r="I44">
+        <v>2588.50529592865</v>
+      </c>
+      <c r="J44">
+        <v>30269.587663037099</v>
+      </c>
+      <c r="K44">
+        <v>50843.185173268197</v>
+      </c>
+      <c r="L44">
+        <v>15303.8015139912</v>
+      </c>
+      <c r="M44">
+        <v>19297.530732323299</v>
+      </c>
+      <c r="N44">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O44">
+        <v>0</v>
+      </c>
+      <c r="P44">
+        <v>237266.087609501</v>
+      </c>
+      <c r="Q44">
+        <v>1127.2750356983499</v>
+      </c>
+      <c r="R44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A45" t="s">
+        <v>22</v>
+      </c>
+      <c r="B45" t="s">
+        <v>21</v>
+      </c>
+      <c r="C45">
+        <v>4</v>
+      </c>
+      <c r="D45">
         <v>120375.156660901</v>
       </c>
-      <c r="E44">
+      <c r="E45">
         <v>282179.671232878</v>
       </c>
-      <c r="F44">
+      <c r="F45">
         <v>0.857351410648304</v>
       </c>
-      <c r="G44">
+      <c r="G45">
         <v>21285.1004075495</v>
       </c>
-      <c r="H44">
+      <c r="H45">
         <v>7426.32532798384</v>
       </c>
-      <c r="I44">
+      <c r="I45">
         <v>5046.79446201879</v>
       </c>
-      <c r="J44">
+      <c r="J45">
         <v>33758.220197552102</v>
       </c>
-      <c r="K44">
+      <c r="K45">
         <v>51144.191344099498</v>
       </c>
-      <c r="L44">
+      <c r="L45">
         <v>16112.7556071296</v>
       </c>
-      <c r="M44">
+      <c r="M45">
         <v>19359.989512119799</v>
       </c>
-      <c r="N44">
+      <c r="N45">
         <v>1006.77939378399</v>
       </c>
-      <c r="O44">
-        <v>0</v>
-      </c>
-      <c r="P44">
+      <c r="O45">
+        <v>0</v>
+      </c>
+      <c r="P45">
         <v>241927.13918778201</v>
       </c>
-      <c r="Q44">
+      <c r="Q45">
         <v>1178.65858109644</v>
       </c>
-      <c r="R44">
+      <c r="R45">
         <v>12586.325853030899</v>
       </c>
-      <c r="S44">
+      <c r="S45">
         <v>466.16021677892502</v>
       </c>
-      <c r="T44">
+      <c r="T45">
         <v>1.3585822738026401</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="G45" s="4"/>
-    </row>
     <row r="46" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A46" s="1" t="s">
+      <c r="G46" s="4"/>
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A47" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="G46" s="4"/>
-      <c r="P46" t="s">
+      <c r="G47" s="4"/>
+      <c r="P47" t="s">
         <v>15</v>
       </c>
-      <c r="Q46" t="s">
+      <c r="Q47" t="s">
         <v>16</v>
       </c>
-      <c r="R46" t="s">
+      <c r="R47" t="s">
         <v>17</v>
       </c>
-      <c r="S46" t="s">
+      <c r="S47" t="s">
         <v>18</v>
       </c>
-      <c r="T46" t="s">
+      <c r="T47" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A47" t="s">
-        <v>0</v>
-      </c>
-      <c r="B47" t="s">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A48" t="s">
+        <v>0</v>
+      </c>
+      <c r="B48" t="s">
         <v>1</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C48" t="s">
         <v>2</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D48" t="s">
         <v>3</v>
       </c>
-      <c r="E47" t="s">
+      <c r="E48" t="s">
         <v>4</v>
       </c>
-      <c r="F47" t="s">
+      <c r="F48" t="s">
         <v>5</v>
       </c>
-      <c r="G47" s="4" t="s">
+      <c r="G48" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="H47" t="s">
+      <c r="H48" t="s">
         <v>7</v>
       </c>
-      <c r="I47" t="s">
+      <c r="I48" t="s">
         <v>8</v>
       </c>
-      <c r="J47" t="s">
+      <c r="J48" t="s">
         <v>9</v>
       </c>
-      <c r="K47" t="s">
+      <c r="K48" t="s">
         <v>10</v>
       </c>
-      <c r="L47" t="s">
+      <c r="L48" t="s">
         <v>11</v>
       </c>
-      <c r="M47" t="s">
+      <c r="M48" t="s">
         <v>12</v>
       </c>
-      <c r="N47" t="s">
+      <c r="N48" t="s">
         <v>13</v>
       </c>
-      <c r="O47" t="s">
+      <c r="O48" t="s">
         <v>14</v>
       </c>
-      <c r="P47">
+      <c r="P48">
         <v>63734.6679</v>
       </c>
-      <c r="Q47">
+      <c r="Q48">
         <v>1078.4492829999999</v>
       </c>
-      <c r="R47">
+      <c r="R48">
         <v>624.70352849999995</v>
       </c>
-      <c r="S47">
+      <c r="S48">
         <v>13.014656840000001</v>
       </c>
-      <c r="T47">
+      <c r="T48">
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.35">
-      <c r="A48" s="2" t="s">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A49" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B49" t="s">
         <v>21</v>
       </c>
-      <c r="C48">
+      <c r="C49">
         <v>4</v>
       </c>
-      <c r="D48">
+      <c r="D49">
         <v>29525.427309999999</v>
       </c>
-      <c r="E48">
+      <c r="E49">
         <v>80391.755990000005</v>
       </c>
-      <c r="F48">
+      <c r="F49">
         <v>0.79280104200000001</v>
       </c>
-      <c r="G48" s="4">
+      <c r="G49" s="4">
         <v>5050.6365619999997</v>
       </c>
-      <c r="H48">
+      <c r="H49">
         <v>4678.3390820000004</v>
       </c>
-      <c r="I48">
+      <c r="I49">
         <v>2508.6600360000002</v>
       </c>
-      <c r="J48">
+      <c r="J49">
         <v>12237.635679999999</v>
       </c>
-      <c r="K48">
+      <c r="K49">
         <v>13920</v>
       </c>
-      <c r="L48">
+      <c r="L49">
         <v>2841.544922</v>
       </c>
-      <c r="M48">
+      <c r="M49">
         <v>5380.5444360000001</v>
       </c>
-      <c r="N48">
+      <c r="N49">
         <v>279.27307350000001</v>
       </c>
-      <c r="O48">
-        <v>0</v>
-      </c>
-      <c r="P48">
+      <c r="O49">
+        <v>0</v>
+      </c>
+      <c r="P49">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q48">
+      <c r="Q49">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R48">
+      <c r="R49">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S48">
+      <c r="S49">
         <v>452.7322633</v>
       </c>
-      <c r="T48">
+      <c r="T49">
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.35">
-      <c r="A49" s="2"/>
+    <row r="50" spans="1:20" x14ac:dyDescent="0.35">
+      <c r="A50" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
re-do results for 2 flex trains to get updated flexiblity metrics
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7682F503-1E77-4599-87A9-53F403D37CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D54FDF3-0911-4EB0-8D32-CA4BA10D1DB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19310" yWindow="10680" windowWidth="19420" windowHeight="10300" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -37,6 +36,7 @@
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
     <author>tc={059B2785-9A39-4C22-958C-B8BAB93BD95A}</author>
+    <author>tc={965CE2E3-2B8D-4852-A22E-FC0AA070113D}</author>
     <author>tc={ABAC2AC6-7A74-4F44-BF4E-754717C772A0}</author>
     <author>tc={9CE96C07-E110-41BE-B453-65310D0A2128}</author>
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
@@ -52,7 +52,15 @@
     Flex_type = rr has same solution</t>
       </text>
     </comment>
-    <comment ref="A24" authorId="1" shapeId="0" xr:uid="{ABAC2AC6-7A74-4F44-BF4E-754717C772A0}">
+    <comment ref="A22" authorId="1" shapeId="0" xr:uid="{965CE2E3-2B8D-4852-A22E-FC0AA070113D}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Will have to re-run to get the flexibility metrics</t>
+      </text>
+    </comment>
+    <comment ref="A24" authorId="2" shapeId="0" xr:uid="{ABAC2AC6-7A74-4F44-BF4E-754717C772A0}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -60,7 +68,7 @@
     Have to re-run with fixed uf recovery and the 2nd order surrogate</t>
       </text>
     </comment>
-    <comment ref="A28" authorId="2" shapeId="0" xr:uid="{9CE96C07-E110-41BE-B453-65310D0A2128}">
+    <comment ref="A28" authorId="3" shapeId="0" xr:uid="{9CE96C07-E110-41BE-B453-65310D0A2128}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -68,7 +76,7 @@
     Summer is the summer hot weekdays + high weekends.</t>
       </text>
     </comment>
-    <comment ref="A29" authorId="3" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A29" authorId="4" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -76,7 +84,7 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
-    <comment ref="T30" authorId="4" shapeId="0" xr:uid="{44AB14B7-66C1-445B-8271-3F9869928B60}">
+    <comment ref="T30" authorId="5" shapeId="0" xr:uid="{44AB14B7-66C1-445B-8271-3F9869928B60}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -84,7 +92,7 @@
     The whole baseline for this might be corrupted</t>
       </text>
     </comment>
-    <comment ref="A34" authorId="5" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A34" authorId="6" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -199,7 +207,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -339,6 +347,12 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1072,6 +1086,9 @@
   <threadedComment ref="A19" dT="2026-05-29T21:01:16.53" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{059B2785-9A39-4C22-958C-B8BAB93BD95A}">
     <text>Flex_type = rr has same solution</text>
   </threadedComment>
+  <threadedComment ref="A22" dT="2026-06-09T01:37:04.84" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{965CE2E3-2B8D-4852-A22E-FC0AA070113D}">
+    <text>Will have to re-run to get the flexibility metrics</text>
+  </threadedComment>
   <threadedComment ref="A24" dT="2026-05-28T22:11:07.28" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{ABAC2AC6-7A74-4F44-BF4E-754717C772A0}">
     <text>Have to re-run with fixed uf recovery and the 2nd order surrogate</text>
   </threadedComment>
@@ -1096,10 +1113,10 @@
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.6328125" customWidth="1"/>
-    <col min="3" max="3" width="12.453125" customWidth="1"/>
+    <col min="3" max="3" width="11.453125" customWidth="1"/>
     <col min="5" max="5" width="10.26953125" customWidth="1"/>
     <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.6328125" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" customWidth="1"/>
     <col min="9" max="9" width="9.08984375" customWidth="1"/>
     <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
@@ -1734,6 +1751,12 @@
       <c r="R15">
         <v>0</v>
       </c>
+      <c r="S15">
+        <v>0</v>
+      </c>
+      <c r="T15">
+        <v>0</v>
+      </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
@@ -1790,6 +1813,12 @@
       <c r="R16">
         <v>0</v>
       </c>
+      <c r="S16">
+        <v>0</v>
+      </c>
+      <c r="T16">
+        <v>0</v>
+      </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.35">
       <c r="G17" s="4"/>
@@ -1849,9 +1878,15 @@
       <c r="R18">
         <v>0</v>
       </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
+      <c r="T18">
+        <v>0</v>
+      </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A19" t="s">
+      <c r="A19" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B19" t="s">
@@ -1902,13 +1937,13 @@
       <c r="Q19">
         <v>1466.9255534444001</v>
       </c>
-      <c r="R19">
+      <c r="R19" s="2">
         <v>22473.732168664301</v>
       </c>
-      <c r="S19">
+      <c r="S19" s="2">
         <v>351.15206513537998</v>
       </c>
-      <c r="T19">
+      <c r="T19" s="2">
         <v>0.79850332454920403</v>
       </c>
     </row>
@@ -1970,9 +2005,15 @@
       <c r="R21">
         <v>0</v>
       </c>
+      <c r="S21">
+        <v>0</v>
+      </c>
+      <c r="T21">
+        <v>0</v>
+      </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A22" t="s">
+      <c r="A22" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B22" t="s">
@@ -2023,13 +2064,13 @@
       <c r="Q22">
         <v>1101.6946284421099</v>
       </c>
-      <c r="R22">
-        <v>0</v>
-      </c>
-      <c r="S22">
+      <c r="R22" s="2">
+        <v>0</v>
+      </c>
+      <c r="S22" s="2">
         <v>487.22587310308802</v>
       </c>
-      <c r="T22">
+      <c r="T22" s="2">
         <v>1.75628458077399</v>
       </c>
     </row>
@@ -2099,7 +2140,7 @@
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.35">
-      <c r="A25" s="3" t="s">
+      <c r="A25" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B25" t="s">
@@ -2150,13 +2191,13 @@
       <c r="Q25">
         <v>1173.3790798621201</v>
       </c>
-      <c r="R25">
+      <c r="R25" s="2">
         <v>12990.682952859001</v>
       </c>
-      <c r="S25">
+      <c r="S25" s="2">
         <v>463.95296260210699</v>
       </c>
-      <c r="T25">
+      <c r="T25" s="2">
         <v>1.63318791126541</v>
       </c>
     </row>
@@ -2510,7 +2551,7 @@
       <c r="F34">
         <v>0.87159189967643702</v>
       </c>
-      <c r="G34">
+      <c r="G34" s="4">
         <v>21072.189860718699</v>
       </c>
       <c r="H34">
@@ -2707,7 +2748,7 @@
       <c r="F41">
         <v>0.840833383054163</v>
       </c>
-      <c r="G41">
+      <c r="G41" s="4">
         <v>20578.507216446698</v>
       </c>
       <c r="H41">
@@ -2763,7 +2804,7 @@
       <c r="F42">
         <v>0.85824890324911396</v>
       </c>
-      <c r="G42">
+      <c r="G42" s="4">
         <v>20824.7129679639</v>
       </c>
       <c r="H42">
@@ -2825,7 +2866,7 @@
       <c r="F44">
         <v>0.84083338305413902</v>
       </c>
-      <c r="G44">
+      <c r="G44" s="4">
         <v>20578.5072164468</v>
       </c>
       <c r="H44">
@@ -2881,7 +2922,7 @@
       <c r="F45">
         <v>0.857351410648304</v>
       </c>
-      <c r="G45">
+      <c r="G45" s="4">
         <v>21285.1004075495</v>
       </c>
       <c r="H45">
@@ -2927,7 +2968,7 @@
     <row r="46" spans="1:20" x14ac:dyDescent="0.35">
       <c r="G46" s="4"/>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>26</v>
       </c>
@@ -2948,7 +2989,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>0</v>
       </c>
@@ -3010,7 +3051,7 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>20</v>
       </c>

</xml_diff>

<commit_message>
Double chekcing baseline costs
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B3C420-F377-46E7-8A7E-73B98C40733A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225C300A-4104-4778-9250-FA3FF0FF0ADF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="33120" windowHeight="18000" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
+    <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
   <sheets>
     <sheet name="wrd_pricetater_flex_type_summar" sheetId="1" r:id="rId1"/>
@@ -35,6 +35,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
+    <author>tc={254E663B-F1EE-4051-97FD-1A302AC42F75}</author>
     <author>tc={DFECE21F-32E0-4210-824A-1E57B1730184}</author>
     <author>tc={F9308CF0-AB74-4ABB-91B6-7382ECEADD39}</author>
     <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
@@ -42,7 +43,15 @@
     <author>tc={7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}</author>
   </authors>
   <commentList>
-    <comment ref="A22" authorId="0" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
+    <comment ref="J4" authorId="0" shapeId="0" xr:uid="{254E663B-F1EE-4051-97FD-1A302AC42F75}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Why is this higher than all the other summer 0 trains options?</t>
+      </text>
+    </comment>
+    <comment ref="A22" authorId="1" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -50,7 +59,7 @@
     Curious if solver would eventually find same solution as the 4 flex trains</t>
       </text>
     </comment>
-    <comment ref="A28" authorId="1" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+    <comment ref="A28" authorId="2" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -58,7 +67,7 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T28" authorId="2" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <comment ref="T28" authorId="3" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -66,7 +75,7 @@
     Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure</t>
       </text>
     </comment>
-    <comment ref="A29" authorId="3" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A29" authorId="4" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -74,7 +83,7 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
-    <comment ref="A34" authorId="4" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A34" authorId="5" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -189,7 +198,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -335,12 +344,6 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1071,6 +1074,9 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="J4" dT="2026-06-26T21:44:43.11" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{254E663B-F1EE-4051-97FD-1A302AC42F75}">
+    <text>Why is this higher than all the other summer 0 trains options?</text>
+  </threadedComment>
   <threadedComment ref="A22" dT="2026-06-11T20:38:07.96" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{DFECE21F-32E0-4210-824A-1E57B1730184}">
     <text>Curious if solver would eventually find same solution as the 4 flex trains</text>
   </threadedComment>
@@ -1092,23 +1098,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:T50"/>
-  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="9.61328125" customWidth="1"/>
-    <col min="3" max="3" width="11.4609375" customWidth="1"/>
-    <col min="5" max="5" width="10.23046875" customWidth="1"/>
-    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.69140625" customWidth="1"/>
-    <col min="9" max="9" width="9.07421875" customWidth="1"/>
-    <col min="20" max="20" width="7.84375" customWidth="1"/>
+    <col min="1" max="1" width="9.6328125" customWidth="1"/>
+    <col min="3" max="3" width="11.453125" customWidth="1"/>
+    <col min="5" max="5" width="10.26953125" customWidth="1"/>
+    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.7265625" customWidth="1"/>
+    <col min="9" max="9" width="9.08984375" customWidth="1"/>
+    <col min="20" max="20" width="7.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1170,7 +1176,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1232,7 +1238,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1294,10 +1300,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1359,7 +1365,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -1421,10 +1427,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1486,7 +1492,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1548,12 +1554,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
         <v>21</v>
@@ -1562,34 +1568,34 @@
         <v>0</v>
       </c>
       <c r="D12">
-        <v>120105.62640119799</v>
+        <v>111142.758477303</v>
       </c>
       <c r="E12">
         <v>282179.67123287602</v>
       </c>
       <c r="F12">
-        <v>0.85639623815652299</v>
+        <v>0.82463325578173197</v>
       </c>
       <c r="G12" s="4">
-        <v>20632.008189972999</v>
+        <v>18240.8407502021</v>
       </c>
       <c r="H12">
-        <v>4931.94871395263</v>
+        <v>4851.2693328072801</v>
       </c>
       <c r="I12">
-        <v>9097.1451203198394</v>
+        <v>2606.1355131391001</v>
       </c>
       <c r="J12">
-        <v>34661.102024245498</v>
+        <v>25698.245596148499</v>
       </c>
       <c r="K12">
-        <v>50843.186957348102</v>
+        <v>50843.1840059237</v>
       </c>
       <c r="L12">
-        <v>15303.8063177357</v>
+        <v>15303.7983857831</v>
       </c>
       <c r="M12">
-        <v>19297.531101868899</v>
+        <v>19297.530489448302</v>
       </c>
       <c r="N12">
         <v>992.31070788530405</v>
@@ -1598,10 +1604,10 @@
         <v>0</v>
       </c>
       <c r="P12">
-        <v>241657.60892808001</v>
+        <v>232694.74100418499</v>
       </c>
       <c r="Q12">
-        <v>1101.9194839550801</v>
+        <v>1101.5718970651201</v>
       </c>
       <c r="R12">
         <v>0</v>
@@ -1613,9 +1619,9 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B13" t="s">
         <v>21</v>
@@ -1624,34 +1630,34 @@
         <v>0</v>
       </c>
       <c r="D13">
-        <v>111142.758477303</v>
+        <v>120105.62640119799</v>
       </c>
       <c r="E13">
         <v>282179.67123287602</v>
       </c>
       <c r="F13">
-        <v>0.82463325578173197</v>
+        <v>0.85639623815652299</v>
       </c>
       <c r="G13" s="4">
-        <v>18240.8407502021</v>
+        <v>20632.008189972999</v>
       </c>
       <c r="H13">
-        <v>4851.2693328072801</v>
+        <v>4931.94871395263</v>
       </c>
       <c r="I13">
-        <v>2606.1355131391001</v>
+        <v>9097.1451203198394</v>
       </c>
       <c r="J13">
-        <v>25698.245596148499</v>
+        <v>34661.102024245498</v>
       </c>
       <c r="K13">
-        <v>50843.1840059237</v>
+        <v>50843.186957348102</v>
       </c>
       <c r="L13">
-        <v>15303.7983857831</v>
+        <v>15303.8063177357</v>
       </c>
       <c r="M13">
-        <v>19297.530489448302</v>
+        <v>19297.531101868899</v>
       </c>
       <c r="N13">
         <v>992.31070788530405</v>
@@ -1660,10 +1666,10 @@
         <v>0</v>
       </c>
       <c r="P13">
-        <v>232694.74100418499</v>
+        <v>241657.60892808001</v>
       </c>
       <c r="Q13">
-        <v>1101.5718970651201</v>
+        <v>1101.9194839550801</v>
       </c>
       <c r="R13">
         <v>0</v>
@@ -1675,10 +1681,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1740,7 +1746,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1802,10 +1808,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1867,7 +1873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19" s="3" t="s">
         <v>22</v>
       </c>
@@ -1929,10 +1935,10 @@
         <v>0.864044481174707</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -1994,7 +2000,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2056,10 +2062,10 @@
         <v>1.20740363486328</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A24" s="3" t="s">
         <v>20</v>
       </c>
@@ -2121,7 +2127,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -2183,13 +2189,13 @@
         <v>1.42140322536358</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G27" s="4"/>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -2251,7 +2257,7 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A29" s="3" t="s">
         <v>20</v>
       </c>
@@ -2313,7 +2319,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>22</v>
       </c>
@@ -2375,7 +2381,7 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>20</v>
       </c>
@@ -2437,10 +2443,10 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
       <c r="G32" s="4"/>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A33" s="3" t="s">
         <v>20</v>
       </c>
@@ -2502,7 +2508,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>22</v>
       </c>
@@ -2564,13 +2570,13 @@
         <v>0.51444695802960605</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A36" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G36" s="4"/>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -2632,7 +2638,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>22</v>
       </c>
@@ -2694,12 +2700,12 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A40" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>20</v>
       </c>
@@ -2755,7 +2761,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>22</v>
       </c>
@@ -2817,7 +2823,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>20</v>
       </c>
@@ -2873,7 +2879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>22</v>
       </c>
@@ -2935,10 +2941,10 @@
         <v>1.3585822738026401</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.35">
       <c r="G46" s="4"/>
     </row>
-    <row r="47" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47" s="1" t="s">
         <v>26</v>
       </c>
@@ -2959,7 +2965,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>0</v>
       </c>
@@ -3021,7 +3027,7 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="49" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>20</v>
       </c>
@@ -3083,7 +3089,7 @@
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A50" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Continuing to check baseline solution
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -1,7 +1,7 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
@@ -198,7 +198,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -338,12 +338,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1098,23 +1092,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
   <dimension ref="A1:T50"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="1" max="1" width="9.6328125" customWidth="1"/>
-    <col min="3" max="3" width="11.453125" customWidth="1"/>
-    <col min="5" max="5" width="10.26953125" customWidth="1"/>
-    <col min="6" max="6" width="11.81640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.7265625" customWidth="1"/>
-    <col min="9" max="9" width="9.08984375" customWidth="1"/>
-    <col min="20" max="20" width="7.81640625" customWidth="1"/>
+    <col min="1" max="1" width="9.61328125" customWidth="1"/>
+    <col min="3" max="3" width="11.4609375" customWidth="1"/>
+    <col min="5" max="5" width="10.23046875" customWidth="1"/>
+    <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.69140625" customWidth="1"/>
+    <col min="9" max="9" width="9.07421875" customWidth="1"/>
+    <col min="20" max="20" width="7.84375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -1176,7 +1170,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>20</v>
       </c>
@@ -1238,7 +1232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A4" t="s">
         <v>22</v>
       </c>
@@ -1300,10 +1294,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1365,7 +1359,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A7" t="s">
         <v>22</v>
       </c>
@@ -1427,10 +1421,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G8" s="4"/>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A9" t="s">
         <v>20</v>
       </c>
@@ -1492,7 +1486,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -1554,10 +1548,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G11" s="4"/>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A12" t="s">
         <v>20</v>
       </c>
@@ -1619,7 +1613,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A13" t="s">
         <v>22</v>
       </c>
@@ -1681,10 +1675,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1746,7 +1740,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A16" t="s">
         <v>22</v>
       </c>
@@ -1808,10 +1802,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1873,7 +1867,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
         <v>22</v>
       </c>
@@ -1935,10 +1929,10 @@
         <v>0.864044481174707</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G20" s="4"/>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -2000,7 +1994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A22" s="3" t="s">
         <v>22</v>
       </c>
@@ -2062,10 +2056,10 @@
         <v>1.20740363486328</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G23" s="4"/>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A24" s="3" t="s">
         <v>20</v>
       </c>
@@ -2127,7 +2121,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A25" t="s">
         <v>22</v>
       </c>
@@ -2189,13 +2183,13 @@
         <v>1.42140322536358</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A27" s="1" t="s">
         <v>27</v>
       </c>
       <c r="G27" s="4"/>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A28" t="s">
         <v>22</v>
       </c>
@@ -2257,7 +2251,7 @@
         <v>-14.696886263168601</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A29" s="3" t="s">
         <v>20</v>
       </c>
@@ -2319,7 +2313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A30" t="s">
         <v>22</v>
       </c>
@@ -2381,7 +2375,7 @@
         <v>-3.6405201993767098</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A31" t="s">
         <v>20</v>
       </c>
@@ -2443,10 +2437,10 @@
         <v>1103.3673370121001</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G32" s="4"/>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A33" s="3" t="s">
         <v>20</v>
       </c>
@@ -2508,7 +2502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>22</v>
       </c>
@@ -2570,13 +2564,13 @@
         <v>0.51444695802960605</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A36" s="1" t="s">
         <v>30</v>
       </c>
       <c r="G36" s="4"/>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A37" t="s">
         <v>22</v>
       </c>
@@ -2638,7 +2632,7 @@
         <v>2.4302910949698302</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
         <v>22</v>
       </c>
@@ -2700,12 +2694,12 @@
         <v>1.09609872121186</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A40" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
         <v>20</v>
       </c>
@@ -2761,7 +2755,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A42" t="s">
         <v>22</v>
       </c>
@@ -2823,7 +2817,7 @@
         <v>1.0959871186973</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
         <v>20</v>
       </c>
@@ -2879,7 +2873,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A45" t="s">
         <v>22</v>
       </c>
@@ -2941,10 +2935,10 @@
         <v>1.3585822738026401</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.4">
       <c r="G46" s="4"/>
     </row>
-    <row r="47" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
       <c r="A47" s="1" t="s">
         <v>26</v>
       </c>
@@ -2965,7 +2959,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="48" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
       <c r="A48" t="s">
         <v>0</v>
       </c>
@@ -3027,7 +3021,7 @@
         <v>27.514184579999998</v>
       </c>
     </row>
-    <row r="49" spans="1:20" hidden="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
       <c r="A49" s="2" t="s">
         <v>20</v>
       </c>
@@ -3089,7 +3083,7 @@
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A50" s="2"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Redoing num flex trains results w/ smaller mip gap
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{225C300A-4104-4778-9250-FA3FF0FF0ADF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D857DAE1-5DC0-4E20-8DFC-3DB63AB89CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={254E663B-F1EE-4051-97FD-1A302AC42F75}</author>
+    <author>tc={69B04875-FCD3-4F29-8B43-FEF02E31358C}</author>
     <author>tc={DFECE21F-32E0-4210-824A-1E57B1730184}</author>
     <author>tc={F9308CF0-AB74-4ABB-91B6-7382ECEADD39}</author>
     <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
@@ -43,12 +43,12 @@
     <author>tc={7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}</author>
   </authors>
   <commentList>
-    <comment ref="J4" authorId="0" shapeId="0" xr:uid="{254E663B-F1EE-4051-97FD-1A302AC42F75}">
+    <comment ref="A12" authorId="0" shapeId="0" xr:uid="{69B04875-FCD3-4F29-8B43-FEF02E31358C}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Why is this higher than all the other summer 0 trains options?</t>
+    Should be just exactly the same as the baseline if given enough time to run and corrected baseline</t>
       </text>
     </comment>
     <comment ref="A22" authorId="1" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
@@ -198,7 +198,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -338,6 +338,26 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="6"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="5"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -681,12 +701,14 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1068,8 +1090,8 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="J4" dT="2026-06-26T21:44:43.11" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{254E663B-F1EE-4051-97FD-1A302AC42F75}">
-    <text>Why is this higher than all the other summer 0 trains options?</text>
+  <threadedComment ref="A12" dT="2026-06-29T16:52:54.51" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{69B04875-FCD3-4F29-8B43-FEF02E31358C}">
+    <text>Should be just exactly the same as the baseline if given enough time to run and corrected baseline</text>
   </threadedComment>
   <threadedComment ref="A22" dT="2026-06-11T20:38:07.96" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{DFECE21F-32E0-4210-824A-1E57B1730184}">
     <text>Curious if solver would eventually find same solution as the 4 flex trains</text>
@@ -1171,44 +1193,44 @@
       </c>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A3" t="s">
+      <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>111737.917851103</v>
+        <v>111145.161086081</v>
       </c>
       <c r="E3">
-        <v>282179.67125484499</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F3">
-        <v>0.826742406143402</v>
-      </c>
-      <c r="G3" s="4">
-        <v>18663.290146715601</v>
+        <v>0.82464177024617602</v>
+      </c>
+      <c r="G3">
+        <v>18242.5461916684</v>
       </c>
       <c r="H3">
-        <v>4963.6224309139197</v>
+        <v>4851.7228614100204</v>
       </c>
       <c r="I3">
-        <v>2666.4923762402</v>
+        <v>2606.3791518481999</v>
       </c>
       <c r="J3">
-        <v>26293.4049538697</v>
+        <v>25700.648204926601</v>
       </c>
       <c r="K3">
-        <v>50843.184012302001</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L3">
-        <v>15303.798393478701</v>
+        <v>15303.798385783</v>
       </c>
       <c r="M3">
-        <v>19297.530491452799</v>
+        <v>19297.5304894482</v>
       </c>
       <c r="N3">
         <v>992.31070788530405</v>
@@ -1217,10 +1239,10 @@
         <v>0</v>
       </c>
       <c r="P3">
-        <v>233289.900377985</v>
+        <v>232697.143612963</v>
       </c>
       <c r="Q3">
-        <v>1127.0837800240299</v>
+        <v>1101.6748792595399</v>
       </c>
       <c r="R3">
         <v>0</v>
@@ -1233,44 +1255,44 @@
       </c>
     </row>
     <row r="4" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A4" t="s">
+      <c r="A4" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C4">
         <v>0</v>
       </c>
       <c r="D4">
-        <v>120897.164660582</v>
+        <v>120097.924543835</v>
       </c>
       <c r="E4">
-        <v>282179.67125255102</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F4">
-        <v>0.85920132414667005</v>
-      </c>
-      <c r="G4" s="4">
-        <v>21103.178564432201</v>
+        <v>0.85636894399557495</v>
+      </c>
+      <c r="G4">
+        <v>20627.43117349</v>
       </c>
       <c r="H4">
-        <v>5044.5785543711099</v>
+        <v>4930.8542128783001</v>
       </c>
       <c r="I4">
-        <v>9304.8946454247507</v>
+        <v>9095.1262763121395</v>
       </c>
       <c r="J4">
-        <v>35452.651764228103</v>
+        <v>34653.411662680403</v>
       </c>
       <c r="K4">
-        <v>50843.1840118412</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L4">
-        <v>15303.7983932269</v>
+        <v>15303.798385783</v>
       </c>
       <c r="M4">
-        <v>19297.530491286099</v>
+        <v>19297.5304894482</v>
       </c>
       <c r="N4">
         <v>992.31070788530405</v>
@@ -1279,10 +1301,10 @@
         <v>0</v>
       </c>
       <c r="P4">
-        <v>242449.147187464</v>
+        <v>241649.90707071699</v>
       </c>
       <c r="Q4">
-        <v>1127.0837796179201</v>
+        <v>1101.6749453094101</v>
       </c>
       <c r="R4">
         <v>0</v>
@@ -1552,10 +1574,10 @@
       <c r="G11" s="4"/>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A12" t="s">
+      <c r="A12" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C12">
@@ -1614,10 +1636,10 @@
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A13" t="s">
+      <c r="A13" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C13">

</xml_diff>

<commit_message>
one flexible train  0 mip gap
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D857DAE1-5DC0-4E20-8DFC-3DB63AB89CBB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ADA1792-FDE0-431C-8A76-29307BDF8056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -198,7 +198,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -352,12 +352,6 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="33">
@@ -1763,64 +1757,58 @@
       </c>
     </row>
     <row r="16" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A16" t="s">
+      <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="6" t="s">
         <v>23</v>
       </c>
       <c r="C16">
         <v>1</v>
       </c>
       <c r="D16">
-        <v>121661.732552156</v>
+        <v>120212.88333435199</v>
       </c>
       <c r="E16">
-        <v>282322.94999999902</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F16">
-        <v>0.86147341220059803</v>
-      </c>
-      <c r="G16" s="4">
-        <v>20583.8776149273</v>
+        <v>0.85677633971623302</v>
+      </c>
+      <c r="G16">
+        <v>20695.8603534904</v>
       </c>
       <c r="H16">
-        <v>6564.2083881818999</v>
+        <v>4947.2117663766303</v>
       </c>
       <c r="I16">
-        <v>9025.7485990471305</v>
+        <v>9125.2983334621895</v>
       </c>
       <c r="J16">
-        <v>36173.834602156297</v>
+        <v>34768.370453329197</v>
       </c>
       <c r="K16">
-        <v>50869</v>
+        <v>50843.184005889801</v>
       </c>
       <c r="L16">
-        <v>15311.569</v>
+        <v>15303.798385692</v>
       </c>
       <c r="M16">
-        <v>19307.328949999999</v>
+        <v>19297.530489441298</v>
       </c>
       <c r="N16">
-        <v>994.09650999907501</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O16">
         <v>0</v>
       </c>
       <c r="P16">
-        <v>243213.715079038</v>
+        <v>241764.86586123399</v>
       </c>
       <c r="Q16">
-        <v>1466.6067124359399</v>
+        <v>1105.32962817471</v>
       </c>
       <c r="R16">
-        <v>0</v>
-      </c>
-      <c r="S16">
-        <v>0</v>
-      </c>
-      <c r="T16">
         <v>0</v>
       </c>
     </row>
@@ -1890,10 +1878,10 @@
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A19" s="3" t="s">
+      <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="5" t="s">
         <v>23</v>
       </c>
       <c r="C19">
@@ -1942,13 +1930,13 @@
         <v>1468.64372040951</v>
       </c>
       <c r="R19">
-        <v>20699.963288031398</v>
+        <v>17615.608874695899</v>
       </c>
       <c r="S19">
-        <v>173.94927132799501</v>
+        <v>266.90316476812001</v>
       </c>
       <c r="T19">
-        <v>0.864044481174707</v>
+        <v>9.6260597723556093E-2</v>
       </c>
     </row>
     <row r="20" spans="1:20" x14ac:dyDescent="0.4">

</xml_diff>

<commit_message>
baseline for TOU 8
</commit_message>
<xml_diff>
--- a/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
+++ b/tutorials/flex_ro/wrd_pricetater_flex_type_summary.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\rchurchi\watertap\tutorials\flex_ro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ADA1792-FDE0-431C-8A76-29307BDF8056}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FF0A6E1-B90F-40B0-9AC7-61A42977BB0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="57480" yWindow="8430" windowWidth="29040" windowHeight="15720" xr2:uid="{C549BF93-41CE-4809-A3B1-A16DB1FF836F}"/>
   </bookViews>
@@ -35,23 +35,35 @@
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
 <comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
   <authors>
-    <author>tc={69B04875-FCD3-4F29-8B43-FEF02E31358C}</author>
+    <author>tc={CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}</author>
+    <author>tc={815F3FDC-C725-4656-9AA0-DDB81C7546AD}</author>
     <author>tc={DFECE21F-32E0-4210-824A-1E57B1730184}</author>
+    <author>tc={D42C0CEC-223C-40FD-88E7-B5BC8DDF118E}</author>
+    <author>tc={82EE7A36-D8EE-4051-AEAE-B403E815DFF2}</author>
     <author>tc={F9308CF0-AB74-4ABB-91B6-7382ECEADD39}</author>
     <author>tc={B08B550A-B779-4CE5-A29D-4C76A4C93C7E}</author>
     <author>tc={FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}</author>
     <author>tc={7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}</author>
+    <author>tc={86E634AB-9E52-4A6D-BE85-5D191C9227C6}</author>
   </authors>
   <commentList>
-    <comment ref="A12" authorId="0" shapeId="0" xr:uid="{69B04875-FCD3-4F29-8B43-FEF02E31358C}">
+    <comment ref="A16" authorId="0" shapeId="0" xr:uid="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Should be just exactly the same as the baseline if given enough time to run and corrected baseline</t>
+    This should be the same as the baseline</t>
       </text>
     </comment>
-    <comment ref="A22" authorId="1" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
+    <comment ref="A22" authorId="1" shapeId="0" xr:uid="{815F3FDC-C725-4656-9AA0-DDB81C7546AD}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Have to rerun if I want to get the correct Flexibility metrics</t>
+      </text>
+    </comment>
+    <comment ref="A25" authorId="2" shapeId="0" xr:uid="{DFECE21F-32E0-4210-824A-1E57B1730184}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -59,7 +71,23 @@
     Curious if solver would eventually find same solution as the 4 flex trains</t>
       </text>
     </comment>
-    <comment ref="A28" authorId="2" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+    <comment ref="A28" authorId="3" shapeId="0" xr:uid="{D42C0CEC-223C-40FD-88E7-B5BC8DDF118E}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Need to rerun to confirm shutdowns are not optimal</t>
+      </text>
+    </comment>
+    <comment ref="A30" authorId="4" shapeId="0" xr:uid="{82EE7A36-D8EE-4051-AEAE-B403E815DFF2}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    With a lower flow change penalty, this might become possible</t>
+      </text>
+    </comment>
+    <comment ref="A34" authorId="5" shapeId="0" xr:uid="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -67,15 +95,17 @@
     Summer week = hot summer weekdays + high weekends</t>
       </text>
     </comment>
-    <comment ref="T28" authorId="3" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <comment ref="T34" authorId="6" shapeId="0" xr:uid="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure</t>
+    Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure
+Reply:
+    The baseline costs have to be updated in accordance with the demand structure type</t>
       </text>
     </comment>
-    <comment ref="A29" authorId="4" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+    <comment ref="A35" authorId="7" shapeId="0" xr:uid="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -83,7 +113,7 @@
     Winter is low winter weekdays + low weekends</t>
       </text>
     </comment>
-    <comment ref="A34" authorId="5" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+    <comment ref="A41" authorId="8" shapeId="0" xr:uid="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -91,12 +121,20 @@
     Result from the fast solve</t>
       </text>
     </comment>
+    <comment ref="T67" authorId="9" shapeId="0" xr:uid="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    These LVOF numbers are nonsense because the baseline costs are not the same</t>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="120" uniqueCount="36">
   <si>
     <t>Season</t>
   </si>
@@ -193,12 +231,24 @@
   <si>
     <t>TOU 8</t>
   </si>
+  <si>
+    <t>Link to result: https://github.com/jakechurchi/watertap/blob/77b0fd3a12650b35dc7419a8ee835ba61fcc1512/tutorials/flex_ro/wrd_pricetaker_summary_results_20260529_155321.csv</t>
+  </si>
+  <si>
+    <t>Simplified Rate Structures</t>
+  </si>
+  <si>
+    <t>Off-Peak Demand Charge</t>
+  </si>
+  <si>
+    <t>On-Peak Demand Charge</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -349,6 +399,19 @@
     <font>
       <sz val="11"/>
       <color theme="5"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -695,7 +758,7 @@
     <xf numFmtId="0" fontId="1" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -703,6 +766,7 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1084,30 +1148,45 @@
 
 <file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="A12" dT="2026-06-29T16:52:54.51" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{69B04875-FCD3-4F29-8B43-FEF02E31358C}">
-    <text>Should be just exactly the same as the baseline if given enough time to run and corrected baseline</text>
+  <threadedComment ref="A16" dT="2026-07-01T17:37:32.24" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{CD2318A4-5B8F-4EC0-9DFB-E52F2D041746}">
+    <text>This should be the same as the baseline</text>
   </threadedComment>
-  <threadedComment ref="A22" dT="2026-06-11T20:38:07.96" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{DFECE21F-32E0-4210-824A-1E57B1730184}">
+  <threadedComment ref="A22" dT="2026-07-01T17:39:57.41" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{815F3FDC-C725-4656-9AA0-DDB81C7546AD}">
+    <text>Have to rerun if I want to get the correct Flexibility metrics</text>
+  </threadedComment>
+  <threadedComment ref="A25" dT="2026-06-11T20:38:07.96" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{DFECE21F-32E0-4210-824A-1E57B1730184}">
     <text>Curious if solver would eventually find same solution as the 4 flex trains</text>
   </threadedComment>
-  <threadedComment ref="A28" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
+  <threadedComment ref="A28" dT="2026-07-01T18:06:46.80" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{D42C0CEC-223C-40FD-88E7-B5BC8DDF118E}">
+    <text>Need to rerun to confirm shutdowns are not optimal</text>
+  </threadedComment>
+  <threadedComment ref="A30" dT="2026-07-01T19:38:50.85" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{82EE7A36-D8EE-4051-AEAE-B403E815DFF2}">
+    <text>With a lower flow change penalty, this might become possible</text>
+  </threadedComment>
+  <threadedComment ref="A34" dT="2026-06-12T21:26:36.67" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{F9308CF0-AB74-4ABB-91B6-7382ECEADD39}">
     <text>Summer week = hot summer weekdays + high weekends</text>
   </threadedComment>
-  <threadedComment ref="T28" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+  <threadedComment ref="T34" dT="2026-06-12T21:26:04.82" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
     <text>Don’t think I trust these metrics. Would have to re-run if we want to provide that number for this rate structure</text>
   </threadedComment>
-  <threadedComment ref="A29" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
+  <threadedComment ref="T34" dT="2026-07-01T19:24:49.07" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{9EBF37B2-9A03-4803-834C-7A4B424AFD1D}" parentId="{B08B550A-B779-4CE5-A29D-4C76A4C93C7E}">
+    <text>The baseline costs have to be updated in accordance with the demand structure type</text>
+  </threadedComment>
+  <threadedComment ref="A35" dT="2026-05-27T21:42:09.38" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{FC7CAB31-3DEE-4F30-9288-CDF327BE04E1}">
     <text>Winter is low winter weekdays + low weekends</text>
   </threadedComment>
-  <threadedComment ref="A34" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
+  <threadedComment ref="A41" dT="2026-06-02T17:16:43.70" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{7C262D24-4F73-4A8D-BEED-4FCDB02EBE54}">
     <text>Result from the fast solve</text>
+  </threadedComment>
+  <threadedComment ref="T67" dT="2026-07-01T19:24:18.69" personId="{114E4FE4-B7B1-4FA3-A72A-3A97E9B9C3CF}" id="{86E634AB-9E52-4A6D-BE85-5D191C9227C6}">
+    <text>These LVOF numbers are nonsense because the baseline costs are not the same</text>
   </threadedComment>
 </ThreadedComments>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{685A11F3-C438-4D9E-9154-F58427CB6366}">
-  <dimension ref="A1:T50"/>
+  <dimension ref="A1:U70"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="9.61328125" customWidth="1"/>
@@ -1116,6 +1195,7 @@
     <col min="6" max="6" width="11.84375" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="10.69140625" customWidth="1"/>
     <col min="9" max="9" width="9.07421875" customWidth="1"/>
+    <col min="15" max="15" width="9.53515625" customWidth="1"/>
     <col min="20" max="20" width="7.84375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1568,10 +1648,10 @@
       <c r="G11" s="4"/>
     </row>
     <row r="12" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C12">
@@ -1630,10 +1710,10 @@
       </c>
     </row>
     <row r="13" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="B13" s="6" t="s">
+      <c r="B13" s="3" t="s">
         <v>21</v>
       </c>
       <c r="C13">
@@ -1691,10 +1771,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
       <c r="G14" s="4"/>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
       <c r="A15" t="s">
         <v>20</v>
       </c>
@@ -1756,7 +1836,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
       <c r="A16" s="6" t="s">
         <v>22</v>
       </c>
@@ -1812,10 +1892,10 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.4">
       <c r="G17" s="4"/>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A18" t="s">
         <v>20</v>
       </c>
@@ -1877,7 +1957,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A19" s="5" t="s">
         <v>22</v>
       </c>
@@ -1939,175 +2019,95 @@
         <v>9.6260597723556093E-2</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="G20" s="4"/>
-    </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="A20" s="5"/>
+      <c r="B20" s="5"/>
+    </row>
+    <row r="21" spans="1:21" x14ac:dyDescent="0.4">
       <c r="A21" t="s">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C21">
         <v>2</v>
       </c>
-      <c r="D21">
+    </row>
+    <row r="22" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="A22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C22" s="2">
+        <v>2</v>
+      </c>
+      <c r="G22" s="4">
+        <v>20277.993676447401</v>
+      </c>
+      <c r="H22">
+        <v>6534.5593757614897</v>
+      </c>
+      <c r="I22">
+        <v>5996.9333902952303</v>
+      </c>
+      <c r="J22">
+        <v>32809.486442504203</v>
+      </c>
+      <c r="L22">
+        <v>15303.798385783</v>
+      </c>
+      <c r="P22">
+        <v>239805.98185054099</v>
+      </c>
+      <c r="U22" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="23" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="G23" s="4"/>
+    </row>
+    <row r="24" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="A24" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="B24" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="C24">
+        <v>2</v>
+      </c>
+      <c r="D24">
         <v>111737.92287843001</v>
       </c>
-      <c r="E21">
+      <c r="E24">
         <v>282179.67125484499</v>
       </c>
-      <c r="F21">
+      <c r="F24">
         <v>0.82674242395945297</v>
       </c>
-      <c r="G21" s="4">
+      <c r="G24" s="4">
         <v>18663.290416404601</v>
       </c>
-      <c r="H21">
+      <c r="H24">
         <v>4963.6225077490999</v>
       </c>
-      <c r="I21">
+      <c r="I24">
         <v>2666.4924108713899</v>
       </c>
-      <c r="J21">
+      <c r="J24">
         <v>26293.405335025102</v>
       </c>
-      <c r="K21">
+      <c r="K24">
         <v>50843.185205157402</v>
       </c>
-      <c r="L21">
+      <c r="L24">
         <v>15303.8015992776</v>
       </c>
-      <c r="M21">
+      <c r="M24">
         <v>19297.530738970301</v>
-      </c>
-      <c r="N21">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O21">
-        <v>0</v>
-      </c>
-      <c r="P21">
-        <v>233289.90540531199</v>
-      </c>
-      <c r="Q21">
-        <v>1127.08379747136</v>
-      </c>
-      <c r="R21">
-        <v>0</v>
-      </c>
-      <c r="S21">
-        <v>0</v>
-      </c>
-      <c r="T21">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A22" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B22" t="s">
-        <v>21</v>
-      </c>
-      <c r="C22">
-        <v>2</v>
-      </c>
-      <c r="D22">
-        <v>117590.90519865</v>
-      </c>
-      <c r="E22">
-        <v>282179.671232878</v>
-      </c>
-      <c r="F22">
-        <v>0.84748446505974995</v>
-      </c>
-      <c r="G22">
-        <v>19872.5530246782</v>
-      </c>
-      <c r="H22">
-        <v>5801.3546413486602</v>
-      </c>
-      <c r="I22">
-        <v>5871.6372791994399</v>
-      </c>
-      <c r="J22">
-        <v>31545.544945226298</v>
-      </c>
-      <c r="K22">
-        <v>50997.445205479402</v>
-      </c>
-      <c r="L22">
-        <v>15718.375359588401</v>
-      </c>
-      <c r="M22">
-        <v>19329.539688356101</v>
-      </c>
-      <c r="N22">
-        <v>1001.30446052474</v>
-      </c>
-      <c r="O22">
-        <v>0</v>
-      </c>
-      <c r="P22">
-        <v>239142.887725532</v>
-      </c>
-      <c r="Q22">
-        <v>1296.16628121386</v>
-      </c>
-      <c r="R22">
-        <v>15990.3109099755</v>
-      </c>
-      <c r="S22">
-        <v>135.51110940657199</v>
-      </c>
-      <c r="T22">
-        <v>1.20740363486328</v>
-      </c>
-    </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="G23" s="4"/>
-    </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A24" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B24" t="s">
-        <v>21</v>
-      </c>
-      <c r="C24">
-        <v>4</v>
-      </c>
-      <c r="D24">
-        <v>103263.067623782</v>
-      </c>
-      <c r="E24">
-        <v>282179.67123287701</v>
-      </c>
-      <c r="F24">
-        <v>0.79670888114802996</v>
-      </c>
-      <c r="G24" s="4">
-        <v>18270.343045682599</v>
-      </c>
-      <c r="H24">
-        <v>4859.1187222275803</v>
-      </c>
-      <c r="I24">
-        <v>2610.3522592715499</v>
-      </c>
-      <c r="J24">
-        <v>25739.814027181699</v>
-      </c>
-      <c r="K24">
-        <v>48809.484574716203</v>
-      </c>
-      <c r="L24">
-        <v>9838.23116441202</v>
-      </c>
-      <c r="M24">
-        <v>18875.537857472798</v>
       </c>
       <c r="N24">
         <v>992.31070788530405</v>
@@ -2116,10 +2116,10 @@
         <v>0</v>
       </c>
       <c r="P24">
-        <v>224815.050150664</v>
+        <v>233289.90540531199</v>
       </c>
       <c r="Q24">
-        <v>1103.3542485400801</v>
+        <v>1127.08379747136</v>
       </c>
       <c r="R24">
         <v>0</v>
@@ -2131,45 +2131,45 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A25" t="s">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="A25" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="6" t="s">
         <v>21</v>
       </c>
       <c r="C25">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D25">
-        <v>117493.882010934</v>
+        <v>117590.90519865</v>
       </c>
       <c r="E25">
-        <v>282179.67123284901</v>
+        <v>282179.671232878</v>
       </c>
       <c r="F25">
-        <v>0.84714063027084496</v>
+        <v>0.84748446505974995</v>
       </c>
       <c r="G25">
-        <v>19869.854426770002</v>
+        <v>19872.5530246782</v>
       </c>
       <c r="H25">
-        <v>5589.63461833969</v>
+        <v>5801.3546413486602</v>
       </c>
       <c r="I25">
-        <v>5989.0327102104202</v>
+        <v>5871.6372791994399</v>
       </c>
       <c r="J25">
-        <v>31448.5217553201</v>
+        <v>31545.544945226298</v>
       </c>
       <c r="K25">
-        <v>50997.445205592398</v>
+        <v>50997.445205479402</v>
       </c>
       <c r="L25">
-        <v>15718.3753616421</v>
+        <v>15718.375359588401</v>
       </c>
       <c r="M25">
-        <v>19329.5396883797</v>
+        <v>19329.539688356101</v>
       </c>
       <c r="N25">
         <v>1001.30446052474</v>
@@ -2178,190 +2178,89 @@
         <v>0</v>
       </c>
       <c r="P25">
-        <v>239045.864537816</v>
+        <v>239142.887725532</v>
       </c>
       <c r="Q25">
-        <v>1248.8628027930299</v>
+        <v>1296.16628121386</v>
       </c>
       <c r="R25">
-        <v>13651.1458247473</v>
+        <v>15990.3109099755</v>
       </c>
       <c r="S25">
-        <v>115.68767648091</v>
+        <v>135.51110940657199</v>
       </c>
       <c r="T25">
-        <v>1.42140322536358</v>
-      </c>
-    </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A27" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="G27" s="4"/>
-    </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A28" t="s">
+        <v>1.20740363486328</v>
+      </c>
+    </row>
+    <row r="26" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+    </row>
+    <row r="27" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="A27" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C27">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="28" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="A28" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="2" t="s">
         <v>23</v>
       </c>
       <c r="C28">
-        <v>0</v>
-      </c>
-      <c r="D28">
-        <v>187020.456722612</v>
-      </c>
-      <c r="E28">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F28">
-        <v>1.09353178385</v>
-      </c>
-      <c r="G28">
-        <v>89520.694507565597</v>
-      </c>
-      <c r="H28">
-        <v>6971.3813103080802</v>
-      </c>
-      <c r="I28">
-        <v>5083.8680235841202</v>
-      </c>
-      <c r="J28">
-        <v>101575.943841457</v>
-      </c>
-      <c r="K28">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L28">
-        <v>15303.798385783</v>
-      </c>
-      <c r="M28">
-        <v>19297.5304894482</v>
-      </c>
-      <c r="N28">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O28">
-        <v>0</v>
-      </c>
-      <c r="P28">
-        <v>308572.439249494</v>
-      </c>
-      <c r="Q28">
-        <v>1106.4527933521999</v>
-      </c>
-      <c r="R28">
-        <v>3451.9307168288801</v>
-      </c>
-      <c r="S28">
-        <v>20.547206647791</v>
-      </c>
-      <c r="T28">
-        <v>-14.696886263168601</v>
-      </c>
-    </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A29" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="29" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="G29" s="4"/>
+    </row>
+    <row r="30" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="A30" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B29" t="s">
-        <v>23</v>
-      </c>
-      <c r="C29">
-        <v>0</v>
-      </c>
-      <c r="D29">
-        <v>247948.64160389101</v>
-      </c>
-      <c r="E29">
-        <v>374203.2</v>
-      </c>
-      <c r="F29">
-        <v>0.98743309552342695</v>
-      </c>
-      <c r="G29" s="4">
-        <v>118659.96685142</v>
-      </c>
-      <c r="H29">
-        <v>9240.5882208594503</v>
-      </c>
-      <c r="I29">
-        <v>6738.6833231561404</v>
-      </c>
-      <c r="J29">
-        <v>134639.23839543501</v>
-      </c>
-      <c r="K29">
-        <v>67424.000002171</v>
-      </c>
-      <c r="L29">
-        <v>20294.624005833801</v>
-      </c>
-      <c r="M29">
-        <v>25590.779200450401</v>
-      </c>
-      <c r="N29">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O29">
-        <v>0</v>
-      </c>
-      <c r="P29">
-        <v>369500.62413077202</v>
-      </c>
-      <c r="Q29">
-        <v>1466.60671595592</v>
-      </c>
-      <c r="R29">
-        <v>0</v>
-      </c>
-      <c r="S29">
-        <v>0</v>
-      </c>
-      <c r="T29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A30" t="s">
-        <v>22</v>
-      </c>
-      <c r="B30" t="s">
+      <c r="B30" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C30">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D30">
-        <v>171564.02128394699</v>
+        <v>103263.067623782</v>
       </c>
       <c r="E30">
         <v>282179.67123287701</v>
       </c>
       <c r="F30">
-        <v>1.03875662810921</v>
-      </c>
-      <c r="G30">
-        <v>73514.1870928641</v>
+        <v>0.79670888114802996</v>
+      </c>
+      <c r="G30" s="4">
+        <v>18270.343045682599</v>
       </c>
       <c r="H30">
-        <v>7482.8438362204697</v>
+        <v>4859.1187222275803</v>
       </c>
       <c r="I30">
-        <v>4044.9309872213798</v>
+        <v>2610.3522592715499</v>
       </c>
       <c r="J30">
-        <v>85041.961916305998</v>
+        <v>25739.814027181699</v>
       </c>
       <c r="K30">
-        <v>51119.832654572398</v>
+        <v>48809.484574716203</v>
       </c>
       <c r="L30">
-        <v>16047.2916290263</v>
+        <v>9838.23116441202</v>
       </c>
       <c r="M30">
-        <v>19354.9350840429</v>
+        <v>18875.537857472798</v>
       </c>
       <c r="N30">
         <v>992.31070788530405</v>
@@ -2370,214 +2269,215 @@
         <v>0</v>
       </c>
       <c r="P30">
-        <v>293116.00381082902</v>
+        <v>224815.050150664</v>
       </c>
       <c r="Q30">
-        <v>1187.62883512946</v>
+        <v>1103.3542485400801</v>
       </c>
       <c r="R30">
-        <v>9393.8913494494009</v>
+        <v>0</v>
       </c>
       <c r="S30">
-        <v>260.94142637359403</v>
+        <v>0</v>
       </c>
       <c r="T30">
-        <v>-3.6405201993767098</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A31" t="s">
-        <v>20</v>
-      </c>
-      <c r="B31" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:21" x14ac:dyDescent="0.4">
+      <c r="A31" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B31" s="5" t="s">
         <v>21</v>
       </c>
       <c r="C31">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="D31">
-        <v>117032.41959359701</v>
+        <v>117493.882010934</v>
       </c>
       <c r="E31">
-        <v>282179.67123286898</v>
+        <v>282179.67123284901</v>
       </c>
       <c r="F31">
-        <v>0.845505280653571</v>
-      </c>
-      <c r="G31" s="4">
-        <v>23683.129427060001</v>
+        <v>0.84714063027084496</v>
+      </c>
+      <c r="G31">
+        <v>19869.854426770002</v>
       </c>
       <c r="H31">
-        <v>6986.3695969997798</v>
+        <v>5589.63461833969</v>
       </c>
       <c r="I31">
-        <v>918.40768838365295</v>
+        <v>5989.0327102104202</v>
       </c>
       <c r="J31">
-        <v>31587.906712443499</v>
+        <v>31448.5217553201</v>
       </c>
       <c r="K31">
-        <v>50843.1840059237</v>
+        <v>50997.445205592398</v>
       </c>
       <c r="L31">
-        <v>15303.7983857823</v>
+        <v>15718.3753616421</v>
       </c>
       <c r="M31">
-        <v>19297.530489448101</v>
+        <v>19329.5396883797</v>
       </c>
       <c r="N31">
-        <v>992.31070788530405</v>
+        <v>1001.30446052474</v>
       </c>
       <c r="O31">
         <v>0</v>
       </c>
       <c r="P31">
-        <v>238584.402120479</v>
+        <v>239045.864537816</v>
       </c>
       <c r="Q31">
-        <v>1108.83163779344</v>
+        <v>1248.8628027930299</v>
       </c>
       <c r="R31">
-        <v>0</v>
+        <v>13651.1458247473</v>
       </c>
       <c r="S31">
-        <v>230512.59606633501</v>
+        <v>115.68767648091</v>
       </c>
       <c r="T31">
-        <v>1103.3673370121001</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="G32" s="4"/>
+        <v>1.42140322536358</v>
+      </c>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A33" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="B33" t="s">
-        <v>21</v>
-      </c>
-      <c r="C33">
-        <v>4</v>
-      </c>
-      <c r="D33">
-        <v>116833.749486644</v>
-      </c>
-      <c r="E33">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F33">
-        <v>0.84480122530439805</v>
-      </c>
-      <c r="G33" s="4">
-        <v>23535.478746437901</v>
-      </c>
-      <c r="H33">
-        <v>6941.2778055266899</v>
-      </c>
-      <c r="I33">
-        <v>912.48005352310201</v>
-      </c>
-      <c r="J33">
-        <v>31389.236605487698</v>
-      </c>
-      <c r="K33">
-        <v>50843.184005923998</v>
-      </c>
-      <c r="L33">
-        <v>15303.798385784499</v>
-      </c>
-      <c r="M33">
-        <v>19297.5304894484</v>
-      </c>
-      <c r="N33">
-        <v>992.31070788530405</v>
-      </c>
-      <c r="O33">
-        <v>0</v>
-      </c>
-      <c r="P33">
-        <v>0</v>
-      </c>
-      <c r="Q33">
-        <v>0</v>
-      </c>
-      <c r="R33">
-        <v>0</v>
-      </c>
-      <c r="S33">
-        <v>0</v>
-      </c>
-      <c r="T33">
-        <v>0</v>
-      </c>
+      <c r="A33" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G33" s="4"/>
     </row>
     <row r="34" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A34" t="s">
         <v>22</v>
       </c>
       <c r="B34" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="C34">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="D34">
-        <v>124393.533174422</v>
+        <v>187020.456722612</v>
       </c>
       <c r="E34">
-        <v>282179.67123444699</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F34">
-        <v>0.87159189967643702</v>
-      </c>
-      <c r="G34" s="4">
-        <v>21072.189860718699</v>
+        <v>1.09353178385</v>
+      </c>
+      <c r="G34">
+        <v>89520.694507565597</v>
       </c>
       <c r="H34">
-        <v>9188.7245080883695</v>
+        <v>6971.3813103080802</v>
       </c>
       <c r="I34">
-        <v>2618.8827210474601</v>
+        <v>5083.8680235841202</v>
       </c>
       <c r="J34">
-        <v>32879.797089854597</v>
+        <v>101575.943841457</v>
       </c>
       <c r="K34">
-        <v>50904.118537438801</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L34">
-        <v>20591.7266090095</v>
+        <v>15303.798385783</v>
       </c>
       <c r="M34">
-        <v>20017.890938119701</v>
+        <v>19297.5304894482</v>
       </c>
       <c r="N34">
-        <v>1040.9289460857101</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O34">
         <v>0</v>
       </c>
       <c r="P34">
-        <v>245945.51570130399</v>
+        <v>308572.439249494</v>
       </c>
       <c r="Q34">
-        <v>1458.3752411216699</v>
+        <v>1106.4527933521999</v>
       </c>
       <c r="R34">
-        <v>35012.612233571497</v>
+        <v>3451.9307168288801</v>
       </c>
       <c r="S34">
-        <v>875.31530583928895</v>
+        <v>20.547206647791</v>
       </c>
       <c r="T34">
-        <v>0.51444695802960605</v>
+        <v>-14.696886263168601</v>
+      </c>
+    </row>
+    <row r="35" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A35" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B35" t="s">
+        <v>23</v>
+      </c>
+      <c r="C35">
+        <v>0</v>
+      </c>
+      <c r="D35">
+        <v>247948.64160389101</v>
+      </c>
+      <c r="E35">
+        <v>374203.2</v>
+      </c>
+      <c r="F35">
+        <v>0.98743309552342695</v>
+      </c>
+      <c r="G35" s="4">
+        <v>118659.96685142</v>
+      </c>
+      <c r="H35">
+        <v>9240.5882208594503</v>
+      </c>
+      <c r="I35">
+        <v>6738.6833231561404</v>
+      </c>
+      <c r="J35">
+        <v>134639.23839543501</v>
+      </c>
+      <c r="K35">
+        <v>67424.000002171</v>
+      </c>
+      <c r="L35">
+        <v>20294.624005833801</v>
+      </c>
+      <c r="M35">
+        <v>25590.779200450401</v>
+      </c>
+      <c r="N35">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O35">
+        <v>0</v>
+      </c>
+      <c r="P35">
+        <v>369500.62413077202</v>
+      </c>
+      <c r="Q35">
+        <v>1466.60671595592</v>
+      </c>
+      <c r="R35">
+        <v>0</v>
+      </c>
+      <c r="S35">
+        <v>0</v>
+      </c>
+      <c r="T35">
+        <v>0</v>
       </c>
     </row>
     <row r="36" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A36" s="1" t="s">
-        <v>30</v>
-      </c>
+      <c r="A36" s="3"/>
       <c r="G36" s="4"/>
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.4">
@@ -2585,302 +2485,318 @@
         <v>22</v>
       </c>
       <c r="B37" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C37">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D37">
-        <v>115472.147206908</v>
+        <v>171564.02128394699</v>
       </c>
       <c r="E37">
-        <v>282495</v>
+        <v>282179.67123287701</v>
       </c>
       <c r="F37">
-        <v>0.83903831831993503</v>
-      </c>
-      <c r="G37" s="4">
-        <v>20221.889710343999</v>
+        <v>1.03875662810921</v>
+      </c>
+      <c r="G37">
+        <v>73514.1870928641</v>
       </c>
       <c r="H37">
-        <v>6553.7440767980397</v>
+        <v>7482.8438362204697</v>
       </c>
       <c r="I37">
-        <v>6160.4249909476703</v>
+        <v>4044.9309872213798</v>
       </c>
       <c r="J37">
-        <v>32936.058778089697</v>
+        <v>85041.961916305998</v>
       </c>
       <c r="K37">
-        <v>50939.5611113743</v>
+        <v>51119.832654572398</v>
       </c>
       <c r="L37">
-        <v>15427.2204868183</v>
+        <v>16047.2916290263</v>
       </c>
       <c r="M37">
-        <v>19327.3039306102</v>
+        <v>19354.9350840429</v>
       </c>
       <c r="N37">
-        <v>1004.9477757237401</v>
+        <v>992.31070788530405</v>
       </c>
       <c r="O37">
-        <v>3157.9970999842499</v>
+        <v>0</v>
       </c>
       <c r="P37">
-        <v>237024.12973379</v>
+        <v>293116.00381082902</v>
       </c>
       <c r="Q37">
-        <v>1464.2687322859999</v>
+        <v>1187.62883512946</v>
       </c>
       <c r="R37">
-        <v>8672.9882445954008</v>
+        <v>9393.8913494494009</v>
       </c>
       <c r="S37">
-        <v>346.91952978381602</v>
+        <v>260.94142637359403</v>
       </c>
       <c r="T37">
-        <v>2.4302910949698302</v>
+        <v>-3.6405201993767098</v>
       </c>
     </row>
     <row r="38" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A38" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B38" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="C38">
+        <v>0</v>
+      </c>
+      <c r="D38">
+        <v>117032.41959359701</v>
+      </c>
+      <c r="E38">
+        <v>282179.67123286898</v>
+      </c>
+      <c r="F38">
+        <v>0.845505280653571</v>
+      </c>
+      <c r="G38" s="4">
+        <v>23683.129427060001</v>
+      </c>
+      <c r="H38">
+        <v>6986.3695969997798</v>
+      </c>
+      <c r="I38">
+        <v>918.40768838365295</v>
+      </c>
+      <c r="J38">
+        <v>31587.906712443499</v>
+      </c>
+      <c r="K38">
+        <v>50843.1840059237</v>
+      </c>
+      <c r="L38">
+        <v>15303.7983857823</v>
+      </c>
+      <c r="M38">
+        <v>19297.530489448101</v>
+      </c>
+      <c r="N38">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O38">
+        <v>0</v>
+      </c>
+      <c r="P38">
+        <v>238584.402120479</v>
+      </c>
+      <c r="Q38">
+        <v>1108.83163779344</v>
+      </c>
+      <c r="R38">
+        <v>0</v>
+      </c>
+      <c r="S38">
+        <v>230512.59606633501</v>
+      </c>
+      <c r="T38">
+        <v>1103.3673370121001</v>
+      </c>
+    </row>
+    <row r="39" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="G39" s="4"/>
+    </row>
+    <row r="40" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A40" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="B40" t="s">
+        <v>21</v>
+      </c>
+      <c r="C40">
         <v>4</v>
       </c>
-      <c r="D38">
-        <v>108958.027502652</v>
-      </c>
-      <c r="E38">
+      <c r="D40">
+        <v>116833.749486644</v>
+      </c>
+      <c r="E40">
         <v>282179.67123287602</v>
       </c>
-      <c r="F38">
-        <v>0.81689091571482797</v>
-      </c>
-      <c r="G38" s="4">
-        <v>20285.098342207999</v>
-      </c>
-      <c r="H38">
-        <v>6552.6722224723899</v>
-      </c>
-      <c r="I38">
-        <v>6068.9240568166097</v>
-      </c>
-      <c r="J38">
-        <v>32906.694621497001</v>
-      </c>
-      <c r="K38">
-        <v>50843.184005923598</v>
-      </c>
-      <c r="L38">
-        <v>16378.7983857829</v>
-      </c>
-      <c r="M38">
-        <v>19449.350489448301</v>
-      </c>
-      <c r="N38">
-        <v>1004.9477757237401</v>
-      </c>
-      <c r="O38">
-        <v>10620</v>
-      </c>
-      <c r="P38">
-        <v>230510.010029533</v>
-      </c>
-      <c r="Q38">
-        <v>1464.02925348484</v>
-      </c>
-      <c r="R38">
-        <v>26064.489084194902</v>
-      </c>
-      <c r="S38">
-        <v>407.257641940545</v>
-      </c>
-      <c r="T38">
-        <v>1.09609872121186</v>
-      </c>
-    </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A40" s="1" t="s">
-        <v>31</v>
+      <c r="F40">
+        <v>0.84480122530439805</v>
+      </c>
+      <c r="G40" s="4">
+        <v>23535.478746437901</v>
+      </c>
+      <c r="H40">
+        <v>6941.2778055266899</v>
+      </c>
+      <c r="I40">
+        <v>912.48005352310201</v>
+      </c>
+      <c r="J40">
+        <v>31389.236605487698</v>
+      </c>
+      <c r="K40">
+        <v>50843.184005923998</v>
+      </c>
+      <c r="L40">
+        <v>15303.798385784499</v>
+      </c>
+      <c r="M40">
+        <v>19297.5304894484</v>
+      </c>
+      <c r="N40">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O40">
+        <v>0</v>
+      </c>
+      <c r="P40">
+        <v>0</v>
+      </c>
+      <c r="Q40">
+        <v>0</v>
+      </c>
+      <c r="R40">
+        <v>0</v>
+      </c>
+      <c r="S40">
+        <v>0</v>
+      </c>
+      <c r="T40">
+        <v>0</v>
       </c>
     </row>
     <row r="41" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A41" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B41" t="s">
         <v>21</v>
       </c>
       <c r="C41">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D41">
-        <v>115714.10508262301</v>
+        <v>124393.533174422</v>
       </c>
       <c r="E41">
-        <v>282179.67125387199</v>
+        <v>282179.67123444699</v>
       </c>
       <c r="F41">
-        <v>0.840833383054163</v>
+        <v>0.87159189967643702</v>
       </c>
       <c r="G41" s="4">
-        <v>20578.507216446698</v>
+        <v>21072.189860718699</v>
       </c>
       <c r="H41">
-        <v>7102.57515066207</v>
+        <v>9188.7245080883695</v>
       </c>
       <c r="I41">
-        <v>2588.5052959285099</v>
+        <v>2618.8827210474601</v>
       </c>
       <c r="J41">
-        <v>30269.587663037299</v>
+        <v>32879.797089854597</v>
       </c>
       <c r="K41">
-        <v>50843.185173268597</v>
+        <v>50904.118537438801</v>
       </c>
       <c r="L41">
-        <v>15303.8015139941</v>
+        <v>20591.7266090095</v>
       </c>
       <c r="M41">
-        <v>19297.530732323401</v>
+        <v>20017.890938119701</v>
       </c>
       <c r="N41">
-        <v>992.31070788530405</v>
+        <v>1040.9289460857101</v>
       </c>
       <c r="O41">
         <v>0</v>
       </c>
       <c r="P41">
-        <v>237266.08760950499</v>
+        <v>245945.51570130399</v>
       </c>
       <c r="Q41">
-        <v>1127.2750356983099</v>
+        <v>1458.3752411216699</v>
       </c>
       <c r="R41">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A42" t="s">
-        <v>22</v>
-      </c>
-      <c r="B42" t="s">
-        <v>21</v>
-      </c>
-      <c r="C42">
-        <v>2</v>
-      </c>
-      <c r="D42">
-        <v>120628.41082793</v>
-      </c>
-      <c r="E42">
-        <v>282179.67123287602</v>
-      </c>
-      <c r="F42">
-        <v>0.85824890324911396</v>
-      </c>
-      <c r="G42" s="4">
-        <v>20824.7129679639</v>
-      </c>
-      <c r="H42">
-        <v>7456.39074483072</v>
-      </c>
-      <c r="I42">
-        <v>5114.4587365303096</v>
-      </c>
-      <c r="J42">
-        <v>33395.562449324898</v>
-      </c>
-      <c r="K42">
-        <v>51302.320205525801</v>
-      </c>
-      <c r="L42">
-        <v>16537.7269222135</v>
-      </c>
-      <c r="M42">
-        <v>19392.801250865799</v>
-      </c>
-      <c r="N42">
-        <v>1004.9477757237401</v>
-      </c>
-      <c r="O42">
-        <v>0</v>
-      </c>
-      <c r="P42">
-        <v>242180.39335481101</v>
-      </c>
-      <c r="Q42">
-        <v>1183.4303612998101</v>
-      </c>
-      <c r="R42">
-        <v>15931.1957490451</v>
-      </c>
-      <c r="S42">
-        <v>346.33034237054602</v>
-      </c>
-      <c r="T42">
-        <v>1.0959871186973</v>
-      </c>
+        <v>35012.612233571497</v>
+      </c>
+      <c r="S41">
+        <v>875.31530583928895</v>
+      </c>
+      <c r="T41">
+        <v>0.51444695802960605</v>
+      </c>
+    </row>
+    <row r="43" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A43" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="G43" s="4"/>
     </row>
     <row r="44" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A44" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B44" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C44">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D44">
-        <v>115714.10508261999</v>
+        <v>115472.147206908</v>
       </c>
       <c r="E44">
-        <v>282179.671253876</v>
+        <v>282495</v>
       </c>
       <c r="F44">
-        <v>0.84083338305413902</v>
+        <v>0.83903831831993503</v>
       </c>
       <c r="G44" s="4">
-        <v>20578.5072164468</v>
+        <v>20221.889710343999</v>
       </c>
       <c r="H44">
-        <v>7102.5751506616798</v>
+        <v>6553.7440767980397</v>
       </c>
       <c r="I44">
-        <v>2588.50529592865</v>
+        <v>6160.4249909476703</v>
       </c>
       <c r="J44">
-        <v>30269.587663037099</v>
+        <v>32936.058778089697</v>
       </c>
       <c r="K44">
-        <v>50843.185173268197</v>
+        <v>50939.5611113743</v>
       </c>
       <c r="L44">
-        <v>15303.8015139912</v>
+        <v>15427.2204868183</v>
       </c>
       <c r="M44">
-        <v>19297.530732323299</v>
+        <v>19327.3039306102</v>
       </c>
       <c r="N44">
-        <v>992.31070788530405</v>
+        <v>1004.9477757237401</v>
       </c>
       <c r="O44">
-        <v>0</v>
+        <v>3157.9970999842499</v>
       </c>
       <c r="P44">
-        <v>237266.087609501</v>
+        <v>237024.12973379</v>
       </c>
       <c r="Q44">
-        <v>1127.2750356983499</v>
+        <v>1464.2687322859999</v>
       </c>
       <c r="R44">
-        <v>0</v>
+        <v>8672.9882445954008</v>
+      </c>
+      <c r="S44">
+        <v>346.91952978381602</v>
+      </c>
+      <c r="T44">
+        <v>2.4302910949698302</v>
       </c>
     </row>
     <row r="45" spans="1:20" x14ac:dyDescent="0.4">
@@ -2888,213 +2804,929 @@
         <v>22</v>
       </c>
       <c r="B45" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="C45">
         <v>4</v>
       </c>
       <c r="D45">
-        <v>120375.156660901</v>
+        <v>108958.027502652</v>
       </c>
       <c r="E45">
-        <v>282179.671232878</v>
+        <v>282179.67123287602</v>
       </c>
       <c r="F45">
-        <v>0.857351410648304</v>
+        <v>0.81689091571482797</v>
       </c>
       <c r="G45" s="4">
-        <v>21285.1004075495</v>
+        <v>20285.098342207999</v>
       </c>
       <c r="H45">
-        <v>7426.32532798384</v>
+        <v>6552.6722224723899</v>
       </c>
       <c r="I45">
-        <v>5046.79446201879</v>
+        <v>6068.9240568166097</v>
       </c>
       <c r="J45">
-        <v>33758.220197552102</v>
+        <v>32906.694621497001</v>
       </c>
       <c r="K45">
-        <v>51144.191344099498</v>
+        <v>50843.184005923598</v>
       </c>
       <c r="L45">
-        <v>16112.7556071296</v>
+        <v>16378.7983857829</v>
       </c>
       <c r="M45">
-        <v>19359.989512119799</v>
+        <v>19449.350489448301</v>
       </c>
       <c r="N45">
-        <v>1006.77939378399</v>
+        <v>1004.9477757237401</v>
       </c>
       <c r="O45">
-        <v>0</v>
+        <v>10620</v>
       </c>
       <c r="P45">
-        <v>241927.13918778201</v>
+        <v>230510.010029533</v>
       </c>
       <c r="Q45">
-        <v>1178.65858109644</v>
+        <v>1464.02925348484</v>
       </c>
       <c r="R45">
-        <v>12586.325853030899</v>
+        <v>26064.489084194902</v>
       </c>
       <c r="S45">
-        <v>466.16021677892502</v>
+        <v>407.257641940545</v>
       </c>
       <c r="T45">
-        <v>1.3585822738026401</v>
-      </c>
-    </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="G46" s="4"/>
-    </row>
-    <row r="47" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+        <v>1.09609872121186</v>
+      </c>
+    </row>
+    <row r="47" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A47" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G47" s="4"/>
-      <c r="P47" t="s">
-        <v>15</v>
-      </c>
-      <c r="Q47" t="s">
-        <v>16</v>
-      </c>
-      <c r="R47" t="s">
-        <v>17</v>
-      </c>
-      <c r="S47" t="s">
-        <v>18</v>
-      </c>
-      <c r="T47" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="48" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
-      <c r="A48" t="s">
-        <v>0</v>
-      </c>
-      <c r="B48" t="s">
-        <v>1</v>
-      </c>
-      <c r="C48" t="s">
-        <v>2</v>
-      </c>
-      <c r="D48" t="s">
-        <v>3</v>
-      </c>
-      <c r="E48" t="s">
-        <v>4</v>
-      </c>
-      <c r="F48" t="s">
-        <v>5</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H48" t="s">
-        <v>7</v>
-      </c>
-      <c r="I48" t="s">
-        <v>8</v>
-      </c>
-      <c r="J48" t="s">
-        <v>9</v>
-      </c>
-      <c r="K48" t="s">
-        <v>10</v>
-      </c>
-      <c r="L48" t="s">
-        <v>11</v>
-      </c>
-      <c r="M48" t="s">
-        <v>12</v>
-      </c>
-      <c r="N48" t="s">
-        <v>13</v>
-      </c>
-      <c r="O48" t="s">
-        <v>14</v>
-      </c>
-      <c r="P48">
-        <v>63734.6679</v>
-      </c>
-      <c r="Q48">
-        <v>1078.4492829999999</v>
-      </c>
-      <c r="R48">
-        <v>624.70352849999995</v>
-      </c>
-      <c r="S48">
-        <v>13.014656840000001</v>
-      </c>
-      <c r="T48">
-        <v>27.514184579999998</v>
-      </c>
-    </row>
-    <row r="49" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="48" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A48" s="1"/>
+    </row>
+    <row r="49" spans="1:20" x14ac:dyDescent="0.4">
       <c r="A49" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C49">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A50" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="C50">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A51" s="1"/>
+    </row>
+    <row r="52" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A52" t="s">
+        <v>20</v>
+      </c>
+      <c r="B52" t="s">
         <v>21</v>
       </c>
-      <c r="C49">
+      <c r="C52">
+        <v>2</v>
+      </c>
+      <c r="D52">
+        <v>115714.10508262301</v>
+      </c>
+      <c r="E52">
+        <v>282179.67125387199</v>
+      </c>
+      <c r="F52">
+        <v>0.840833383054163</v>
+      </c>
+      <c r="G52" s="4">
+        <v>20578.507216446698</v>
+      </c>
+      <c r="H52">
+        <v>7102.57515066207</v>
+      </c>
+      <c r="I52">
+        <v>2588.5052959285099</v>
+      </c>
+      <c r="J52">
+        <v>30269.587663037299</v>
+      </c>
+      <c r="K52">
+        <v>50843.185173268597</v>
+      </c>
+      <c r="L52">
+        <v>15303.8015139941</v>
+      </c>
+      <c r="M52">
+        <v>19297.530732323401</v>
+      </c>
+      <c r="N52">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O52">
+        <v>0</v>
+      </c>
+      <c r="P52">
+        <v>237266.08760950499</v>
+      </c>
+      <c r="Q52">
+        <v>1127.2750356983099</v>
+      </c>
+      <c r="R52">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A53" t="s">
+        <v>22</v>
+      </c>
+      <c r="B53" t="s">
+        <v>21</v>
+      </c>
+      <c r="C53">
+        <v>2</v>
+      </c>
+      <c r="D53">
+        <v>120628.41082793</v>
+      </c>
+      <c r="E53">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F53">
+        <v>0.85824890324911396</v>
+      </c>
+      <c r="G53" s="4">
+        <v>20824.7129679639</v>
+      </c>
+      <c r="H53">
+        <v>7456.39074483072</v>
+      </c>
+      <c r="I53">
+        <v>5114.4587365303096</v>
+      </c>
+      <c r="J53">
+        <v>33395.562449324898</v>
+      </c>
+      <c r="K53">
+        <v>51302.320205525801</v>
+      </c>
+      <c r="L53">
+        <v>16537.7269222135</v>
+      </c>
+      <c r="M53">
+        <v>19392.801250865799</v>
+      </c>
+      <c r="N53">
+        <v>1004.9477757237401</v>
+      </c>
+      <c r="O53">
+        <v>0</v>
+      </c>
+      <c r="P53">
+        <v>242180.39335481101</v>
+      </c>
+      <c r="Q53">
+        <v>1183.4303612998101</v>
+      </c>
+      <c r="R53">
+        <v>15931.1957490451</v>
+      </c>
+      <c r="S53">
+        <v>346.33034237054602</v>
+      </c>
+      <c r="T53">
+        <v>1.0959871186973</v>
+      </c>
+    </row>
+    <row r="55" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A55" t="s">
+        <v>20</v>
+      </c>
+      <c r="B55" t="s">
+        <v>21</v>
+      </c>
+      <c r="C55">
         <v>4</v>
       </c>
-      <c r="D49">
+      <c r="D55">
+        <v>115714.10508261999</v>
+      </c>
+      <c r="E55">
+        <v>282179.671253876</v>
+      </c>
+      <c r="F55">
+        <v>0.84083338305413902</v>
+      </c>
+      <c r="G55" s="4">
+        <v>20578.5072164468</v>
+      </c>
+      <c r="H55">
+        <v>7102.5751506616798</v>
+      </c>
+      <c r="I55">
+        <v>2588.50529592865</v>
+      </c>
+      <c r="J55">
+        <v>30269.587663037099</v>
+      </c>
+      <c r="K55">
+        <v>50843.185173268197</v>
+      </c>
+      <c r="L55">
+        <v>15303.8015139912</v>
+      </c>
+      <c r="M55">
+        <v>19297.530732323299</v>
+      </c>
+      <c r="N55">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O55">
+        <v>0</v>
+      </c>
+      <c r="P55">
+        <v>237266.087609501</v>
+      </c>
+      <c r="Q55">
+        <v>1127.2750356983499</v>
+      </c>
+      <c r="R55">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A56" t="s">
+        <v>22</v>
+      </c>
+      <c r="B56" t="s">
+        <v>21</v>
+      </c>
+      <c r="C56">
+        <v>4</v>
+      </c>
+      <c r="D56">
+        <v>120375.156660901</v>
+      </c>
+      <c r="E56">
+        <v>282179.671232878</v>
+      </c>
+      <c r="F56">
+        <v>0.857351410648304</v>
+      </c>
+      <c r="G56" s="4">
+        <v>21285.1004075495</v>
+      </c>
+      <c r="H56">
+        <v>7426.32532798384</v>
+      </c>
+      <c r="I56">
+        <v>5046.79446201879</v>
+      </c>
+      <c r="J56">
+        <v>33758.220197552102</v>
+      </c>
+      <c r="K56">
+        <v>51144.191344099498</v>
+      </c>
+      <c r="L56">
+        <v>16112.7556071296</v>
+      </c>
+      <c r="M56">
+        <v>19359.989512119799</v>
+      </c>
+      <c r="N56">
+        <v>1006.77939378399</v>
+      </c>
+      <c r="O56">
+        <v>0</v>
+      </c>
+      <c r="P56">
+        <v>241927.13918778201</v>
+      </c>
+      <c r="Q56">
+        <v>1178.65858109644</v>
+      </c>
+      <c r="R56">
+        <v>12586.325853030899</v>
+      </c>
+      <c r="S56">
+        <v>466.16021677892502</v>
+      </c>
+      <c r="T56">
+        <v>1.3585822738026401</v>
+      </c>
+    </row>
+    <row r="57" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="G57" s="4"/>
+    </row>
+    <row r="58" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A58" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G58" s="4"/>
+      <c r="P58" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q58" t="s">
+        <v>16</v>
+      </c>
+      <c r="R58" t="s">
+        <v>17</v>
+      </c>
+      <c r="S58" t="s">
+        <v>18</v>
+      </c>
+      <c r="T58" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="59" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A59" t="s">
+        <v>0</v>
+      </c>
+      <c r="B59" t="s">
+        <v>1</v>
+      </c>
+      <c r="C59" t="s">
+        <v>2</v>
+      </c>
+      <c r="D59" t="s">
+        <v>3</v>
+      </c>
+      <c r="E59" t="s">
+        <v>4</v>
+      </c>
+      <c r="F59" t="s">
+        <v>5</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="H59" t="s">
+        <v>7</v>
+      </c>
+      <c r="I59" t="s">
+        <v>8</v>
+      </c>
+      <c r="J59" t="s">
+        <v>9</v>
+      </c>
+      <c r="K59" t="s">
+        <v>10</v>
+      </c>
+      <c r="L59" t="s">
+        <v>11</v>
+      </c>
+      <c r="M59" t="s">
+        <v>12</v>
+      </c>
+      <c r="N59" t="s">
+        <v>13</v>
+      </c>
+      <c r="O59" t="s">
+        <v>14</v>
+      </c>
+      <c r="P59">
+        <v>63734.6679</v>
+      </c>
+      <c r="Q59">
+        <v>1078.4492829999999</v>
+      </c>
+      <c r="R59">
+        <v>624.70352849999995</v>
+      </c>
+      <c r="S59">
+        <v>13.014656840000001</v>
+      </c>
+      <c r="T59">
+        <v>27.514184579999998</v>
+      </c>
+    </row>
+    <row r="60" spans="1:20" hidden="1" x14ac:dyDescent="0.4">
+      <c r="A60" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="B60" t="s">
+        <v>21</v>
+      </c>
+      <c r="C60">
+        <v>4</v>
+      </c>
+      <c r="D60">
         <v>29525.427309999999</v>
       </c>
-      <c r="E49">
+      <c r="E60">
         <v>80391.755990000005</v>
       </c>
-      <c r="F49">
+      <c r="F60">
         <v>0.79280104200000001</v>
       </c>
-      <c r="G49" s="4">
+      <c r="G60" s="4">
         <v>5050.6365619999997</v>
       </c>
-      <c r="H49">
+      <c r="H60">
         <v>4678.3390820000004</v>
       </c>
-      <c r="I49">
+      <c r="I60">
         <v>2508.6600360000002</v>
       </c>
-      <c r="J49">
+      <c r="J60">
         <v>12237.635679999999</v>
       </c>
-      <c r="K49">
+      <c r="K60">
         <v>13920</v>
       </c>
-      <c r="L49">
+      <c r="L60">
         <v>2841.544922</v>
       </c>
-      <c r="M49">
+      <c r="M60">
         <v>5380.5444360000001</v>
       </c>
-      <c r="N49">
+      <c r="N60">
         <v>279.27307350000001</v>
       </c>
-      <c r="O49">
-        <v>0</v>
-      </c>
-      <c r="P49">
+      <c r="O60">
+        <v>0</v>
+      </c>
+      <c r="P60">
         <v>64865.028310000002</v>
       </c>
-      <c r="Q49">
+      <c r="Q60">
         <v>1191.7509680000001</v>
       </c>
-      <c r="R49">
+      <c r="R60">
         <v>7243.7162129999997</v>
       </c>
-      <c r="S49">
+      <c r="S60">
         <v>452.7322633</v>
       </c>
-      <c r="T49">
+      <c r="T60">
         <v>5.8154128590000003</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.4">
-      <c r="A50" s="2"/>
+    <row r="61" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A61" s="7" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="63" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A63" t="s">
+        <v>34</v>
+      </c>
+      <c r="B63" t="s">
+        <v>35</v>
+      </c>
+      <c r="C63" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A64">
+        <v>20</v>
+      </c>
+      <c r="B64">
+        <v>60</v>
+      </c>
+      <c r="C64">
+        <v>2</v>
+      </c>
+      <c r="D64">
+        <v>119696.652328767</v>
+      </c>
+      <c r="E64">
+        <v>282179.67123285501</v>
+      </c>
+      <c r="F64">
+        <v>0.854946898908852</v>
+      </c>
+      <c r="G64">
+        <v>18681.222424938602</v>
+      </c>
+      <c r="H64">
+        <v>5354.6114985546601</v>
+      </c>
+      <c r="I64">
+        <v>8156.08309050551</v>
+      </c>
+      <c r="J64">
+        <v>32191.917013998798</v>
+      </c>
+      <c r="K64">
+        <v>51372.124296964801</v>
+      </c>
+      <c r="L64">
+        <v>16725.325417965501</v>
+      </c>
+      <c r="M64">
+        <v>19407.285599838699</v>
+      </c>
+      <c r="N64">
+        <v>1016.03855436447</v>
+      </c>
+      <c r="O64">
+        <v>0</v>
+      </c>
+      <c r="P64">
+        <v>241248.634855649</v>
+      </c>
+      <c r="Q64">
+        <v>1192.7637589594799</v>
+      </c>
+      <c r="R64">
+        <v>19736.206339365101</v>
+      </c>
+      <c r="S64">
+        <v>481.37088632597801</v>
+      </c>
+      <c r="T64" s="6">
+        <v>0.12591688076390301</v>
+      </c>
+    </row>
+    <row r="65" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A65">
+        <v>20</v>
+      </c>
+      <c r="B65">
+        <v>50</v>
+      </c>
+      <c r="C65">
+        <v>2</v>
+      </c>
+      <c r="D65">
+        <v>118381.960809661</v>
+      </c>
+      <c r="E65">
+        <v>282254.81855225202</v>
+      </c>
+      <c r="F65">
+        <v>0.85006146065890897</v>
+      </c>
+      <c r="G65">
+        <v>19407.840072768398</v>
+      </c>
+      <c r="H65">
+        <v>5891.8301217549197</v>
+      </c>
+      <c r="I65">
+        <v>6659.4942697455399</v>
+      </c>
+      <c r="J65">
+        <v>31959.164464268899</v>
+      </c>
+      <c r="K65">
+        <v>51102.045942938203</v>
+      </c>
+      <c r="L65">
+        <v>15967.176494174801</v>
+      </c>
+      <c r="M65">
+        <v>19353.573908279199</v>
+      </c>
+      <c r="N65">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O65">
+        <v>0</v>
+      </c>
+      <c r="P65">
+        <v>239933.943336542</v>
+      </c>
+      <c r="Q65">
+        <v>1312.43161993582</v>
+      </c>
+      <c r="R65">
+        <v>18377.616631847999</v>
+      </c>
+      <c r="S65">
+        <v>459.4404157962</v>
+      </c>
+      <c r="T65" s="6">
+        <v>0.14758705239613301</v>
+      </c>
+    </row>
+    <row r="66" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A66">
+        <v>20</v>
+      </c>
+      <c r="B66">
+        <v>40</v>
+      </c>
+      <c r="C66">
+        <v>2</v>
+      </c>
+      <c r="D66">
+        <v>116766.56672038</v>
+      </c>
+      <c r="E66">
+        <v>282179.67123287299</v>
+      </c>
+      <c r="F66">
+        <v>0.84456314023622803</v>
+      </c>
+      <c r="G66">
+        <v>19298.245593088301</v>
+      </c>
+      <c r="H66">
+        <v>5682.0016560700296</v>
+      </c>
+      <c r="I66">
+        <v>5350.3346939491703</v>
+      </c>
+      <c r="J66">
+        <v>30330.5819431075</v>
+      </c>
+      <c r="K66">
+        <v>51097.733915068202</v>
+      </c>
+      <c r="L66">
+        <v>15987.901266609</v>
+      </c>
+      <c r="M66">
+        <v>19350.349595595701</v>
+      </c>
+      <c r="N66">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O66">
+        <v>0</v>
+      </c>
+      <c r="P66">
+        <v>238318.54924726201</v>
+      </c>
+      <c r="Q66">
+        <v>1265.6913868611</v>
+      </c>
+      <c r="R66">
+        <v>17746.163883660702</v>
+      </c>
+      <c r="S66">
+        <v>507.03325381887902</v>
+      </c>
+      <c r="T66" s="6">
+        <v>-0.25983751983286502</v>
+      </c>
+    </row>
+    <row r="67" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A67">
+        <v>20</v>
+      </c>
+      <c r="B67">
+        <v>30</v>
+      </c>
+      <c r="C67">
+        <v>2</v>
+      </c>
+      <c r="D67">
+        <v>115610.996393592</v>
+      </c>
+      <c r="E67">
+        <v>282182.50548365602</v>
+      </c>
+      <c r="F67">
+        <v>0.84045954058697003</v>
+      </c>
+      <c r="G67">
+        <v>19302.752565837702</v>
+      </c>
+      <c r="H67">
+        <v>6226.5181629292701</v>
+      </c>
+      <c r="I67">
+        <v>3974.5318253822402</v>
+      </c>
+      <c r="J67">
+        <v>29503.802554149199</v>
+      </c>
+      <c r="K67">
+        <v>51013.610661725899</v>
+      </c>
+      <c r="L67">
+        <v>15760.601295416</v>
+      </c>
+      <c r="M67">
+        <v>19332.981882301501</v>
+      </c>
+      <c r="N67">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O67">
+        <v>0</v>
+      </c>
+      <c r="P67">
+        <v>237162.97892047401</v>
+      </c>
+      <c r="Q67">
+        <v>1386.9848841974899</v>
+      </c>
+      <c r="R67">
+        <v>18436.445202769701</v>
+      </c>
+      <c r="S67">
+        <v>209.50505912238299</v>
+      </c>
+      <c r="T67" s="6">
+        <v>0.28049716262959101</v>
+      </c>
+    </row>
+    <row r="68" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A68" s="3">
+        <v>20</v>
+      </c>
+      <c r="B68" s="3">
+        <v>20</v>
+      </c>
+      <c r="C68" s="3">
+        <v>2</v>
+      </c>
+      <c r="D68">
+        <v>114184.286860504</v>
+      </c>
+      <c r="E68">
+        <v>282179.67123297497</v>
+      </c>
+      <c r="F68">
+        <v>0.83541194997266699</v>
+      </c>
+      <c r="G68">
+        <v>19351.2255529412</v>
+      </c>
+      <c r="H68">
+        <v>6002.0469674603501</v>
+      </c>
+      <c r="I68">
+        <v>2645.4376652921501</v>
+      </c>
+      <c r="J68">
+        <v>27998.710185693701</v>
+      </c>
+      <c r="K68">
+        <v>51033.4442867088</v>
+      </c>
+      <c r="L68">
+        <v>15815.1228903871</v>
+      </c>
+      <c r="M68">
+        <v>19337.009497714302</v>
+      </c>
+      <c r="N68">
+        <v>1014.17312250211</v>
+      </c>
+      <c r="O68">
+        <v>0</v>
+      </c>
+      <c r="P68">
+        <v>235736.26938738499</v>
+      </c>
+      <c r="Q68">
+        <v>1336.98290493166</v>
+      </c>
+      <c r="R68">
+        <v>18577.307877855899</v>
+      </c>
+      <c r="S68">
+        <v>432.030415764091</v>
+      </c>
+      <c r="T68" s="6">
+        <v>-0.122490141098651</v>
+      </c>
+    </row>
+    <row r="69" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A69">
+        <v>20</v>
+      </c>
+      <c r="B69">
+        <v>15</v>
+      </c>
+      <c r="C69">
+        <v>2</v>
+      </c>
+      <c r="D69">
+        <v>113440.79599059001</v>
+      </c>
+      <c r="E69">
+        <v>282179.67123267101</v>
+      </c>
+      <c r="F69">
+        <v>0.83277713625127903</v>
+      </c>
+      <c r="G69">
+        <v>19390.977969205</v>
+      </c>
+      <c r="H69">
+        <v>5599.5405456203798</v>
+      </c>
+      <c r="I69">
+        <v>2128.1287863747102</v>
+      </c>
+      <c r="J69">
+        <v>27118.647301200101</v>
+      </c>
+      <c r="K69">
+        <v>51068.507704320902</v>
+      </c>
+      <c r="L69">
+        <v>15909.3558282099</v>
+      </c>
+      <c r="M69">
+        <v>19344.285156859401</v>
+      </c>
+      <c r="N69">
+        <v>1010.46273302954</v>
+      </c>
+      <c r="O69">
+        <v>0</v>
+      </c>
+      <c r="P69">
+        <v>234992.778517472</v>
+      </c>
+      <c r="Q69">
+        <v>1247.3228025527501</v>
+      </c>
+      <c r="R69">
+        <v>16417.502561416801</v>
+      </c>
+      <c r="S69">
+        <v>469.07150175476602</v>
+      </c>
+      <c r="T69" s="6">
+        <v>0.46004655114715598</v>
+      </c>
+    </row>
+    <row r="70" spans="1:20" x14ac:dyDescent="0.4">
+      <c r="A70">
+        <v>20</v>
+      </c>
+      <c r="B70">
+        <v>12</v>
+      </c>
+      <c r="C70">
+        <v>2</v>
+      </c>
+      <c r="D70">
+        <v>113795.448700252</v>
+      </c>
+      <c r="E70">
+        <v>282179.67123287602</v>
+      </c>
+      <c r="F70">
+        <v>0.83403396920434802</v>
+      </c>
+      <c r="G70">
+        <v>20436.472361711199</v>
+      </c>
+      <c r="H70">
+        <v>4946.5396722567002</v>
+      </c>
+      <c r="I70">
+        <v>2967.9237851293901</v>
+      </c>
+      <c r="J70">
+        <v>28350.9358190973</v>
+      </c>
+      <c r="K70">
+        <v>50843.184005923598</v>
+      </c>
+      <c r="L70">
+        <v>15303.798385783</v>
+      </c>
+      <c r="M70">
+        <v>19297.530489448302</v>
+      </c>
+      <c r="N70">
+        <v>992.31070788530405</v>
+      </c>
+      <c r="O70">
+        <v>0</v>
+      </c>
+      <c r="P70">
+        <v>235347.43122713399</v>
+      </c>
+      <c r="Q70">
+        <v>1101.8639118583401</v>
+      </c>
+      <c r="R70">
+        <v>13.380488321454299</v>
+      </c>
+      <c r="S70">
+        <v>2.67609766429086</v>
+      </c>
+      <c r="T70" s="6">
+        <v>-198.021555533488</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>